<commit_message>
estein - hooks - davis -luxemburg
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-americains.xlsx
+++ b/data/frise-philosophes-americains.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="497">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="500">
   <si>
     <t xml:space="preserve">FRISE DES PHILOSOPHES AMÉRICAINS ET LATINO-AMÉRICAINS — Données source</t>
   </si>
@@ -367,6 +367,7 @@
         <sz val="9"/>
         <rFont val="Microsoft YaHei"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">｜</t>
     </r>
@@ -1571,10 +1572,57 @@
     <t xml:space="preserve">1952 - 2021</t>
   </si>
   <si>
-    <t xml:space="preserve">bell HOOKS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Bell_hooks"  title=" Wikipedia"&gt;bell HOOKS&lt;/a&gt; (1952-2021), de son vrai nom Gloria Jean Watkins, est une autrice, professeure et militante féministe afro-américaine. Née dans le Kentucky, dans le Sud ségrégationniste, elle prit le nom de son arrière-grand-mère, qu'elle écrivait en minuscules pour que l'attention se porte sur ses idées plutôt que sur sa personne.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Ne suis-je pas une femme ?&lt;/em&gt; (1981), elle montre que les femmes noires ont été oubliées à la fois par le mouvement féministe, dominé par des femmes blanches de classe moyenne, et par le mouvement pour les droits civiques, dominé par des hommes. Elle développe l'idée que le sexisme, le racisme et l'exploitation économique forment un même système de domination, qu'elle appelle le « patriarcat capitaliste suprémaciste blanc ».&lt;/p&gt; &lt;p&gt;Ses idées ont profondément influencé ce que l'on appelle aujourd'hui l'intersectionnalité, c'est-à-dire l'étude de la manière dont différentes formes de discrimination se croisent et se renforcent. Elle écrivait dans un style simple et direct, refusant le jargon universitaire, pour que ses livres soient lus au-delà des cercles savants. Elle a aussi consacré plusieurs ouvrages à l'amour, qu'elle considérait comme une force politique capable de transformer la société.&lt;/p&gt; &lt;p&gt;Elle a écrit une quarantaine de livres, sur le féminisme, l'amour, les médias, la culture populaire et l'éducation. Dans &lt;em&gt;Apprendre à transgresser&lt;/em&gt; (1994), inspirée par Paulo Freire, elle défend une pédagogie de la liberté où l'enseignement devient une pratique d'émancipation. Pour elle, le féminisme n'est pas une guerre contre les hommes mais un mouvement pour mettre fin à toute forme de domination, porté par une « éthique de l'amour ».&lt;/p&gt;</t>
+    <t xml:space="preserve">Bell HOOKS</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Bell_hooks"  title=" Wikipedia"&gt;Bell HOOKS&lt;/a&gt; , de son vrai nom Gloria Jean Watkins, est une autrice, professeure et militante féministe afro-américaine. Née dans le Kentucky, dans le Sud ségrégationniste, elle prit le nom de son arrière-grand-mère, qu'elle écrivait en minuscules pour que l'attention se porte sur ses idées plutôt que sur sa personne.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Ne suis-je pas une femme ?&lt;/em&gt; (1981), elle montre que les femmes noires ont été oubliées à la fois par le mouvement féministe, dominé par des femmes blanches de classe moyenne, et par le mouvement pour les droits civiques, dominé par des hommes. Elle </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve"> &lt;a href="https://www.youtube.com/watch?v=pCwMdHBSQgM" title=" bell hooks, un féminisme anticapitaliste et intersectionnel par META "&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">développe l'idée &lt;/a&gt; que le sexisme, le racisme et l'exploitation économique forment un même système de domination, qu'elle appelle le « patriarcat capitaliste suprémaciste blanc ».&lt;/p&gt; &lt;p&gt;Ses idées ont profondément influencé ce que l'on appelle aujourd'hui l'intersectionnalité, c'est-à-dire l'étude de la manière dont différentes formes de discrimination se croisent et se renforcent. Elle écrivait dans un style simple et direct, refusant le jargon universitaire, pour que ses livres soient lus au-delà des cercles savants. Elle a aussi consacré plusieurs ouvrages à l'amour, qu'elle considérait comme une force politique capable de transformer la société.&lt;/p&gt; &lt;p&gt;Elle a écrit une quarantaine de livres, sur le féminisme, l'amour, les médias, la culture populaire et l'éducation. Dans &lt;em&gt;Apprendre à transgresser&lt;/em&gt; (1994), inspirée par Paulo Freire, elle défend une pédagogie de la liberté où l'enseignement devient une pratique d'émancipation. Pour elle, le féminisme n'est pas une guerre contre les hommes mais un mouvement pour mettre fin à toute forme de domination, porté par une « éthique de l'amour ».&lt;/p&gt;  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">  &lt;audio controls title="Lire bell hooks aujourd’hui par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/23875-15.11.2023-ITEMA_23552434-2023C49162S0319-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;  
+</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">IFFd_Zqo5cc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L’amour, selon bell hooks par France Culture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.laphilo.fr/pho/bhooks-mini.webp</t>
   </si>
   <si>
     <t xml:space="preserve">Féminisme</t>
@@ -1593,7 +1641,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1683,6 +1731,7 @@
       <sz val="9"/>
       <name val="Microsoft YaHei"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1711,6 +1760,18 @@
       <name val="Georgia"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1793,71 +1854,71 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2113,7 +2174,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFD59"/>
+  <dimension ref="A1:P1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.06"/>
@@ -2126,9 +2187,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="26.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="8.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="20.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="2" width="28.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="2" width="23.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="2" width="26.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="16.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="11.53"/>
   </cols>
   <sheetData>
@@ -2246,10 +2308,10 @@
       <c r="M4" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N4" s="0" t="s">
+      <c r="N4" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P4" s="0" t="s">
+      <c r="P4" s="1" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2288,10 +2350,10 @@
       <c r="L5" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="N5" s="0" t="s">
+      <c r="N5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P5" s="0" t="s">
+      <c r="P5" s="1" t="s">
         <v>40</v>
       </c>
     </row>
@@ -2330,7 +2392,7 @@
       <c r="L6" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="N6" s="0" t="s">
+      <c r="N6" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2369,10 +2431,10 @@
       <c r="L7" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="N7" s="0" t="s">
+      <c r="N7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P7" s="0" t="s">
+      <c r="P7" s="1" t="s">
         <v>62</v>
       </c>
     </row>
@@ -2411,7 +2473,7 @@
       <c r="L8" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="N8" s="0" t="s">
+      <c r="N8" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2450,7 +2512,7 @@
       <c r="L9" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="N9" s="0" t="s">
+      <c r="N9" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2489,7 +2551,7 @@
       <c r="L10" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="N10" s="0" t="s">
+      <c r="N10" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2528,7 +2590,7 @@
       <c r="L11" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="N11" s="0" t="s">
+      <c r="N11" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2567,7 +2629,7 @@
       <c r="L12" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="N12" s="0" t="s">
+      <c r="N12" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2606,10 +2668,10 @@
       <c r="L13" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="N13" s="0" t="s">
+      <c r="N13" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P13" s="0" t="s">
+      <c r="P13" s="1" t="s">
         <v>62</v>
       </c>
     </row>
@@ -2648,10 +2710,10 @@
       <c r="L14" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="N14" s="0" t="s">
+      <c r="N14" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P14" s="0" t="s">
+      <c r="P14" s="1" t="s">
         <v>130</v>
       </c>
     </row>
@@ -2690,10 +2752,10 @@
       <c r="L15" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="N15" s="0" t="s">
+      <c r="N15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P15" s="0" t="s">
+      <c r="P15" s="1" t="s">
         <v>140</v>
       </c>
     </row>
@@ -2732,7 +2794,7 @@
       <c r="L16" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="N16" s="0" t="s">
+      <c r="N16" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2771,10 +2833,10 @@
       <c r="L17" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="N17" s="0" t="s">
+      <c r="N17" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P17" s="0" t="s">
+      <c r="P17" s="1" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2813,10 +2875,10 @@
       <c r="L18" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="N18" s="0" t="s">
+      <c r="N18" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P18" s="0" t="s">
+      <c r="P18" s="1" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2858,7 +2920,7 @@
       <c r="M19" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="N19" s="0" t="s">
+      <c r="N19" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2897,10 +2959,10 @@
       <c r="L20" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="N20" s="0" t="s">
+      <c r="N20" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P20" s="0" t="s">
+      <c r="P20" s="1" t="s">
         <v>62</v>
       </c>
     </row>
@@ -2939,10 +3001,10 @@
       <c r="L21" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="N21" s="0" t="s">
+      <c r="N21" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P21" s="0" t="s">
+      <c r="P21" s="1" t="s">
         <v>193</v>
       </c>
     </row>
@@ -2981,7 +3043,7 @@
       <c r="M22" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N22" s="0" t="s">
+      <c r="N22" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3020,7 +3082,7 @@
       <c r="L23" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="N23" s="0" t="s">
+      <c r="N23" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3059,10 +3121,10 @@
       <c r="L24" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="N24" s="0" t="s">
+      <c r="N24" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P24" s="0" t="s">
+      <c r="P24" s="1" t="s">
         <v>30</v>
       </c>
     </row>
@@ -3104,7 +3166,7 @@
       <c r="M25" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="N25" s="0" t="s">
+      <c r="N25" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3146,7 +3208,7 @@
       <c r="M26" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="N26" s="0" t="s">
+      <c r="N26" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3187,7 +3249,7 @@
       <c r="M27" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="N27" s="0" t="s">
+      <c r="N27" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3229,7 +3291,7 @@
       <c r="M28" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="N28" s="0" t="s">
+      <c r="N28" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3271,10 +3333,10 @@
       <c r="M29" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="N29" s="0" t="s">
+      <c r="N29" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="O29" s="0" t="n">
+      <c r="O29" s="1" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3316,7 +3378,7 @@
       <c r="M30" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="N30" s="0" t="s">
+      <c r="N30" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3355,7 +3417,7 @@
       <c r="L31" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="N31" s="0" t="s">
+      <c r="N31" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3394,10 +3456,10 @@
       <c r="L32" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="N32" s="0" t="s">
+      <c r="N32" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P32" s="0" t="s">
+      <c r="P32" s="1" t="s">
         <v>30</v>
       </c>
     </row>
@@ -3436,7 +3498,7 @@
       <c r="L33" s="14" t="s">
         <v>304</v>
       </c>
-      <c r="N33" s="0" t="s">
+      <c r="N33" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3475,7 +3537,7 @@
       <c r="L34" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="N34" s="0" t="s">
+      <c r="N34" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3517,7 +3579,7 @@
       <c r="M35" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="N35" s="0" t="s">
+      <c r="N35" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3556,7 +3618,7 @@
       <c r="L36" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="N36" s="0" t="s">
+      <c r="N36" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3598,7 +3660,7 @@
       <c r="M37" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="N37" s="0" t="s">
+      <c r="N37" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3640,7 +3702,7 @@
       <c r="M38" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="N38" s="0" t="s">
+      <c r="N38" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3682,7 +3744,7 @@
       <c r="M39" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="N39" s="0" t="s">
+      <c r="N39" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3724,7 +3786,7 @@
       <c r="M40" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="N40" s="0" t="s">
+      <c r="N40" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3763,7 +3825,7 @@
       <c r="L41" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="N41" s="0" t="s">
+      <c r="N41" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3802,7 +3864,7 @@
       <c r="L42" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="N42" s="0" t="s">
+      <c r="N42" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3825,10 +3887,10 @@
       <c r="F43" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="G43" s="1" t="s">
+      <c r="G43" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="H43" s="1" t="s">
+      <c r="H43" s="2" t="s">
         <v>389</v>
       </c>
       <c r="I43" s="1"/>
@@ -3838,13 +3900,13 @@
       <c r="K43" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="L43" s="1" t="s">
+      <c r="L43" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="N43" s="0" t="s">
+      <c r="N43" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="P43" s="0" t="s">
+      <c r="P43" s="1" t="s">
         <v>392</v>
       </c>
     </row>
@@ -3881,7 +3943,7 @@
       <c r="L44" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="N44" s="0" t="s">
+      <c r="N44" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3920,13 +3982,13 @@
       <c r="L45" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="N45" s="0" t="s">
+      <c r="N45" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O45" s="0" t="n">
+      <c r="O45" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="P45" s="0" t="s">
+      <c r="P45" s="1" t="s">
         <v>62</v>
       </c>
     </row>
@@ -3965,7 +4027,7 @@
       <c r="L46" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="N46" s="0" t="s">
+      <c r="N46" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -4046,7 +4108,7 @@
       <c r="L48" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="N48" s="0" t="s">
+      <c r="N48" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -4127,7 +4189,7 @@
       <c r="L50" s="2" t="s">
         <v>448</v>
       </c>
-      <c r="N50" s="0" t="s">
+      <c r="N50" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -4150,10 +4212,10 @@
       <c r="F51" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="G51" s="1" t="s">
+      <c r="G51" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="H51" s="1" t="s">
+      <c r="H51" s="2" t="s">
         <v>454</v>
       </c>
       <c r="J51" s="1" t="s">
@@ -4162,20 +4224,18 @@
       <c r="K51" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="L51" s="1" t="s">
+      <c r="L51" s="2" t="s">
         <v>457</v>
       </c>
       <c r="M51" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="N51" s="0" t="s">
+      <c r="N51" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="P51" s="0" t="s">
+      <c r="P51" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="XFC51" s="0"/>
-      <c r="XFD51" s="0"/>
     </row>
     <row r="52" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="n">
@@ -4212,7 +4272,7 @@
       <c r="L52" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="N52" s="0" t="s">
+      <c r="N52" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -4251,7 +4311,7 @@
       <c r="L53" s="2" t="s">
         <v>475</v>
       </c>
-      <c r="N53" s="0" t="s">
+      <c r="N53" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -4293,7 +4353,7 @@
       <c r="M54" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N54" s="0" t="s">
+      <c r="N54" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -4334,83 +4394,68 @@
       <c r="M55" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N55" s="0" t="s">
+      <c r="N55" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E56" s="14"/>
-    </row>
-    <row r="57" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="1" t="n">
+    <row r="56" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="n">
         <v>1952</v>
       </c>
-      <c r="B57" s="1" t="n">
+      <c r="B56" s="1" t="n">
         <v>2021</v>
       </c>
-      <c r="C57" s="1" t="s">
+      <c r="C56" s="1" t="s">
         <v>491</v>
       </c>
-      <c r="D57" s="1" t="s">
+      <c r="D56" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="E57" s="2" t="s">
+      <c r="E56" s="2" t="s">
         <v>493</v>
       </c>
-      <c r="G57" s="1"/>
-      <c r="H57" s="1"/>
+      <c r="F56" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="I56" s="1"/>
+      <c r="J56" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K56" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="L56" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="M56" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="N56" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="O56" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="293.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E57" s="1"/>
       <c r="I57" s="1"/>
-      <c r="J57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="K57" s="1" t="s">
-        <v>494</v>
-      </c>
-      <c r="L57" s="1" t="s">
-        <v>495</v>
-      </c>
-      <c r="M57" s="1" t="s">
-        <v>496</v>
-      </c>
-      <c r="N57" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="O57" s="0" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="293.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="0"/>
-      <c r="B58" s="0"/>
-      <c r="C58" s="0"/>
-      <c r="D58" s="0"/>
-      <c r="E58" s="0"/>
-      <c r="F58" s="0"/>
-      <c r="G58" s="0"/>
-      <c r="H58" s="0"/>
-      <c r="I58" s="0"/>
-      <c r="J58" s="0"/>
-      <c r="K58" s="0"/>
-      <c r="L58" s="0"/>
-      <c r="M58" s="0"/>
-      <c r="XFC58" s="0"/>
-      <c r="XFD58" s="0"/>
-    </row>
-    <row r="59" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="0"/>
-      <c r="B59" s="0"/>
-      <c r="C59" s="0"/>
-      <c r="D59" s="0"/>
-      <c r="E59" s="0"/>
-      <c r="F59" s="0"/>
-      <c r="G59" s="0"/>
-      <c r="H59" s="0"/>
-      <c r="I59" s="0"/>
-      <c r="J59" s="0"/>
-      <c r="K59" s="0"/>
-      <c r="L59" s="0"/>
-      <c r="M59" s="0"/>
-    </row>
+      <c r="J57" s="1"/>
+      <c r="K57" s="1"/>
+    </row>
+    <row r="58" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E58" s="1"/>
+      <c r="I58" s="1"/>
+      <c r="J58" s="1"/>
+      <c r="K58" s="1"/>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
@@ -4454,6 +4499,7 @@
     <hyperlink ref="H48" r:id="rId35" display="https://www.laphilo.fr/pho/rmadams-mini.webp"/>
     <hyperlink ref="E49" r:id="rId36" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Robert_Nozick&quot;  title=&quot; Wikipedia&quot;&gt;Robert NOZICK&lt;/a&gt; était un philosophe américain connu pour &lt;a href=&quot;https://www.youtube.com/watch?v=Q-t3cpFAk4o&quot;  title=&quot; Libertarianisme par Vadim Media&quot;&gt; son libertarianisme &lt;/a&gt; et sa critique des théories égalitaristes comme celle de John Rawls. Professeur à Harvard, il a marqué la philosophie politique, morale et épistémologique par son œuvre principale, Anarchie, État et utopie (1974), qui défend un  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Minarchisme&quot;  title=&quot; Minarchisme par Wikipédia&quot;&gt; Etat Minimal. &lt;/a&gt; &lt;/p&gt; &lt;p&gt; Il argue que seul l'État minimal, ou &quot;État gardien de nuit&quot;, est légitime, car il se limite à protéger les individus contre la force, la fraude et le vol, sans redistribuer les richesses. Il rejette l'anarcho-capitalisme en montrant, via des agences de protection privée, comment un État dominant émerge naturellement pour monopoliser la coercition légitime, justifié par le droit naturel à la personne. &lt;/p&gt; &lt;p&gt; Contrairement à la justice distributive de Rawls, il propose une théorie de l'entitlement : une acquisition initiale juste et des transferts volontaires rendent la distribution légitime, sans besoin d'égalisation par l'État. Toute intervention redistributive viole les droits individuels, traitant les personnes comme des moyens plutôt que des fins, en écho à Kant. &lt;/p&gt; &lt;p&gt; Dans Anarchie, État et utopie, Il réfute l'utilitarisme via l'expérience de pensée de la &lt;a href=&quot;https://www.youtube.com/watch?v=2FVwXaNWPQ0&quot;  title=&quot; La machine à expérience par Monsieur Phi&quot;&gt;&quot;machine à expérience&quot; :&lt;/a&gt;  même si elle offre un bonheur parfait et indistinguable de la réalité, les gens préfèrent vivre des actions réelles et façonner leur identité plutôt que des simulations. Cela prouve que le bonheur n'est pas le seul bien suprême. &lt;/p&gt; &lt;p&gt; Plus tard, dans Explications philosophiques (1981), il développe une théorie du suivi (tracking theory) en épistémologie, où la connaissance repose sur des conditionnels contrefactuels fiables, contournant le scepticisme sans justification traditionnelle. Son anti-coercitivisme intellectuel invite à une philosophie ouverte, non imposée. &lt;/p&gt; &#10;&lt;audio controls title=&quot;Qui a peur des Libertariens par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10467-14.06.2022-ITEMA_23058436-2022C12410S0165-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt;&lt;/audio&gt;&#10;"/>
     <hyperlink ref="H55" r:id="rId37" display="https://www.laphilo.fr/pho/imyoung-mini.webp"/>
+    <hyperlink ref="H56" r:id="rId38" display="https://www.laphilo.fr/pho/bhooks-mini.webp"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Amériques & Caraïbes : Guamán Poma, Martí, C. L. R. James, Freire, Glissant, Sylvia Wynter ; carte « Caraïbes » ; Hispaniques élargis (Cuba…) ; bandeau compact du panneau des liens dans les frises ; portrait Biko
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-americains.xlsx
+++ b/data/frise-philosophes-americains.xlsx
@@ -2237,7 +2237,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFD59"/>
+  <dimension ref="A1:XFD60"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.06"/>
@@ -4554,24 +4554,183 @@
       </c>
     </row>
     <row r="58" customFormat="false" ht="293.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="0"/>
-      <c r="B58" s="0"/>
-      <c r="C58" s="0"/>
-      <c r="D58" s="0"/>
-      <c r="E58" s="0"/>
+      <c r="A58" s="0">
+        <v>1535</v>
+      </c>
+      <c r="B58" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1616</t>
+        </is>
+      </c>
+      <c r="C58" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 1535 – vers 1616</t>
+        </is>
+      </c>
+      <c r="D58" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Felipe GUAMÁN POMA de Ayala</t>
+        </is>
+      </c>
+      <c r="E58" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Felipe_Guam%C3%A1n_Poma_de_Ayala" title=" Wikipedia"&gt;Felipe GUAMÁN POMA de Ayala&lt;/a&gt; est un noble andin de langue quechua, auteur de l’un des documents les plus extraordinaires de l’époque coloniale. Né dans la province de Lucanas, au Pérou, peu après la conquête espagnole, il descend par sa mère d’une lignée liée aux souverains de l’&lt;a href="https://fr.wikipedia.org/wiki/Empire_inca" title=" Wikipedia"&gt;Empire inca&lt;/a&gt;. Élevé parmi les Espagnols, il apprend leur langue, se fait chrétien et travaille comme interprète auprès d’un prêtre chargé d’extirper les « idolâtries », puis auprès de juges de Huamanga, avant d’être dépouillé de ses terres et banni vers 1600.&lt;/p&gt; &lt;p&gt;Il parcourt alors les Andes pendant des années et rédige, vers 1615, une lettre de près de 1 200 pages adressée au roi d’Espagne Philippe III : la &lt;em&gt;Nouvelle Chronique et bon gouvernement&lt;/em&gt;. Ses quelque 400 dessins à la plume racontent l’histoire des Incas, le calendrier, les travaux des champs, puis les abus des colons : prêtres, corregidors et propriétaires qui exploitent, volent et maltraitent les Indiens. Il y décrit un « monde à l’envers » (&lt;em&gt;mundo al revés&lt;/em&gt;), où l’ordre juste a été renversé par la conquête.&lt;/p&gt; &lt;p&gt;Il ne réclame pas le départ des Espagnols, mais un « bon gouvernement » : que les Andins se gouvernent eux-mêmes sous l’autorité lointaine du roi, et que les colons qui abusent soient chassés des villages. Il défend aussi la valeur de la civilisation andine, qui connaissait selon lui la justice et un ordre moral bien avant l’arrivée des Européens. Le manuscrit, qui n’atteignit sans doute jamais le roi, dormit pendant trois siècles avant d’être découvert en 1908 à la Bibliothèque royale de Copenhague. Il est aujourd’hui une source majeure sur le monde andin et l’une des premières critiques de la colonisation écrites par un colonisé.&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="F58" s="0"/>
       <c r="G58" s="0"/>
-      <c r="H58" s="0"/>
+      <c r="H58" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/guamanpoma-mini.webp</t>
+        </is>
+      </c>
       <c r="I58" s="0"/>
-      <c r="J58" s="0"/>
-      <c r="K58" s="0"/>
-      <c r="L58" s="0"/>
+      <c r="J58" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">politique ; ethique</t>
+        </is>
+      </c>
+      <c r="K58" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anticolonialisme</t>
+        </is>
+      </c>
+      <c r="L58" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chroniqueur andin, auteur d’une immense lettre illustrée au roi d’Espagne dénonçant la colonisation du Pérou.</t>
+        </is>
+      </c>
       <c r="M58" s="0"/>
-      <c r="P58" s="0"/>
+      <c r="N58" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="O58" s="1">
+        <v>2</v>
+      </c>
+      <c r="P58" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Péruvienne</t>
+        </is>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1">
+        <v>1853</v>
+      </c>
+      <c r="B59" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1895</t>
+        </is>
+      </c>
+      <c r="C59" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1853 – 1895</t>
+        </is>
+      </c>
+      <c r="D59" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">José MARTÍ</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jos%C3%A9_Mart%C3%AD" title=" Wikipedia"&gt;José MARTÍ&lt;/a&gt; est le grand penseur de l’indépendance cubaine et l’une des voix majeures de l’Amérique latine. Né à La Havane de parents espagnols, il est arrêté à seize ans pour ses idées indépendantistes et condamné aux travaux forcés dans une carrière, avant d’être déporté en Espagne, où il étudie le droit et la philosophie à Saragosse. Il vit ensuite au Mexique, au Guatemala et au Venezuela, puis s’installe en 1881 à New York, où il passe près de quinze ans comme journaliste, diplomate et organisateur de l’exil cubain. Il y écrit, pour de grands journaux d’Amérique latine, des chroniques sur la vie nord-américaine.&lt;/p&gt; &lt;p&gt;Dans son essai &lt;em&gt;Notre Amérique&lt;/em&gt; (1891), il appelle les nations latino-américaines à se penser à partir de leur propre réalité, métisse, indienne, noire et paysanne, plutôt qu’en copiant l’Europe ou les États-Unis : « Le gouvernement doit naître du pays. » Il y affirme aussi : « Il n’y a pas de haine des races, parce qu’il n’y a pas de races. » Observateur lucide de la puissance nord-américaine, il met en garde contre les ambitions des États-Unis sur Cuba et sur tout le continent.&lt;/p&gt; &lt;p&gt;Poète novateur, l’un des fondateurs du modernisme hispanique, il écrit les &lt;em&gt;Vers simples&lt;/em&gt; (1891), dont certains forment les paroles de la célèbre chanson &lt;em&gt;Guantanamera&lt;/em&gt;, et une revue pour les enfants, &lt;em&gt;L’Âge d’or&lt;/em&gt;. En 1892, il fonde le Parti révolutionnaire cubain et prépare la &lt;a href="https://fr.wikipedia.org/wiki/Guerre_d%27ind%C3%A9pendance_cubaine" title=" Wikipedia"&gt;guerre d’indépendance&lt;/a&gt;. Débarqué à Cuba avec les insurgés, il est tué au combat à Dos Ríos le 19 mai 1895. Il est considéré à Cuba comme le héros national et « l’Apôtre » de l’indépendance.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/marti-mini.webp</t>
+        </is>
+      </c>
       <c r="I59" s="1"/>
-      <c r="K59" s="1"/>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">politique ; esthetique</t>
+        </is>
+      </c>
+      <c r="K59" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anticolonialisme ; Humanisme</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">poète et penseur de l’indépendance cubaine, auteur de « Notre Amérique », héros national de Cuba.</t>
+        </is>
+      </c>
+      <c r="N59" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="O59" s="1">
+        <v>2</v>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cubaine</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1">
+        <v>1921</v>
+      </c>
+      <c r="B60" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1997</t>
+        </is>
+      </c>
+      <c r="C60" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1921 – 1997</t>
+        </is>
+      </c>
+      <c r="D60" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paulo FREIRE</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Paulo_Freire" title=" Wikipedia"&gt;Paulo FREIRE&lt;/a&gt; est un pédagogue et philosophe brésilien, l’un des penseurs de l’éducation les plus lus au monde. Né à Recife, dans le Nordeste, il connaît la faim pendant la crise des années 1930, ce qui le marque pour toute sa vie. Formé au droit et à la philosophie, lecteur de Marx comme des penseurs chrétiens, il se consacre à l’&lt;a href="https://fr.wikipedia.org/wiki/Alphab%C3%A9tisation" title=" Wikipedia"&gt;alphabétisation&lt;/a&gt; des adultes pauvres. En 1963, à Angicos, sa méthode permet à 300 travailleurs agricoles d’apprendre à lire et à écrire en une quarantaine d’heures.&lt;/p&gt; &lt;p&gt;Sa méthode part des « mots générateurs » tirés de la vie des apprenants, comme la brique, la terre ou le salaire, et fait de la lecture une prise de conscience : apprendre à lire le mot, c’est apprendre à lire le monde. Après le coup d’État militaire de 1964, il est emprisonné puis contraint à un exil de seize ans. Au Chili, il écrit &lt;a href="https://fr.wikipedia.org/wiki/P%C3%A9dagogie_des_opprim%C3%A9s" title=" Wikipedia"&gt;&lt;em&gt;Pédagogie des opprimés&lt;/em&gt;&lt;/a&gt; (1968), où il critique l’éducation « bancaire », qui dépose des savoirs dans des élèves passifs comme on remplit un coffre, et lui oppose une éducation par le dialogue, où maître et élèves cherchent ensemble.&lt;/p&gt; &lt;p&gt;« Personne n’éduque autrui, personne ne s’éduque seul, les hommes s’éduquent ensemble par l’intermédiaire du monde. » L’éducation n’est jamais neutre : elle maintient l’oppression ou aide les opprimés à s’en libérer, sans devenir à leur tour oppresseurs. Rentré au Brésil en 1980, il dirige l’éducation de la ville de São Paulo. Son œuvre est à l’origine de la &lt;a href="https://fr.wikipedia.org/wiki/P%C3%A9dagogie_critique" title=" Wikipedia"&gt;pédagogie critique&lt;/a&gt;, et il a été proclamé en 2012 patron de l’éducation brésilienne.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/freire-mini.webp</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ethique ; politique</t>
+        </is>
+      </c>
+      <c r="K60" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Humanisme ; Marxisme</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pédagogue brésilien, auteur de Pédagogie des opprimés, penseur de l’éducation comme pratique de la liberté.</t>
+        </is>
+      </c>
+      <c r="N60" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="O60" s="1">
+        <v>3</v>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brésilienne</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Lots 8 « Sud » et 9 « Europe de l'Est » (19 fiches) : Walda Heywat, Hostos, Black Elk, Taha, Ki-Zerbo, Fals Borda, Maturana, Varela, Okot p'Bitek, Cordova, Hau'ofa, Soyinka, Rivera Cusicanqui, Kazantzákis, Ingarden, Patočka, Eliade, Kołakowski, Havel ; éditeur : fenêtre d'application, liste repliable
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-americains.xlsx
+++ b/data/frise-philosophes-americains.xlsx
@@ -2237,7 +2237,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFD67"/>
+  <dimension ref="A1:XFD71"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.06"/>
@@ -5140,6 +5140,248 @@
       <c r="P67" t="inlineStr">
         <is>
           <t xml:space="preserve">Péruvienne</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="1">
+        <v>1839</v>
+      </c>
+      <c r="B68" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1903</t>
+        </is>
+      </c>
+      <c r="C68" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1839 – 1903</t>
+        </is>
+      </c>
+      <c r="D68" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eugenio María de HOSTOS</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Eugenio_Mar%C3%ADa_de_Hostos" title=" Wikipedia (en)"&gt;Eugenio María de HOSTOS&lt;/a&gt; est un philosophe, éducateur, sociologue et écrivain de &lt;a href="https://fr.wikipedia.org/wiki/Porto_Rico" title=" Wikipedia"&gt;Porto Rico&lt;/a&gt;, surnommé « le Grand Citoyen des Amériques ». Né à Mayagüez dans une famille aisée, il fait ses études en Espagne, où il étudie le droit et la philosophie à Madrid et publie en 1863 un roman, &lt;em&gt;Le Pèlerinage de Bayoán&lt;/em&gt;, qui évoque déjà le destin des Antilles. Déçu que la République espagnole refuse l’autonomie de Porto Rico, il quitte l’Espagne en 1869 pour se consacrer à l’indépendance des colonies antillaises.&lt;/p&gt; &lt;p&gt;Il rêve d’une Confédération des Antilles, réunissant Porto Rico, Cuba et la République dominicaine, et parcourt pour la défendre les États-Unis, le Pérou, le Chili, l’Argentine, le Brésil et le Venezuela. Partout, il fonde ou réforme des écoles. En République dominicaine, il crée en 1880 la première école normale, qui forme des instituteurs à une pédagogie scientifique et laïque. Au Chili, il plaide pour que les femmes aient accès à l’enseignement supérieur et aux professions savantes.&lt;/p&gt; &lt;p&gt;Sa &lt;em&gt;Morale sociale&lt;/em&gt; (1888), inspirée du &lt;a href="https://fr.wikipedia.org/wiki/Positivisme" title=" Wikipedia"&gt;positivisme&lt;/a&gt;, fonde les devoirs de l’individu non sur la religion, mais sur la raison et sur les liens qui l’unissent à la famille, à la société et à l’humanité ; l’éducation doit former des consciences libres et responsables. Après la guerre de 1898, qui fait passer Porto Rico sous domination américaine, il milite pour que l’île puisse décider elle-même de son avenir. Il laisse aussi un traité de sociologie, l’un des premiers d’Amérique latine. Il meurt en exil à Saint-Domingue en 1903.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/hostos-mini.webp</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ethique ; politique</t>
+        </is>
+      </c>
+      <c r="K68" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivisme</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">éducateur et penseur portoricain, apôtre d’une confédération des Antilles et d’une morale sociale laïque.</t>
+        </is>
+      </c>
+      <c r="N68" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="O68" s="1">
+        <v>2</v>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portoricaine</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="1">
+        <v>1925</v>
+      </c>
+      <c r="B69" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2008</t>
+        </is>
+      </c>
+      <c r="C69" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1925 – 2008</t>
+        </is>
+      </c>
+      <c r="D69" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Orlando FALS BORDA</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Orlando_Fals_Borda" title=" Wikipedia (en)"&gt;Orlando FALS BORDA&lt;/a&gt; est un sociologue colombien, l’un des grands penseurs latino-américains des sciences sociales et le fondateur de la « recherche-action participative ». Né à Barranquilla, sur la côte caraïbe, formé aux États-Unis, il fonde en 1959 à l’Université nationale de Colombie, avec le prêtre Camilo Torres, l’une des premières facultés de sociologie d’Amérique latine. Son livre &lt;em&gt;La Violence en Colombie&lt;/em&gt; (1962), écrit avec Germán Guzmán et Eduardo Umaña, étudie pour la première fois la guerre civile qui ravage les campagnes.&lt;/p&gt; &lt;p&gt;Déçu par une sociologie qui observe les pauvres de l’extérieur sans rien changer à leur sort, il quitte l’université dans les années 1970 pour travailler avec les paysans et les communautés de la côte caraïbe. Il y développe la &lt;a href="https://fr.wikipedia.org/wiki/Recherche-action" title=" Wikipedia"&gt;recherche-action&lt;/a&gt; participative : le chercheur ne doit pas monopoliser le savoir ni imposer sa technique, mais travailler avec les communautés comme avec des partenaires et des co-chercheurs, recueillir leurs savoirs, leur mémoire et leurs récits, et partager les résultats sous une forme que tous peuvent comprendre.&lt;/p&gt; &lt;p&gt;La science n’est pas, selon lui, une affaire d’experts neutres : elle doit servir la transformation de la société et la libération des opprimés. Il parle d’une « subversion positive » qui conteste l’ordre injuste pour en construire un meilleur. Ses idées se sont répandues dans le monde entier, en éducation, en santé et en développement. Il participe aussi à l’Assemblée constituante qui rédige la Constitution colombienne de 1991. Il meurt à Bogotá en 2008.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/falsborda-mini.webp</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">epistemologie ; politique</t>
+        </is>
+      </c>
+      <c r="K69" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tiers-mondisme</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sociologue colombien, fondateur de la recherche-action participative, penseur d’un savoir construit avec le peuple.</t>
+        </is>
+      </c>
+      <c r="N69" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="O69" s="1">
+        <v>2</v>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Colombienne</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="1">
+        <v>1928</v>
+      </c>
+      <c r="B70" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2021</t>
+        </is>
+      </c>
+      <c r="C70" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1928 – 2021</t>
+        </is>
+      </c>
+      <c r="D70" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Humberto MATURANA</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Humberto_Maturana" title=" Wikipedia"&gt;Humberto MATURANA&lt;/a&gt; est un biologiste et philosophe chilien, l’un des penseurs les plus originaux de la biologie de la connaissance. Né à Santiago, il étudie la médecine et la biologie au Chili, puis en Angleterre et à Harvard. Au Massachusetts Institute of Technology, il participe en 1959 à une étude devenue célèbre sur ce que l’œil de la grenouille transmet à son cerveau, qui montre que la perception n’est pas une simple copie du monde extérieur. Il fonde ensuite à l’université du Chili un laboratoire d’« épistémologie expérimentale ».&lt;/p&gt; &lt;p&gt;Avec son élève Francisco Varela, il propose au début des années 1970 le concept d’&lt;a href="https://fr.wikipedia.org/wiki/Autopo%C3%AF%C3%A8se" title=" Wikipedia"&gt;autopoïèse&lt;/a&gt;, du grec « se produire soi-même » : un être vivant est un système qui produit et renouvelle sans cesse ses propres composants, et maintient ainsi sa propre organisation. La cellule en est le modèle. Le vivant n’est donc pas défini par ce qu’il contient, mais par cette manière de s’entretenir lui-même, en échange constant avec son milieu.&lt;/p&gt; &lt;p&gt;Il en tire une théorie de la connaissance : « Tout ce qui est dit est dit par un observateur. » Connaître n’est pas refléter un monde tout fait, mais une activité du vivant, qui fait émerger un monde à travers son action. Dans &lt;em&gt;L’Arbre de la connaissance&lt;/em&gt; (1984), écrit avec Varela, il montre aussi que le langage et la société naissent de la coordination entre les êtres, et que l’amour, l’acceptation de l’autre, est le fondement biologique de la vie sociale. Ses idées ont nourri le &lt;a href="https://fr.wikipedia.org/wiki/Constructivisme_%28%C3%A9pist%C3%A9mologie%29" title=" Wikipedia"&gt;constructivisme&lt;/a&gt;, la thérapie familiale et la théorie des systèmes sociaux de &lt;a href="https://fr.wikipedia.org/wiki/Niklas_Luhmann" title=" Wikipedia"&gt;Niklas Luhmann&lt;/a&gt;. Il meurt à Santiago en 2021.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/maturana-mini.webp</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">epistemologie ; metaphysique</t>
+        </is>
+      </c>
+      <c r="K70" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Constructivisme</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">biologiste et philosophe chilien, inventeur avec Varela de l’autopoïèse, penseur de la connaissance comme fait biologique.</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="N70" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O70" s="1">
+        <v>2</v>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chilienne</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="1">
+        <v>1946</v>
+      </c>
+      <c r="B71" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2001</t>
+        </is>
+      </c>
+      <c r="C71" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1946 – 2001</t>
+        </is>
+      </c>
+      <c r="D71" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Francisco VARELA</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Francisco_Varela" title=" Wikipedia"&gt;Francisco VARELA&lt;/a&gt; est un biologiste, neuroscientifique et philosophe chilien, l’un des fondateurs des sciences cognitives « incarnées ». Né à Talcahuano, élève d’Humberto Maturana, il soutient une thèse de biologie à Harvard, puis invente avec son maître le concept d’&lt;a href="https://fr.wikipedia.org/wiki/Autopo%C3%AF%C3%A8se" title=" Wikipedia"&gt;autopoïèse&lt;/a&gt;, qui définit le vivant par sa capacité à se produire lui-même. Après le coup d’État de Pinochet en 1973, il doit s’exiler aux États-Unis. Il s’installe en France en 1986 et dirige jusqu’à sa mort une équipe de recherche au CNRS, à Paris.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;L’Inscription corporelle de l’esprit&lt;/em&gt; (1991), écrit avec Evan Thompson et Eleanor Rosch, il critique l’idée que l’esprit serait un ordinateur qui traite des représentations d’un monde extérieur déjà donné. Il propose à la place l’« &lt;a href="https://fr.wikipedia.org/wiki/%C3%89naction" title=" Wikipedia"&gt;énaction&lt;/a&gt; » : la cognition est une action incarnée, par laquelle un être vivant fait émerger son monde à travers son corps, ses sens et ses gestes. Il fonde aussi la « neurophénoménologie », qui veut unir les mesures du cerveau et la description rigoureuse de l’expérience vécue, à la manière de Husserl et de Merleau-Ponty.&lt;/p&gt; &lt;p&gt;Pratiquant du bouddhisme tibétain depuis les années 1970, il voit dans la méditation une méthode précise pour explorer l’expérience. En 1987, il cofonde le &lt;a href="https://fr.wikipedia.org/wiki/Mind_and_Life_Institute" title=" Wikipedia"&gt;Mind and Life Institute&lt;/a&gt;, qui organise des rencontres entre scientifiques et le dalaï-lama. Il est l’un des inspirateurs de l’idée d’un esprit « incarné », aujourd’hui centrale en &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_l%27esprit" title=" Wikipedia"&gt;philosophie de l’esprit&lt;/a&gt;. Il meurt à Paris en 2001, à cinquante-quatre ans, d’une maladie du foie.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/varela-mini.webp</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">epistemologie ; metaphysique</t>
+        </is>
+      </c>
+      <c r="K71" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Constructivisme ; Phénoménologie</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">neurobiologiste et philosophe chilien, penseur de l’énaction et du dialogue entre sciences cognitives et bouddhisme.</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="N71" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O71" s="1">
+        <v>2</v>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chilienne</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fiches — 1 fiche nouvelle : Aldous HUXLEY ; 9 fiches modifiées : Arthur SCHOPENHAUER, Ayn RAND, HÉLOÏSE, Karl POPPER, Mircea ELIADE, BÉROSE et 3 autre(s) ; 3 images
Publié depuis l'éditeur des fiches.
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-americains.xlsx
+++ b/data/frise-philosophes-americains.xlsx
@@ -3451,8 +3451,10 @@
       <c r="D29" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="E29" s="9" t="s">
-        <v>252</v>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt; &lt;a href="https://fr.wikipedia.org/wiki/Ayn_Rand" title=" Wikipedia"&gt; Ayn RAND&lt;/a&gt; était une écrivaine, philosophe et théoricienne politique russo-américaine. Elle est née à Saint-Pétersbourg, en Russie, sous le nom d'Alissa Zinovievna Rosenbaum et a vécu une grande partie de sa vie aux États-Unis, où elle a émigré en 1926.   &lt;/p&gt; &lt;p&gt; Son courant de pensée, &lt;a href="https://www.youtube.com/watch?v=w-54oWWvw-k&amp;amp;ab_channel=BiTS%2Cmagazinepresqueculte-ARTE" title="Objectivisme: la philo pour les égoîste par Arte "&gt;l'Objectivisme&lt;/a&gt; met l'accent sur la primauté de la raison, l'éthique de&lt;a href="https://www.youtube.com/watch?v=k2mVwk16ifQ" title="AYN RAND - L'égoïsme est une vertu par Le Précepteur"&gt; l'égoïsme rationnel&lt;/a&gt;, le capitalisme de laissez-faire et la défense des droits individuels. Selon elle, l'individu rationnel est la plus haute valeur morale et la poursuite de son propre intérêt rationnel est le but de la vie. &lt;/p&gt; &lt;p&gt; Connue pour ses deux romans principaux :  &lt;a href="https://fr.wikipedia.org/wiki/La_Source_vive" title="La source vive par Wikipédia "&gt;"La Source vive"&lt;/a&gt; (The Fountainhead), où elle présente un architecte individualiste et indépendant qui se bat pour préserver son intégrité et son travail créatif face à une société qui valorise la conformité et le collectivisme. &lt;/p&gt; &lt;p&gt; Le plus célèbre, &lt;a href="https://www.youtube.com/watch?v=Rti2fNcf10U&amp;amp;ab_channel=Lextopia" title="La grève pour capitalistes par Lextopia "&gt;"La Grève"&lt;/a&gt; (Atlas Shrugged), où elle explore les conséquences d'une société où les esprits créatifs et les entrepreneurs se retirent pour protester contre les politiques gouvernementales oppressives. Ce livre présente également des concepts clés de sa philosophie, tels que la notion de "l'homme qui arrête le moteur du monde" et la croyance en la libre entreprise et en la recherche du  &lt;a href="https://www.youtube.com/watch?v=D-fU2DMB8T0&amp;amp;ab_channel=Kosmos" title="Faut il ne pensée qu'à soi ? par Kosmos "&gt;profit personnel&lt;/a&gt; comme moteurs de progrès. &lt;/p&gt; &lt;p&gt; &lt;a href="https://www.youtube.com/watch?v=MA1gKCD1h30&amp;amp;ab_channel=gio" title="Interview de 1959 par gio "&gt;Ses idées&lt;/a&gt; ont suscité des réactions diverses et passionnées. Ses partisans la considèrent comme une championne de la liberté individuelle, du capitalisme et de la raison. Ses détracteurs la critiquent souvent pour son individualisme radical, son rejet des systèmes de soutien social et son manque d'empathie envers les faibles. &lt;/p&gt;  &lt;audio controls title="Egoïste et fier de l'être par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/23118-15.06.2022-ITEMA_23059653-2022C12410S0166-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fiches — 1 fiche nouvelle : ÂNKHSHESHONQ ; 24 fiches modifiées : Aníbal QUIJANO, Sulak SIVARAKSA, LEUCIPPE, PARMÉNIDE, STILPON de Mégare, HIPPARCHIA de Maronée et 18 autre(s) ; 1 fiche retirée : ÂNKHSHESHONQY ; 10 images
Publié depuis l'éditeur des fiches.
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-americains.xlsx
+++ b/data/frise-philosophes-americains.xlsx
@@ -4124,810 +4124,807 @@
         <v>51</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="n">
+    <row r="44" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1">
+        <v>1930</v>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2018</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1930 – 2018</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aníbal QUIJANO</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/An%C3%ADbal_Quijano" title=" Wikipedia"&gt;Aníbal QUIJANO&lt;/a&gt; est un sociologue péruvien, l’un des grands penseurs latino-américains du XXe siècle et le fondateur de la pensée décoloniale. Né en 1928 à Yanama, dans les Andes péruviennes, il étudie à l’université de San Marcos, à Lima, où il enseigne ensuite la sociologie. Dans les années 1960 et 1970, il participe aux travaux de la &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9orie_de_la_d%C3%A9pendance" title=" Wikipedia"&gt;théorie de la dépendance&lt;/a&gt;, qui explique le sous-développement de l’Amérique latine par sa place subordonnée dans l’économie mondiale, et étudie la condition des populations indiennes et métisses des villes.&lt;/p&gt; &lt;p&gt;En 1992, pour le cinquième centenaire de l’arrivée de Christophe Colomb, il publie l’article « Colonialité et modernité/rationalité », qui forge la notion de « colonialité du pouvoir ». La conquête de l’Amérique a donné naissance à la fois au capitalisme mondial et à une idée nouvelle, celle de « race », qui a permis de classer les peuples en supérieurs et inférieurs et de distribuer entre eux le travail : le salariat pour les Européens, le servage pour les Indiens, l’esclavage pour les Africains. Cette classification a survécu à l’indépendance des colonies : elle structure encore les rapports sociaux, le savoir et la manière dont chacun se perçoit. Quijano critique aussi l’« eurocentrisme », qui fait de l’histoire européenne le modèle de l’histoire universelle.&lt;/p&gt; &lt;p&gt;Professeur à l’université de Binghamton, aux États-Unis, il anime le &lt;a href="https://fr.wikipedia.org/wiki/Groupe_modernit%C3%A9/colonialit%C3%A9" title=" Wikipedia"&gt;groupe « modernité/colonialité »&lt;/a&gt; avec Walter Mignolo et Enrique Dussel. La philosophe argentine &lt;a href="https://fr.wikipedia.org/wiki/Mar%C3%ADa_Lugones" title=" Wikipedia"&gt;María Lugones&lt;/a&gt; a prolongé son concept dans celui de « colonialité du genre ». Il meurt à Lima en 2018.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/quijano-mini.webp</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">politique ; epistemologie</t>
+        </is>
+      </c>
+      <c r="K44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensée décoloniale</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sociologue péruvien, inventeur de la « colonialité du pouvoir » et fondateur de la pensée décoloniale.</t>
+        </is>
+      </c>
+      <c r="N44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="O44" s="1"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Péruvienne</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="7" t="n">
         <v>1931</v>
       </c>
-      <c r="B44" s="7" t="s">
+      <c r="B45" s="7" t="s">
         <v>374</v>
       </c>
-      <c r="C44" s="7" t="s">
+      <c r="C45" s="7" t="s">
         <v>375</v>
       </c>
-      <c r="D44" s="8" t="s">
+      <c r="D45" s="8" t="s">
         <v>376</v>
       </c>
-      <c r="E44" s="10" t="inlineStr">
+      <c r="E45" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Richard_Rorty" title=" Wikipedia"&gt;Richard RORTY&lt;/a&gt; était un  philosophe américain, figure majeure du  &lt;a href="https://www.youtube.com/watch?v=lfx4Jag1ic4"  title="Le pragmatisme : définition, exemples par le savoir partagé"&gt;pragmatisme&lt;/a&gt; et du postmodernisme, il a remis en cause les fondements de la philosophie occidentale et proposé une &lt;a href="https://laviedesidees.fr/Rorty-Pragmatism-Anti-Authoritarianism" title=" a bas l'autorité par laviedesidees"&gt;vision radicale&lt;/a&gt;  de la vérité, de la culture et de la société. Il rejette l'idée que la vérité soit une correspondance entre le langage et la réalité. Pour lui, la vérité est simplement ce qui est utile ou avantageux à croire dans une communauté donnée et il propose d'abandonner la quête de fondements absolus de la connaissance, jugée vaine. &lt;/p&gt; &lt;p&gt; Inspiré par Wittgenstein et Davidson, il considère le langage non pas comme un miroir de la réalité, mais comme un ensemble d'outils pour résoudre des problèmes pratiques.  Les vocabularies que nous utilisons sont historiquement et culturellement contingents, non pas "vrais" ou "faux". &lt;/p&gt; &lt;p&gt; Dans ces oeuvres principales, on trouve  &lt;a href="https://www.youtube.com/watch?v=MgU0dXZ3umM" title="L’ironiste libéral chez Rorty : Contingence, ironie et solidarité par Darina Metreveli"&gt;" Contingence, ironie et solidarité "&lt;/a&gt; (1989) ou il décrit l'ironiste comme quelqu'un qui doute de ses propres croyances tout en œuvrant pour une société plus juste. Dans " Achieving Our Country" (1998),  il y appelle la gauche américaine à abandonner le "culturalisme" pour se recentrer sur les inégalités économiques et sociales. Cet ouvrage est souvent cité pour avoir anticipé les crises politiques du XXIe siècle. &lt;/p&gt; &lt;p&gt;  Ses thèses sur la contingence de la vérité sont souvent invoquées pour analyser l'ère de la "post-vérité". Son insistance sur la conversation comme fondement du lien social influence la philosophie politique contemporaine. Il  a bouleversé la philosophie en démystifiant ses prétentions à la vérité absolue. Son œuvre, à la fois provocante et humaniste, invite à remplacer la quête métaphysique par un engagement en faveur d'une société plus juste et plus inclusive. &lt;/p&gt; </t>
         </is>
       </c>
-      <c r="F44" s="7" t="s">
+      <c r="F45" s="7" t="s">
         <v>378</v>
       </c>
-      <c r="G44" s="9" t="s">
+      <c r="G45" s="9" t="s">
         <v>379</v>
       </c>
-      <c r="H44" s="9" t="s">
+      <c r="H45" s="9" t="s">
         <v>380</v>
       </c>
-      <c r="I44" s="9"/>
-      <c r="J44" s="2" t="s">
+      <c r="I45" s="9"/>
+      <c r="J45" s="2" t="s">
         <v>381</v>
       </c>
-      <c r="K44" s="2" t="s">
+      <c r="K45" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="L44" s="2" t="s">
+      <c r="L45" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="N44" s="1" t="s">
+      <c r="N45" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="293.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="1" t="n">
+    <row r="46" customFormat="false" ht="293.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="1" t="n">
         <v>1932</v>
       </c>
-      <c r="B45" s="1" t="n">
+      <c r="B46" s="1" t="n">
         <v>2025</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="C46" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="D46" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/John_Searle"  title=" Wikipedia"&gt;John SEARLE&lt;/a&gt; était un philosophe américain  connu pour ses travaux influents dans plusieurs domaines, notamment la philosophie du langage, la philosophie de l'esprit et la philosophie sociale. Il  a développé et systématisé la théorie des &lt;a href="https://www.youtube.com/watch?v=pIbkpLfrD6A" title="
 La théorie des actes de langage (2) - John Searle par Heraut du Mont Parnasse"&gt;actes de langage&lt;/a&gt; car, pour lui, parler une langue, ce n'est pas seulement émettre des sons ou des suites de symboles, mais accomplir des actions. &lt;/p&gt; &lt;p&gt; Défenseur du "naturalisme biologique" en philosophie de l'esprit. Il s'oppose au dualisme cartésien tout en refusant le matérialisme réducteur qui nierait l'existence de &lt;a href="https://www.youtube.com/watch?v=EriAhi0mj7w" title=" Conscience et matière grise par TEDx Talks"&gt;la conscience&lt;/a&gt; ou la réduirirait à de simples phénomènes physiques. Pour lui, les états mentaux (douleur, croyances, désirs, conscience) sont des phénomènes  &lt;a href="https://www.youtube.com/watch?v=Bq2bfSzkTfU"  title="John Searle - Une personne peut-elle être une âme ? par Closer To Truth"&gt;biologiques réels&lt;/a&gt;, causés par des processus neuronaux du cerveau, mais ils ne sont pas réductibles à ces processus au sens où ils émergent à un niveau supérieur et possèdent des propriétés irréductibles.&lt;/p&gt; &lt;p&gt; L'une des ses contributions les plus célèbres est son argument de la &lt;a href="https://www.youtube.com/watch?v=P5DtwDr9YEc" title=" La Chambre chinoise par Ian et frank"&gt;Chambre Chinoise&lt;/a&gt;. Cet argument vise à réfuter la thèse de l'IA forte (position selon laquelle un ordinateur programmé de manière appropriée n'est pas seulement un outil pour l'étude de l'esprit, mais qu'il est véritablement un esprit, capable de comprendre et de posséder d'autres états cognitifs) opposé à l'IA faible (position selon laquelle les ordinateurs sont des outils utiles pour étudier l'esprit, mais qu'ils ne sont pas eux-mêmes des esprits). &lt;/p&gt; &lt;p&gt; Dans son ouvrage &lt;a href="https://labo.nonmarchand.org/pmwiki/uploads/Textes/JohnSearleLaConstructionDeLaRealiteSociale/JohnSearle_LaConstructionDeLaRealiteSociale.pdf"  title=" La construction e la réalité sociale par nonmarchand"&gt;"La Construction de la Réalité Sociale"&lt;/a&gt;, il étend sa théorie des actes de langage et de l'intentionnalité pour expliquer comment nous construisons des faits institutionnels et sociaux. Il distingue les "Faits bruts" qui existent indépendamment de toute institution humaine (par exemple, la montagne Everest) des "Faits institutionnels" qui n'existent qu'en vertu d'institutions humaines et de l'accord collectif (par exemple, l'argent, le mariage, la propriété). &lt;/p&gt; 
 </t>
         </is>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="F46" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="G45" s="2" t="s">
+      <c r="G46" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="H45" s="2" t="s">
+      <c r="H46" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="I45" s="1"/>
-      <c r="J45" s="2" t="s">
+      <c r="I46" s="1"/>
+      <c r="J46" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="K45" s="1" t="s">
+      <c r="K46" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="L45" s="2" t="s">
+      <c r="L46" s="2" t="s">
         <v>391</v>
-      </c>
-      <c r="N45" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="P45" s="1" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="171.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7" t="n">
-        <v>1933</v>
-      </c>
-      <c r="B46" s="7" t="s">
-        <v>322</v>
-      </c>
-      <c r="C46" s="7" t="s">
-        <v>393</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>394</v>
-      </c>
-      <c r="E46" s="13" t="s">
-        <v>395</v>
-      </c>
-      <c r="F46" s="7"/>
-      <c r="G46" s="9"/>
-      <c r="H46" s="9" t="s">
-        <v>396</v>
-      </c>
-      <c r="I46" s="10" t="s">
-        <v>397</v>
-      </c>
-      <c r="J46" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="L46" s="2" t="s">
-        <v>399</v>
       </c>
       <c r="N46" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="47" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P46" s="1" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="171.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="n">
+        <v>1933</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="D47" s="8" t="s">
+        <v>394</v>
+      </c>
+      <c r="E47" s="13" t="s">
+        <v>395</v>
+      </c>
+      <c r="F47" s="7"/>
+      <c r="G47" s="9"/>
+      <c r="H47" s="9" t="s">
+        <v>396</v>
+      </c>
+      <c r="I47" s="10" t="s">
+        <v>397</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="L47" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="N47" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="7" t="n">
         <v>1934</v>
       </c>
-      <c r="B47" s="7" t="s">
+      <c r="B48" s="7" t="s">
         <v>400</v>
       </c>
-      <c r="C47" s="7" t="s">
+      <c r="C48" s="7" t="s">
         <v>401</v>
       </c>
-      <c r="D47" s="8" t="s">
+      <c r="D48" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="E47" s="9" t="inlineStr">
+      <c r="E48" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Enrique_Dussel"  title=" Wikipedia"&gt;Enrique DUSSEL&lt;/a&gt; était un philosophe argentin majeurs de la décolonialité et de la philosophie latino-américaine de la liberation.  Jeune intellectuel engagé dans les mouvements étudiants et opposé aux régimes autoritaires, il a été persécuté en Argentine avant de s’exiler au Mexique en 1975, où il a poursuivi sa carrière académique et développé sa pensée. Il élabore une &lt;a href="https://www.youtube.com/watch?v=QGPosp7lYlM" title="Enrique Dussel and the Philosophy of Liberation – Decolonizing Thought par Darina Metreveli"&gt;philosophie de la libération &lt;/a&gt; qui remet en question l’ontologie monologique de la modernité et introduit une approche éthique et alteritaire inspirée par Levinas, souvent décrite sous le nom d’analectique ou de dialectique positive. &lt;/p&gt; &lt;p&gt; Pionnier du décolonialisme latino-américain, il contribue à la construction des cadres Modernité/Colonialité et à l’idée d’une transmodernité, articulant critique de la modernité et invitation à repenser les rapports Nord-Sud et centre-périphérie. &lt;/p&gt; &lt;p&gt; Ses oeuvres majeures : &lt;a href="https://www.youtube.com/watch?v=nXNyqKCrKLY" title="Enrique Dussel, métaphysicien de la libération - Emmanuel Lévine par lundimatin"&gt;"Méthode pour une philosophie de la libération" &lt;/a&gt; paru en  1974 et "Filosofía ética latinoamericana" (période majeure)  posent les bases d’une philosophie enracinée dans les expériences des peuples opprimés et des contextes colonisés. &lt;/p&gt; &lt;p&gt; Il est reconnu dans les &lt;a href="https://lestempsquirestent.org/fr/numeros/numero-7/enrique-dussel-un-philosophe-indispensable-pour-decoloniser-la-theologie-politique" title="Enrique Dussel,
 un philosophe indispensable pour décoloniser la théologie politique par les temps qui restent"&gt;milieux décoloniaux &lt;/a&gt; et philosophie de la libération, mais demeure moins connu du grand public français, bien que des traductions et des analyses apparaissent et stimulent l’intérêt académique en France. Son travail nourrit le courant décolonial qui met en évidence l’interdépendance entre modernité et colonialité depuis 1492 et propose des axes pour une pensée transmoderne, dépassant les cadres classiques de la philosophie occidentale. &lt;/p&gt; </t>
         </is>
       </c>
-      <c r="F47" s="7" t="s">
+      <c r="F48" s="7" t="s">
         <v>404</v>
       </c>
-      <c r="G47" s="9" t="s">
+      <c r="G48" s="9" t="s">
         <v>405</v>
       </c>
-      <c r="H47" s="9" t="s">
+      <c r="H48" s="9" t="s">
         <v>406</v>
-      </c>
-      <c r="I47" s="9"/>
-      <c r="J47" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiers-mondisme ; Théologie de la libération ; Philosophie de la libération ; Pensée décoloniale</t>
-        </is>
-      </c>
-      <c r="L47" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="N47" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="O47" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="P47" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="240.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7" t="n">
-        <v>1934</v>
-      </c>
-      <c r="B48" s="7" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C48" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="D48" s="8" t="s">
-        <v>409</v>
-      </c>
-      <c r="E48" s="11" t="s">
-        <v>410</v>
-      </c>
-      <c r="F48" s="7" t="s">
-        <v>411</v>
-      </c>
-      <c r="G48" s="9" t="s">
-        <v>412</v>
-      </c>
-      <c r="H48" s="10" t="s">
-        <v>413</v>
       </c>
       <c r="I48" s="9"/>
       <c r="J48" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tiers-mondisme ; Théologie de la libération ; Philosophie de la libération ; Pensée décoloniale</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="N48" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O48" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="P48" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="240.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="7" t="n">
+        <v>1934</v>
+      </c>
+      <c r="B49" s="7" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="E49" s="11" t="s">
+        <v>410</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="H49" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="I49" s="9"/>
+      <c r="J49" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="K48" s="2" t="s">
+      <c r="K49" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="L48" s="2" t="s">
+      <c r="L49" s="2" t="s">
         <v>415</v>
-      </c>
-      <c r="N48" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="240.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="1" t="n">
-        <v>1934</v>
-      </c>
-      <c r="B49" s="1" t="n">
-        <v>2019</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>417</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>418</v>
-      </c>
-      <c r="F49" s="1" t="s">
-        <v>419</v>
-      </c>
-      <c r="G49" s="15" t="s">
-        <v>420</v>
-      </c>
-      <c r="H49" s="2" t="s">
-        <v>421</v>
-      </c>
-      <c r="I49" s="1"/>
-      <c r="J49" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="K49" s="1" t="s">
-        <v>390</v>
-      </c>
-      <c r="L49" s="2" t="s">
-        <v>422</v>
-      </c>
-      <c r="M49" s="1" t="s">
-        <v>423</v>
       </c>
       <c r="N49" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="P49" s="1" t="s">
+    </row>
+    <row r="50" customFormat="false" ht="240.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="1" t="n">
+        <v>1934</v>
+      </c>
+      <c r="B50" s="1" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="G50" s="15" t="s">
+        <v>420</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="I50" s="1"/>
+      <c r="J50" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="K50" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="L50" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="M50" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="N50" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="P50" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="XFC49" s="0"/>
-      <c r="XFD49" s="0"/>
-    </row>
-    <row r="50" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="16" t="n">
+      <c r="XFC50" s="0"/>
+      <c r="XFD50" s="0"/>
+    </row>
+    <row r="51" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="16" t="n">
         <v>1935</v>
       </c>
-      <c r="B50" s="16" t="n">
+      <c r="B51" s="16" t="n">
         <v>2003</v>
       </c>
-      <c r="C50" s="16" t="s">
+      <c r="C51" s="16" t="s">
         <v>425</v>
       </c>
-      <c r="D50" s="17" t="s">
+      <c r="D51" s="17" t="s">
         <v>426</v>
       </c>
-      <c r="E50" s="13" t="s">
+      <c r="E51" s="13" t="s">
         <v>427</v>
       </c>
-      <c r="F50" s="16" t="s">
+      <c r="F51" s="16" t="s">
         <v>428</v>
       </c>
-      <c r="G50" s="18" t="s">
+      <c r="G51" s="18" t="s">
         <v>429</v>
       </c>
-      <c r="H50" s="10" t="s">
+      <c r="H51" s="10" t="s">
         <v>430</v>
       </c>
-      <c r="I50" s="18"/>
-      <c r="J50" s="2" t="s">
+      <c r="I51" s="18"/>
+      <c r="J51" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="K50" s="2" t="s">
+      <c r="K51" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="L50" s="14" t="s">
+      <c r="L51" s="14" t="s">
         <v>432</v>
       </c>
-      <c r="M50" s="14" t="s">
+      <c r="M51" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="N50" s="14" t="s">
+      <c r="N51" s="14" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7" t="n">
+    <row r="52" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="7" t="n">
         <v>1937</v>
       </c>
-      <c r="B51" s="7" t="s">
+      <c r="B52" s="7" t="s">
         <v>322</v>
       </c>
-      <c r="C51" s="7" t="s">
+      <c r="C52" s="7" t="s">
         <v>433</v>
       </c>
-      <c r="D51" s="8" t="s">
+      <c r="D52" s="8" t="s">
         <v>434</v>
       </c>
-      <c r="E51" s="11" t="s">
+      <c r="E52" s="11" t="s">
         <v>435</v>
       </c>
-      <c r="F51" s="7" t="s">
+      <c r="F52" s="7" t="s">
         <v>436</v>
       </c>
-      <c r="G51" s="9" t="s">
+      <c r="G52" s="9" t="s">
         <v>437</v>
       </c>
-      <c r="H51" s="10" t="s">
+      <c r="H52" s="10" t="s">
         <v>438</v>
-      </c>
-      <c r="I51" s="9"/>
-      <c r="J51" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="K51" s="2" t="s">
-        <v>439</v>
-      </c>
-      <c r="L51" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="N51" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="167.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="7" t="n">
-        <v>1938</v>
-      </c>
-      <c r="B52" s="7" t="n">
-        <v>2002</v>
-      </c>
-      <c r="C52" s="7" t="s">
-        <v>441</v>
-      </c>
-      <c r="D52" s="8" t="s">
-        <v>442</v>
-      </c>
-      <c r="E52" s="13" t="s">
-        <v>443</v>
-      </c>
-      <c r="F52" s="7" t="s">
-        <v>444</v>
-      </c>
-      <c r="G52" s="9" t="s">
-        <v>445</v>
-      </c>
-      <c r="H52" s="10" t="s">
-        <v>446</v>
       </c>
       <c r="I52" s="9"/>
       <c r="J52" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="K52" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Libéralisme ; Minarchisme ; Déontologisme</t>
-        </is>
+        <v>127</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>439</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="M52" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="N52" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="N52" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="167.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="n">
         <v>1938</v>
       </c>
-      <c r="B53" s="7" t="s">
-        <v>449</v>
+      <c r="B53" s="7" t="n">
+        <v>2002</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>450</v>
+        <v>441</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>451</v>
-      </c>
-      <c r="E53" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Tom_Regan"  title=" Wikipedia"&gt;Tom REGAN&lt;/a&gt; était un philosophe américain   &lt;a href="https://www.youtube.com/watch?v=hgVMf3q4Vh4"  title=" Les animaux aussi ont une valeur. Valeur inhérente &amp; respect. - Tom Regan - Pensées antispécistes par The Critical Vegan"&gt;antispéciste &lt;/a&gt; influent dans le domaine de l'éthique animale, considéré comme un pionnier de la théorie des droits des animaux sur une base déontologique. Né à Pittsburgh, il enseigne de 1967 à 2001 à l’université d’État de Caroline du Nord. Il développe une approche abolitionniste opposée à l'utilitarisme de Peter Singer, arguant que les mammifères normaux d'un an ou plus sont des "sujets-d'une-vie" dotés d'une valeur inhérente, méritant des droits moraux fondamentaux indépendamment de leur utilité. Inspiré par Kant mais étendu aux non-humains, il définit ces sujets comme des êtres conscients pour qui leur vie importe intrinsèquement, justifiant l'interdiction absolue de l'exploitation. &lt;/p&gt; &lt;p&gt; Ses Œuvres principales sont : "The Case for Animal Rights" paru en 1983, traduit en français comme  &lt;a href="http://tomregan.free.fr/" title=" Les animaux aussi ont une valeur. Valeur inhérente &amp; respect. - Tom Regan - Les Droits des animaux par Tom Regan"&gt;"Les Droits des animaux" &lt;/a&gt; en 2013 : son magnum opus, salué comme un classique moderne critiquant Descartes et plaidant pour le "principe de respect" envers tout sujet-d'une-vie. "All That Dwell Therein" paru en  1982 : recueil d'essais sur le végétarisme et l'éthique animale. &lt;/p&gt; &lt;p&gt; Ses idées ont profondément marqué le mouvement des droits des animaux, influençant débats sur végétarisme, anti-vivisection et critique de l'environnementalisme indirect, tout en étant cité par des penseurs comme Derrida ou dans des ouvrages comme ceux de Jean-Baptiste Jeangène Vilmer. Dans &lt;em&gt;Empty Cages&lt;/em&gt; (2004), destiné au grand public, il résume son combat : il ne s’agit pas d’agrandir les cages, mais de les vider. &lt;/p&gt; </t>
-        </is>
+        <v>442</v>
+      </c>
+      <c r="E53" s="13" t="s">
+        <v>443</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>453</v>
+        <v>444</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>454</v>
-      </c>
-      <c r="H53" s="9" t="s">
-        <v>455</v>
+        <v>445</v>
+      </c>
+      <c r="H53" s="10" t="s">
+        <v>446</v>
       </c>
       <c r="I53" s="9"/>
       <c r="J53" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Libéralisme ; Minarchisme ; Déontologisme</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="M53" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="N53" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7" t="n">
+        <v>1938</v>
+      </c>
+      <c r="B54" s="7" t="s">
+        <v>449</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Tom_Regan"  title=" Wikipedia"&gt;Tom REGAN&lt;/a&gt; était un philosophe américain   &lt;a href="https://www.youtube.com/watch?v=hgVMf3q4Vh4"  title=" Les animaux aussi ont une valeur. Valeur inhérente &amp; respect. - Tom Regan - Pensées antispécistes par The Critical Vegan"&gt;antispéciste &lt;/a&gt; influent dans le domaine de l'éthique animale, considéré comme un pionnier de la théorie des droits des animaux sur une base déontologique. Né à Pittsburgh, il enseigne de 1967 à 2001 à l’université d’État de Caroline du Nord. Il développe une approche abolitionniste opposée à l'utilitarisme de Peter Singer, arguant que les mammifères normaux d'un an ou plus sont des "sujets-d'une-vie" dotés d'une valeur inhérente, méritant des droits moraux fondamentaux indépendamment de leur utilité. Inspiré par Kant mais étendu aux non-humains, il définit ces sujets comme des êtres conscients pour qui leur vie importe intrinsèquement, justifiant l'interdiction absolue de l'exploitation. &lt;/p&gt; &lt;p&gt; Ses Œuvres principales sont : "The Case for Animal Rights" paru en 1983, traduit en français comme  &lt;a href="http://tomregan.free.fr/" title=" Les animaux aussi ont une valeur. Valeur inhérente &amp; respect. - Tom Regan - Les Droits des animaux par Tom Regan"&gt;"Les Droits des animaux" &lt;/a&gt; en 2013 : son magnum opus, salué comme un classique moderne critiquant Descartes et plaidant pour le "principe de respect" envers tout sujet-d'une-vie. "All That Dwell Therein" paru en  1982 : recueil d'essais sur le végétarisme et l'éthique animale. &lt;/p&gt; &lt;p&gt; Ses idées ont profondément marqué le mouvement des droits des animaux, influençant débats sur végétarisme, anti-vivisection et critique de l'environnementalisme indirect, tout en étant cité par des penseurs comme Derrida ou dans des ouvrages comme ceux de Jean-Baptiste Jeangène Vilmer. Dans &lt;em&gt;Empty Cages&lt;/em&gt; (2004), destiné au grand public, il résume son combat : il ne s’agit pas d’agrandir les cages, mais de les vider. &lt;/p&gt; </t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="s">
+        <v>453</v>
+      </c>
+      <c r="G54" s="9" t="s">
+        <v>454</v>
+      </c>
+      <c r="H54" s="9" t="s">
+        <v>455</v>
+      </c>
+      <c r="I54" s="9"/>
+      <c r="J54" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="K53" s="2" t="s">
+      <c r="K54" s="2" t="s">
         <v>456</v>
       </c>
-      <c r="L53" s="2" t="s">
+      <c r="L54" s="2" t="s">
         <v>457</v>
-      </c>
-      <c r="N53" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="1" t="n">
-        <v>1940</v>
-      </c>
-      <c r="B54" s="1" t="n">
-        <v>2022</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>458</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Saul_Kripke"  title=" Wikipedia"&gt;Saul KRIPKE&lt;/a&gt; était un philosophe américain de la tradition analytique connu pour ses apports décisifs en logique modale, en métaphysique et en philosophie du langage. Très jeune, il révolutionne la logique en introduisant la sémantique des mondes possibles, aujourd’hui appelée &lt;a href="https://www.youtube.com/watch?v=_sIgAdvhruU"title="Qui est Saul Kripke ? par Monsieur Phi"&gt;"cadres de Kripke"&lt;/a&gt;, qui permet de formaliser la modalité (le nécessaire et le possible) de façon rigoureuse. &lt;/p&gt; &lt;p&gt; Son œuvre la plus influente est "Naming and Necessity", où il critique la conception descriptiviste des noms défendue par Frege et Russell. Selon lui, un  &lt;a href="https://www.youtube.com/watch?v=d7-8Avem7EE" title="Saul Kripke, La logique des noms propres. par Jtgrandtour"&gt; nom propre&lt;/a&gt; n’équivaut pas à une description mais fonctionne comme un « désignateur rigide » : il désigne le même individu dans tous les mondes possibles. Cette idée bouleverse la philosophie du langage et entraîne une redéfinition de la notion de référence.&lt;/p&gt; &lt;p&gt;  Il montre également qu’il existe des vérités nécessaires découvertes empiriquement : par exemple, l’identité « l’eau est H₂O » est nécessaire, mais nous ne l’avons apprise qu’a posteriori. Ce concept de nécessité a posteriori a marqué un tournant dans la métaphysique contemporaine. À l’inverse, il identifie la possibilité de certaines vérités contingentes connues a priori, ce qui remet en cause des distinctions classiques entre connaissance et modalité. &lt;/p&gt; &lt;p&gt; Il s’oppose au physicalisme en arguant que l’on peut concevoir un monde où tous les états cérébraux existent sans que la conscience subjective "le qualia" ne soit présente. Cette critique alimente encore aujourd’hui les débats sur la nature de la conscience. Son ouvrage "Wittgenstein on Rules and Private Language" propose une lecture radicale de Wittgenstein, selon laquelle toute règle est sujette à un scepticisme profond sur son application. Bien que controversée, cette interprétation a largement stimulé les discussions en philosophie du langage et en épistémologie. &lt;/p&gt; &lt;p&gt; Connu aussi pour son ouvrage " On two Paradoxes of Knowledge" et son  &lt;a href="https://www.youtube.com/watch?v=AzaUSC--2G0"  title="Le Paradoxe de l'Examen selon Saul Kripke par Silogic"&gt;"paradoxe de l'examen"&lt;/a&gt;. &lt;/p&gt; </t>
-        </is>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>461</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>462</v>
-      </c>
-      <c r="H54" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="J54" s="2" t="s">
-        <v>464</v>
-      </c>
-      <c r="K54" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="L54" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="M54" s="1" t="s">
-        <v>176</v>
       </c>
       <c r="N54" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="P54" s="1" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="7" t="n">
-        <v>1941</v>
-      </c>
-      <c r="B55" s="7" t="s">
-        <v>467</v>
-      </c>
-      <c r="C55" s="7" t="s">
-        <v>468</v>
-      </c>
-      <c r="D55" s="8" t="s">
-        <v>469</v>
-      </c>
-      <c r="E55" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/David_Lewis_(philosophe)"  title=" Wikipedia"&gt;David LEWIS&lt;/a&gt; était un philosophe américain connu pour sa théorie du  réalisme modal, selon laquelle il existe un nombre infini de mondes possibles concrets et causalement isolés les uns des autres. Son ouvrage majeur   &lt;a href="https://www.youtube.com/watch?v=-QlqLDLifuc" title="David Lewis - "De la pluralité des mondes" - De quoi parle ce livre ? par Philosophie 21"&gt;"On the Plurality of Worlds"&lt;/a&gt;  sortie en 1986, expose cette position révolutionnaire : pour lui, chaque monde possible existe aussi réellement que notre monde actuel, et sert à comprendre la modalité, c'est-à-dire ce qui pourrait être ou ce qui doit être. &lt;/p&gt; &lt;p&gt; Il a également proposé la théorie des contreparties en logique modale : au lieu de supposer que les personnes ou objets existent dans plusieurs mondes possibles, il affirme que chaque individu de notre monde a des « contreparties » dans les autres mondes possibles qui partagent certaines caractéristiques mais ne sont pas identiques à lui. Cette approche constitue une alternative à la logique modale traditionnelle, notamment celle de Saul Kripke. &lt;/p&gt; &lt;p&gt; Sa métaphysique est marquée par une conception atomiste (pointilliste) : la réalité n’est qu’une vaste mosaïque de faits locaux, chaque fait étant centré sur un « point » ayant des propriétés intrinsèques. Ce point de vue s’inspire de David Hume, d’où le nom « survenance humienne », refusant les liens nécessaires entre les faits et privilégiant une juxtaposition de qualités locales. &lt;/p&gt; &lt;p&gt; Il  a beaucoup écrit sur la philosophie du langage, la philosophie de l’esprit, l’épistémologie, la logique philosophique et la philosophie des mathématiques. Son premier grand ouvrage, "Convention" de 1969, analyse les conventions sociales à l’aide de la théorie des jeux, en montrant leur caractère arbitraire et leur diffusion par la connaissance commune et le précédent. Il s a marqué durablement la philosophie analytique.  &lt;a href="https://www.youtube.com/watch?v=g3jQwDP_Lyc" title="David Lewis - "David Lewis Speaks at La Trobe University par TimeSparrow"&gt;"Ses théories&lt;/a&gt; sont incontournables dans les débats sur les mondes possibles, la modalité, la causalité, la convention sociale, et l’atomisme métaphysique. Ses ouvrages, tels que Counterfactuals et Philosophical Papers, restent des références dans l’analyse logique et conceptuelle contemporaine. &lt;/p&gt; &lt;audio controls title=" On dit de David Lewis que c'est le plus grand métaphysicien qu’on ait vu depuis Leibniz par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/18292-28.02.2019-ITEMA_21995453-0.mp3" type="audio/mpeg" align="center"&gt;&lt;/audio&gt;  </t>
-        </is>
-      </c>
-      <c r="F55" s="7" t="s">
-        <v>471</v>
-      </c>
-      <c r="G55" s="9" t="s">
-        <v>472</v>
-      </c>
-      <c r="H55" s="9" t="s">
-        <v>473</v>
-      </c>
-      <c r="I55" s="9"/>
+    </row>
+    <row r="55" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="1" t="n">
+        <v>1940</v>
+      </c>
+      <c r="B55" s="1" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Saul_Kripke"  title=" Wikipedia"&gt;Saul KRIPKE&lt;/a&gt; était un philosophe américain de la tradition analytique connu pour ses apports décisifs en logique modale, en métaphysique et en philosophie du langage. Très jeune, il révolutionne la logique en introduisant la sémantique des mondes possibles, aujourd’hui appelée &lt;a href="https://www.youtube.com/watch?v=_sIgAdvhruU"title="Qui est Saul Kripke ? par Monsieur Phi"&gt;"cadres de Kripke"&lt;/a&gt;, qui permet de formaliser la modalité (le nécessaire et le possible) de façon rigoureuse. &lt;/p&gt; &lt;p&gt; Son œuvre la plus influente est "Naming and Necessity", où il critique la conception descriptiviste des noms défendue par Frege et Russell. Selon lui, un  &lt;a href="https://www.youtube.com/watch?v=d7-8Avem7EE" title="Saul Kripke, La logique des noms propres. par Jtgrandtour"&gt; nom propre&lt;/a&gt; n’équivaut pas à une description mais fonctionne comme un « désignateur rigide » : il désigne le même individu dans tous les mondes possibles. Cette idée bouleverse la philosophie du langage et entraîne une redéfinition de la notion de référence.&lt;/p&gt; &lt;p&gt;  Il montre également qu’il existe des vérités nécessaires découvertes empiriquement : par exemple, l’identité « l’eau est H₂O » est nécessaire, mais nous ne l’avons apprise qu’a posteriori. Ce concept de nécessité a posteriori a marqué un tournant dans la métaphysique contemporaine. À l’inverse, il identifie la possibilité de certaines vérités contingentes connues a priori, ce qui remet en cause des distinctions classiques entre connaissance et modalité. &lt;/p&gt; &lt;p&gt; Il s’oppose au physicalisme en arguant que l’on peut concevoir un monde où tous les états cérébraux existent sans que la conscience subjective "le qualia" ne soit présente. Cette critique alimente encore aujourd’hui les débats sur la nature de la conscience. Son ouvrage "Wittgenstein on Rules and Private Language" propose une lecture radicale de Wittgenstein, selon laquelle toute règle est sujette à un scepticisme profond sur son application. Bien que controversée, cette interprétation a largement stimulé les discussions en philosophie du langage et en épistémologie. &lt;/p&gt; &lt;p&gt; Connu aussi pour son ouvrage " On two Paradoxes of Knowledge" et son  &lt;a href="https://www.youtube.com/watch?v=AzaUSC--2G0"  title="Le Paradoxe de l'Examen selon Saul Kripke par Silogic"&gt;"paradoxe de l'examen"&lt;/a&gt;. &lt;/p&gt; </t>
+        </is>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>463</v>
+      </c>
       <c r="J55" s="2" t="s">
-        <v>474</v>
-      </c>
-      <c r="K55" s="2" t="s">
-        <v>475</v>
+        <v>464</v>
+      </c>
+      <c r="K55" s="1" t="s">
+        <v>465</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>476</v>
+        <v>466</v>
+      </c>
+      <c r="M55" s="1" t="s">
+        <v>176</v>
       </c>
       <c r="N55" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="56" customFormat="false" ht="332.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P55" s="1" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="n">
+        <v>1941</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>468</v>
+      </c>
+      <c r="D56" s="8" t="s">
+        <v>469</v>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/David_Lewis_(philosophe)"  title=" Wikipedia"&gt;David LEWIS&lt;/a&gt; était un philosophe américain connu pour sa théorie du  réalisme modal, selon laquelle il existe un nombre infini de mondes possibles concrets et causalement isolés les uns des autres. Son ouvrage majeur   &lt;a href="https://www.youtube.com/watch?v=-QlqLDLifuc" title="David Lewis - "De la pluralité des mondes" - De quoi parle ce livre ? par Philosophie 21"&gt;"On the Plurality of Worlds"&lt;/a&gt;  sortie en 1986, expose cette position révolutionnaire : pour lui, chaque monde possible existe aussi réellement que notre monde actuel, et sert à comprendre la modalité, c'est-à-dire ce qui pourrait être ou ce qui doit être. &lt;/p&gt; &lt;p&gt; Il a également proposé la théorie des contreparties en logique modale : au lieu de supposer que les personnes ou objets existent dans plusieurs mondes possibles, il affirme que chaque individu de notre monde a des « contreparties » dans les autres mondes possibles qui partagent certaines caractéristiques mais ne sont pas identiques à lui. Cette approche constitue une alternative à la logique modale traditionnelle, notamment celle de Saul Kripke. &lt;/p&gt; &lt;p&gt; Sa métaphysique est marquée par une conception atomiste (pointilliste) : la réalité n’est qu’une vaste mosaïque de faits locaux, chaque fait étant centré sur un « point » ayant des propriétés intrinsèques. Ce point de vue s’inspire de David Hume, d’où le nom « survenance humienne », refusant les liens nécessaires entre les faits et privilégiant une juxtaposition de qualités locales. &lt;/p&gt; &lt;p&gt; Il  a beaucoup écrit sur la philosophie du langage, la philosophie de l’esprit, l’épistémologie, la logique philosophique et la philosophie des mathématiques. Son premier grand ouvrage, "Convention" de 1969, analyse les conventions sociales à l’aide de la théorie des jeux, en montrant leur caractère arbitraire et leur diffusion par la connaissance commune et le précédent. Il s a marqué durablement la philosophie analytique.  &lt;a href="https://www.youtube.com/watch?v=g3jQwDP_Lyc" title="David Lewis - "David Lewis Speaks at La Trobe University par TimeSparrow"&gt;"Ses théories&lt;/a&gt; sont incontournables dans les débats sur les mondes possibles, la modalité, la causalité, la convention sociale, et l’atomisme métaphysique. Ses ouvrages, tels que Counterfactuals et Philosophical Papers, restent des références dans l’analyse logique et conceptuelle contemporaine. &lt;/p&gt; &lt;audio controls title=" On dit de David Lewis que c'est le plus grand métaphysicien qu’on ait vu depuis Leibniz par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/18292-28.02.2019-ITEMA_21995453-0.mp3" type="audio/mpeg" align="center"&gt;&lt;/audio&gt;  </t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="s">
+        <v>471</v>
+      </c>
+      <c r="G56" s="9" t="s">
+        <v>472</v>
+      </c>
+      <c r="H56" s="9" t="s">
+        <v>473</v>
+      </c>
+      <c r="I56" s="9"/>
+      <c r="J56" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="L56" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="N56" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="332.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="7" t="n">
         <v>1942</v>
       </c>
-      <c r="B56" s="7" t="s">
+      <c r="B57" s="7" t="s">
         <v>322</v>
       </c>
-      <c r="C56" s="7" t="s">
+      <c r="C57" s="7" t="s">
         <v>477</v>
       </c>
-      <c r="D56" s="8" t="s">
+      <c r="D57" s="8" t="s">
         <v>478</v>
       </c>
-      <c r="E56" s="9" t="inlineStr">
+      <c r="E57" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Daniel_Dennett"  style="color:#6A142A"  title=" Wikipedia"&gt;Daniel DENNETT&lt;/a&gt; était un  philosophe américain, figure importante et  influente de la philosophie de l'esprit, de la biologie et des sciences cognitives. Ses travaux se caractérisent par une volonté d'intégrer les découvertes scientifiques (biologie évolutionniste, neurosciences, intelligence artificielle) à la réflexion philosophique, souvent pour démanteler des intuitions traditionnelles qu'il juge erronées. &lt;/p&gt; &lt;p&gt; La Théorie de l'Esprit comme &lt;a href="https://www.youtube.com/watch?v=LKJJpvdqkFA" style="color:#88A1E9" title="Cette histoire va vous retourner le cerveau. | "Où suis-je" de Daniel Dennett par Monsieur Phi"&gt;"Position Intentionnelle"&lt;/a&gt; est sa contribution majeure. Il propose que pour prédire et expliquer le comportement d'un système (qu'il s'agisse d'un humain, d'un animal, d'un ordinateur ou même d'un thermostat), nous pouvons adopter trois "stances" : &lt;/p&gt; &lt;p&gt;La stance physique : On décrit le système par sa physique et sa chimie. Très difficile pour des systèmes complexes. &lt;/p&gt; &lt;p&gt;La stance du design : On considère le système comme conçu pour une fonction spécifique (ex: "ce thermostat est fait pour réguler la température"). &lt;/p&gt; &lt;p&gt;La stance intentionnelle : On traite le système comme s'il avait des croyances, des désirs et une rationalité. C'est une stratégie de prédiction extrêmement efficace, même si les croyances et désirs ne sont pas "réels" au sens littéral. Pour lui, avoir des croyances, c'est être un système dont le comportement peut être prédit avec succès par la stance intentionnelle. &lt;/p&gt; &lt;p&gt; Il est un matérialiste farouche et  rejette l'idée d'un &lt;a href="https://www.nonfiction.fr/article-1116-daniel_dennett_est_il_le_diable_.htm" title="Daniel Dennett est-il le diable ? par nonfiction"&gt;"théâtre cartésien"&lt;/a&gt;, un endroit dans le cerveau où tout se réunirait pour être "vu" par un &lt;a href="https://www.youtube.com/watch?v=0It9fwSj6xM"  title="Le moi comme illusion (Daniel Dennett, la conscience expliquée 4) par Philosophie Analytique"&gt;"spectateur" (le soi)&lt;/a&gt;. Pour lui, c'est une illusion.
 Il défend plutôt un modèle de "espace de travail global" : la conscience émerge de processus cérébraux parallèles et compétitifs. Une information devient "consciente" lorsqu'elle gagne une compétition pour être diffusée à grande échelle dans le cerveau, rendant ainsi disponible pour d'autres systèmes (mémoire, langage, prise de décision). Il n'y a pas de "centre" unique. &lt;/p&gt; &lt;p&gt; Il  considère que l'idée de la sélection naturelle de Darwin est "l'idée la plus dangereuse de tous les temps" car elle a un pouvoir explicatif immense, bien au-delà de la biologie. Il l'étend à d'autres domaines grâce au concept de "mèmes" (introduit par Richard Dawkins).
 Les mèmes sont des unités de culture (idées, mélodies, modes, concepts) qui se répliquent, mutent et sont sélectionnées dans le "payage" des esprits humains. Le langage,&lt;a href="https://www.youtube.com/shorts/bG3YBavy29Y" title="Cette histoire va vous retourner le cerveau | Daniel Dennett par StopCroyance"&gt; la religion&lt;/a&gt;, la morale peuvent être analysés comme des produits d'un processus darwinien. &lt;/p&gt; &lt;p&gt; Il défend une forme de libre arbitre qu'il estime compatible avec le déterminisme scientifique (le fait que l'univers soit régi par des lois causales). Pour lui, le libre arbitre n'est pas une "causalité magique" qui échapperait aux lois de la nature.  C'est la capacité d'un agent complexe (comme un être humain) à se projeter dans le futur, à évaluer les conséquences de ses actes et à agir en fonction de ses raisons. Ce libre arbitre est le produit de l'évolution et de la culture. Il est réel et précieux, même s'il n'est pas "libre" au sens d'une exemption des lois de la physique. &lt;/p&gt; &lt;audio controls title=" "Daniel Dennett, le penseur qui a révolutionné la philosophie des sciences et de l’esprit" par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/24419-10.05.2024-ITEMA_23737219-2024C51851S0131-21.mp3" type="audio/mpeg" align="center"&gt;&lt;/audio&gt; </t>
         </is>
       </c>
-      <c r="F56" s="7" t="s">
+      <c r="F57" s="7" t="s">
         <v>480</v>
       </c>
-      <c r="G56" s="9" t="s">
+      <c r="G57" s="9" t="s">
         <v>481</v>
       </c>
-      <c r="H56" s="9" t="s">
+      <c r="H57" s="9" t="s">
         <v>482</v>
       </c>
-      <c r="I56" s="9"/>
-      <c r="J56" s="2" t="s">
+      <c r="I57" s="9"/>
+      <c r="J57" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="K56" s="2" t="s">
+      <c r="K57" s="2" t="s">
         <v>483</v>
       </c>
-      <c r="L56" s="2" t="s">
+      <c r="L57" s="2" t="s">
         <v>484</v>
       </c>
-      <c r="N56" s="1" t="s">
+      <c r="N57" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="207" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="7" t="n">
+    <row r="58" customFormat="false" ht="207" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="7" t="n">
         <v>1943</v>
       </c>
-      <c r="B57" s="7" t="s">
+      <c r="B58" s="7" t="s">
         <v>449</v>
       </c>
-      <c r="C57" s="7" t="s">
+      <c r="C58" s="7" t="s">
         <v>485</v>
       </c>
-      <c r="D57" s="8" t="inlineStr">
+      <c r="D58" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Marilyn MCCORD-ADAMS</t>
         </is>
       </c>
-      <c r="E57" s="11" t="inlineStr">
+      <c r="E58" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Marilyn_McCord_Adams" title=" Wikipedia"&gt;Marilyn McCORD ADAMS&lt;/a&gt; était une philosophe américaine et une théologienne anglicane, reconnue pour son travail en philosophie de la religion et en philosophie médiévale. Elle a aussi été ordonnée prêtre épiscopalienne, ce qui donnait à sa réflexion philosophique une forte dimension spirituelle et pastorale. Elle a étudié à l’Université de l’Illinois puis à Cornell, où elle a obtenu son doctorat en philosophie en 1967. Sa carrière universitaire l’a menée à Michigan, UCLA, Yale, Oxford et elle a été la première femme, ainsi que la première Américaine, à occuper la chaire Regius de divinité à Oxford. &lt;/p&gt; &lt;p&gt;  &lt;a href="https://senate.universityofcalifornia.edu/in-memoriam/files/marilyn-adams.html" title="Marilyn Adans par university of california"&gt;Son apport le plus célèbre &lt;/a&gt; concerne l’étude de Guillaume d’Ockham, à qui elle a consacré une grande étude en deux volumes qui a beaucoup compté dans les recherches sur la théologie médiévale. Elle a aussi travaillé sur l’eucharistie, le christologie et d’autres auteurs médiévaux comme Thomas d’Aquin, Gilles de Rome et Duns Scot. &lt;/p&gt; &lt;p&gt; En  &lt;a href="https://www.youtube.com/watch?v=nFRGDG__ELM" title="Marilyn Adans par Real Atheology"&gt;philosophie de la religion, &lt;/a&gt; elle est connue pour ses analyses du mal extrême, qu’elle appelait les horrendous evils. Son idée centrale est qu’une théologie sérieuse doit prendre au sérieux les souffrances qui semblent détruire toute possibilité de sens, et montrer comment elles peuvent malgré tout être intégrées dans une vision de la bonté divine. &lt;/p&gt; &lt;p&gt; Son œuvre a eu une influence durable parce qu’elle relie la rigueur philosophique, l’érudition médiévale et l’expérience religieuse vécue. Elle reste une figure majeure pour comprendre à la fois la philosophie analytique de la religion et la redécouverte moderne de la pensée médiévale. &lt;/p&gt; 
 </t>
         </is>
       </c>
-      <c r="F57" s="7" t="s">
+      <c r="F58" s="7" t="s">
         <v>488</v>
       </c>
-      <c r="G57" s="9" t="s">
+      <c r="G58" s="9" t="s">
         <v>489</v>
       </c>
-      <c r="H57" s="9" t="s">
+      <c r="H58" s="9" t="s">
         <v>490</v>
       </c>
-      <c r="I57" s="9"/>
-      <c r="J57" s="2" t="s">
+      <c r="I58" s="9"/>
+      <c r="J58" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="K57" s="2" t="s">
+      <c r="K58" s="2" t="s">
         <v>475</v>
       </c>
-      <c r="L57" s="2" t="s">
+      <c r="L58" s="2" t="s">
         <v>491</v>
       </c>
-      <c r="M57" s="1" t="s">
+      <c r="M58" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N57" s="1" t="s">
+      <c r="N58" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="1" t="n">
+    <row r="59" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1" t="n">
         <v>1949</v>
       </c>
-      <c r="B58" s="1" t="n">
+      <c r="B59" s="1" t="n">
         <v>2006</v>
       </c>
-      <c r="C58" s="1" t="s">
+      <c r="C59" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="D58" s="1" t="s">
+      <c r="D59" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="E58" s="14" t="inlineStr">
+      <c r="E59" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Iris_Marion_Young" title=" Wikipedia"&gt;Iris Marion YOUNG&lt;/a&gt; était une philosophe politique américaine majeure, figure centrale du féminisme contemporain et de la théorie de la justice. Professeure à l'Université de Chicago, elle articule phénoménologie existentialiste, marxisme, théorie critique et postmodernisme pour repenser l'oppression, la domination et la démocratie au-delà des approches universalistes traditionnelles. &lt;/p&gt; &lt;p&gt; Sa contribution la plus célèbre est sa théorie des &lt;a href="https://www.youtube.com/watch?v=KyOut8zqJRI" title="les cinq visages de l’oppression par Eliot Goodine"&gt; cinq visages de l'oppression,&lt;/a&gt;  qu'elle développe dans Justice and the Politics of Difference (1990) ou elle développe également une,&lt;a href="https://www.persee.fr/doc/phlou_0035-3841_2018_num_116_4_8681" title="le féminisme phénoménologique par persée"&gt; phénoménologie féministe &lt;/a&gt; du corps, notamment dans son essai célèbre « Throwing Like a Girl » (1980). Elle y décrit comment les femmes vivent leur corps comme limité, fragmenté et constamment surveillé, ce qui produit une « immanence » sociale qui entrave leur capacité d'action et d'autodétermination. Le corps n'est pas seulement biologique mais politique, façonné par les normes sociales et les rapports de pouvoir. &lt;/p&gt; &lt;p&gt; Elle défend une conception de la justice fondée sur l'inclusion différenciée plutôt que sur l'universalisme abstrait. Pour Young, une société juste doit reconnaître les différences de groupe (genre, race, classe, sexualité) et créer des espaces où chacun puisse participer à la vie démocratique sans être forcé d'abandonner son identité particulière. Elle propose aussi le concept de responsabilité sociale diffuse, selon lequel tous les membres d'une société sont responsables des injustice structurelles, pas seulement les auteurs directs. &lt;/p&gt; &lt;p&gt; Elle évite tout essentialisme en conceptualisant « les femmes » comme un groupe social sériel, au sens de Sartre : un groupe dont les membres ne partagent pas une essence commune mais sont reliés par des conditions sociales similaires et des rapports de pouvoir. Cette approche permet un féminisme pluriel, Alliant diverses luttes (racisme, homophobie, validisme, écologie) dans des coalitions contre les rapports de domination. &lt;/p&gt; 
 </t>
         </is>
       </c>
-      <c r="F58" s="1" t="s">
+      <c r="F59" s="1" t="s">
         <v>495</v>
       </c>
-      <c r="G58" s="2" t="s">
+      <c r="G59" s="2" t="s">
         <v>496</v>
       </c>
-      <c r="H58" s="2" t="s">
+      <c r="H59" s="2" t="s">
         <v>497</v>
       </c>
-      <c r="J58" s="2" t="s">
+      <c r="J59" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="K58" s="2" t="s">
+      <c r="K59" s="2" t="s">
         <v>498</v>
       </c>
-      <c r="L58" s="2" t="s">
+      <c r="L59" s="2" t="s">
         <v>499</v>
       </c>
-      <c r="M58" s="1" t="s">
+      <c r="M59" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N58" s="1" t="s">
+      <c r="N59" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="1" t="n">
+    <row r="60" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1" t="n">
         <v>1952</v>
       </c>
-      <c r="B59" s="1" t="n">
+      <c r="B60" s="1" t="n">
         <v>2021</v>
       </c>
-      <c r="C59" s="1" t="s">
+      <c r="C60" s="1" t="s">
         <v>500</v>
       </c>
-      <c r="D59" s="1" t="s">
+      <c r="D60" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Bell_hooks"  title=" Wikipedia"&gt;Bell HOOKS&lt;/a&gt;, de son vrai nom Gloria Jean Watkins, est une autrice, professeure et militante féministe afro-américaine. Née dans le Kentucky, dans le Sud ségrégationniste, elle prit le nom de son arrière-grand-mère, qu'elle écrivait en minuscules pour que l'attention se porte sur ses idées plutôt que sur sa personne.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Ne suis-je pas une femme ?&lt;/em&gt; (1981), elle montre que les femmes noires ont été oubliées à la fois par le mouvement féministe, dominé par des femmes blanches de classe moyenne, et par le mouvement pour les droits civiques, dominé par des hommes. Elle  &lt;a href="https://www.youtube.com/watch?v=pCwMdHBSQgM" title=" bell hooks, un féminisme anticapitaliste et intersectionnel par META "&gt;développe l'idée &lt;/a&gt; que le sexisme, le racisme et l'exploitation économique forment un même système de domination, qu'elle appelle le « patriarcat capitaliste suprémaciste blanc ».&lt;/p&gt; &lt;p&gt;Ses idées ont profondément influencé ce que l'on appelle aujourd'hui l'intersectionnalité, c'est-à-dire l'étude de la manière dont différentes formes de discrimination se croisent et se renforcent. Elle écrivait dans un style simple et direct, refusant le jargon universitaire, pour que ses livres soient lus au-delà des cercles savants. Elle a aussi consacré plusieurs ouvrages à l'amour, qu'elle considérait comme une force politique capable de transformer la société.&lt;/p&gt; &lt;p&gt;Elle a écrit une quarantaine de livres, sur le féminisme, l'amour, les médias, la culture populaire et l'éducation. Dans &lt;em&gt;Apprendre à transgresser&lt;/em&gt; (1994), inspirée par Paulo Freire, elle défend une pédagogie de la liberté où l'enseignement devient une pratique d'émancipation. Pour elle, le féminisme n'est pas une guerre contre les hommes mais un mouvement pour mettre fin à toute forme de domination, porté par une « éthique de l'amour ».&lt;/p&gt;    &lt;audio controls title="Lire bell hooks aujourd’hui par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/23875-15.11.2023-ITEMA_23552434-2023C49162S0319-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;  
 </t>
         </is>
       </c>
-      <c r="F59" s="1" t="s">
+      <c r="F60" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="G59" s="2" t="s">
+      <c r="G60" s="2" t="s">
         <v>504</v>
       </c>
-      <c r="H59" s="2" t="s">
+      <c r="H60" s="2" t="s">
         <v>505</v>
       </c>
-      <c r="I59" s="1"/>
-      <c r="J59" s="2" t="s">
+      <c r="I60" s="1"/>
+      <c r="J60" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="K59" s="1" t="inlineStr">
+      <c r="K60" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Féminisme ; Wokisme</t>
         </is>
       </c>
-      <c r="L59" s="2" t="s">
+      <c r="L60" s="2" t="s">
         <v>507</v>
       </c>
-      <c r="M59" s="1" t="s">
+      <c r="M60" s="1" t="s">
         <v>508</v>
       </c>
-      <c r="N59" s="1" t="s">
+      <c r="N60" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="O59" s="1" t="n">
+      <c r="O60" s="1" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="293.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="0">
+    <row r="61" customFormat="false" ht="293.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="0">
         <v>1535</v>
       </c>
-      <c r="B60" s="0" t="inlineStr">
+      <c r="B61" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">1616</t>
         </is>
       </c>
-      <c r="C60" s="0" t="inlineStr">
+      <c r="C61" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">vers 1535 – vers 1616</t>
         </is>
       </c>
-      <c r="D60" s="0" t="inlineStr">
+      <c r="D61" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Felipe GUAMÁN POMA de Ayala</t>
         </is>
       </c>
-      <c r="E60" s="0" t="inlineStr">
+      <c r="E61" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Felipe_Guam%C3%A1n_Poma_de_Ayala" title=" Wikipedia"&gt;Felipe GUAMÁN POMA de Ayala&lt;/a&gt; est un noble andin de langue quechua, auteur de l’un des documents les plus extraordinaires de l’époque coloniale. Né dans la province de Lucanas, au Pérou, peu après la conquête espagnole, il descend par sa mère d’une lignée liée aux souverains de l’&lt;a href="https://fr.wikipedia.org/wiki/Empire_inca" title=" Wikipedia"&gt;Empire inca&lt;/a&gt;. Élevé parmi les Espagnols, il apprend leur langue, se fait chrétien et travaille comme interprète auprès d’un prêtre chargé d’extirper les « idolâtries », puis auprès de juges de Huamanga, avant d’être dépouillé de ses terres et banni vers 1600.&lt;/p&gt; &lt;p&gt;Il parcourt alors les Andes pendant des années et rédige, vers 1615, une lettre de près de 1 200 pages adressée au roi d’Espagne Philippe III : la &lt;em&gt;Nouvelle Chronique et bon gouvernement&lt;/em&gt;. Ses quelque 400 dessins à la plume racontent l’histoire des Incas, le calendrier, les travaux des champs, puis les abus des colons : prêtres, corregidors et propriétaires qui exploitent, volent et maltraitent les Indiens. Il y décrit un « monde à l’envers » (&lt;em&gt;mundo al revés&lt;/em&gt;), où l’ordre juste a été renversé par la conquête.&lt;/p&gt; &lt;p&gt;Il ne réclame pas le départ des Espagnols, mais un « bon gouvernement » : que les Andins se gouvernent eux-mêmes sous l’autorité lointaine du roi, et que les colons qui abusent soient chassés des villages. Il défend aussi la valeur de la civilisation andine, qui connaissait selon lui la justice et un ordre moral bien avant l’arrivée des Européens. Le manuscrit, qui n’atteignit sans doute jamais le roi, dormit pendant trois siècles avant d’être découvert en 1908 à la Bibliothèque royale de Copenhague. Il est aujourd’hui une source majeure sur le monde andin et l’une des premières critiques de la colonisation écrites par un colonisé.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F60" s="0"/>
-      <c r="G60" s="0"/>
-      <c r="H60" s="0" t="inlineStr">
+      <c r="F61" s="0"/>
+      <c r="G61" s="0"/>
+      <c r="H61" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/guamanpoma-mini.webp</t>
         </is>
       </c>
-      <c r="I60" s="0"/>
-      <c r="J60" s="0" t="inlineStr">
+      <c r="I61" s="0"/>
+      <c r="J61" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">politique ; ethique</t>
         </is>
       </c>
-      <c r="K60" s="0" t="inlineStr">
+      <c r="K61" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Anticolonialisme</t>
         </is>
       </c>
-      <c r="L60" s="0" t="inlineStr">
+      <c r="L61" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">chroniqueur andin, auteur d’une immense lettre illustrée au roi d’Espagne dénonçant la colonisation du Pérou.</t>
         </is>
       </c>
-      <c r="M60" s="0"/>
-      <c r="N60" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sud</t>
-        </is>
-      </c>
-      <c r="O60" s="1">
-        <v>2</v>
-      </c>
-      <c r="P60" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Péruvienne</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="1">
-        <v>1853</v>
-      </c>
-      <c r="B61" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1895</t>
-        </is>
-      </c>
-      <c r="C61" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1853 – 1895</t>
-        </is>
-      </c>
-      <c r="D61" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">José MARTÍ</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jos%C3%A9_Mart%C3%AD" title=" Wikipedia"&gt;José MARTÍ&lt;/a&gt; est le grand penseur de l’indépendance cubaine et l’une des voix majeures de l’Amérique latine. Né à La Havane de parents espagnols, il est arrêté à seize ans pour ses idées indépendantistes et condamné aux travaux forcés dans une carrière, avant d’être déporté en Espagne, où il étudie le droit et la philosophie à Saragosse. Il vit ensuite au Mexique, au Guatemala et au Venezuela, puis s’installe en 1881 à New York, où il passe près de quinze ans comme journaliste, diplomate et organisateur de l’exil cubain. Il y écrit, pour de grands journaux d’Amérique latine, des chroniques sur la vie nord-américaine.&lt;/p&gt; &lt;p&gt;Dans son essai &lt;em&gt;Notre Amérique&lt;/em&gt; (1891), il appelle les nations latino-américaines à se penser à partir de leur propre réalité, métisse, indienne, noire et paysanne, plutôt qu’en copiant l’Europe ou les États-Unis : « Le gouvernement doit naître du pays. » Il y affirme aussi : « Il n’y a pas de haine des races, parce qu’il n’y a pas de races. » Observateur lucide de la puissance nord-américaine, il met en garde contre les ambitions des États-Unis sur Cuba et sur tout le continent.&lt;/p&gt; &lt;p&gt;Poète novateur, l’un des fondateurs du modernisme hispanique, il écrit les &lt;em&gt;Vers simples&lt;/em&gt; (1891), dont certains forment les paroles de la célèbre chanson &lt;em&gt;Guantanamera&lt;/em&gt;, et une revue pour les enfants, &lt;em&gt;L’Âge d’or&lt;/em&gt;. En 1892, il fonde le Parti révolutionnaire cubain et prépare la &lt;a href="https://fr.wikipedia.org/wiki/Guerre_d%27ind%C3%A9pendance_cubaine" title=" Wikipedia"&gt;guerre d’indépendance&lt;/a&gt;. Débarqué à Cuba avec les insurgés, il est tué au combat à Dos Ríos le 19 mai 1895. Il est considéré à Cuba comme le héros national et « l’Apôtre » de l’indépendance.&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="H61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/marti-mini.webp</t>
-        </is>
-      </c>
-      <c r="I61" s="1"/>
-      <c r="J61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">politique ; esthetique</t>
-        </is>
-      </c>
-      <c r="K61" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Anticolonialisme ; Humanisme</t>
-        </is>
-      </c>
-      <c r="L61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">poète et penseur de l’indépendance cubaine, auteur de « Notre Amérique », héros national de Cuba.</t>
-        </is>
-      </c>
+      <c r="M61" s="0"/>
       <c r="N61" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">sud</t>
@@ -4936,54 +4933,55 @@
       <c r="O61" s="1">
         <v>2</v>
       </c>
-      <c r="P61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cubaine</t>
+      <c r="P61" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Péruvienne</t>
         </is>
       </c>
     </row>
     <row r="62" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1">
-        <v>1921</v>
+        <v>1853</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1997</t>
+          <t xml:space="preserve">1895</t>
         </is>
       </c>
       <c r="C62" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1921 – 1997</t>
+          <t xml:space="preserve">1853 – 1895</t>
         </is>
       </c>
       <c r="D62" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paulo FREIRE</t>
+          <t xml:space="preserve">José MARTÍ</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Paulo_Freire" title=" Wikipedia"&gt;Paulo FREIRE&lt;/a&gt; est un pédagogue et philosophe brésilien, l’un des penseurs de l’éducation les plus lus au monde. Né à Recife, dans le Nordeste, il connaît la faim pendant la crise des années 1930, ce qui le marque pour toute sa vie. Formé au droit et à la philosophie, lecteur de Marx comme des penseurs chrétiens, il se consacre à l’&lt;a href="https://fr.wikipedia.org/wiki/Alphab%C3%A9tisation" title=" Wikipedia"&gt;alphabétisation&lt;/a&gt; des adultes pauvres. En 1963, à Angicos, sa méthode permet à 300 travailleurs agricoles d’apprendre à lire et à écrire en une quarantaine d’heures.&lt;/p&gt; &lt;p&gt;Sa méthode part des « mots générateurs » tirés de la vie des apprenants, comme la brique, la terre ou le salaire, et fait de la lecture une prise de conscience : apprendre à lire le mot, c’est apprendre à lire le monde. Après le coup d’État militaire de 1964, il est emprisonné puis contraint à un exil de seize ans. Au Chili, il écrit &lt;a href="https://fr.wikipedia.org/wiki/P%C3%A9dagogie_des_opprim%C3%A9s" title=" Wikipedia"&gt;&lt;em&gt;Pédagogie des opprimés&lt;/em&gt;&lt;/a&gt; (1968), où il critique l’éducation « bancaire », qui dépose des savoirs dans des élèves passifs comme on remplit un coffre, et lui oppose une éducation par le dialogue, où maître et élèves cherchent ensemble.&lt;/p&gt; &lt;p&gt;« Personne n’éduque autrui, personne ne s’éduque seul, les hommes s’éduquent ensemble par l’intermédiaire du monde. » L’éducation n’est jamais neutre : elle maintient l’oppression ou aide les opprimés à s’en libérer, sans devenir à leur tour oppresseurs. Rentré au Brésil en 1980, il dirige l’éducation de la ville de São Paulo. Son œuvre est à l’origine de la &lt;a href="https://fr.wikipedia.org/wiki/P%C3%A9dagogie_critique" title=" Wikipedia"&gt;pédagogie critique&lt;/a&gt;, et il a été proclamé en 2012 patron de l’éducation brésilienne.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jos%C3%A9_Mart%C3%AD" title=" Wikipedia"&gt;José MARTÍ&lt;/a&gt; est le grand penseur de l’indépendance cubaine et l’une des voix majeures de l’Amérique latine. Né à La Havane de parents espagnols, il est arrêté à seize ans pour ses idées indépendantistes et condamné aux travaux forcés dans une carrière, avant d’être déporté en Espagne, où il étudie le droit et la philosophie à Saragosse. Il vit ensuite au Mexique, au Guatemala et au Venezuela, puis s’installe en 1881 à New York, où il passe près de quinze ans comme journaliste, diplomate et organisateur de l’exil cubain. Il y écrit, pour de grands journaux d’Amérique latine, des chroniques sur la vie nord-américaine.&lt;/p&gt; &lt;p&gt;Dans son essai &lt;em&gt;Notre Amérique&lt;/em&gt; (1891), il appelle les nations latino-américaines à se penser à partir de leur propre réalité, métisse, indienne, noire et paysanne, plutôt qu’en copiant l’Europe ou les États-Unis : « Le gouvernement doit naître du pays. » Il y affirme aussi : « Il n’y a pas de haine des races, parce qu’il n’y a pas de races. » Observateur lucide de la puissance nord-américaine, il met en garde contre les ambitions des États-Unis sur Cuba et sur tout le continent.&lt;/p&gt; &lt;p&gt;Poète novateur, l’un des fondateurs du modernisme hispanique, il écrit les &lt;em&gt;Vers simples&lt;/em&gt; (1891), dont certains forment les paroles de la célèbre chanson &lt;em&gt;Guantanamera&lt;/em&gt;, et une revue pour les enfants, &lt;em&gt;L’Âge d’or&lt;/em&gt;. En 1892, il fonde le Parti révolutionnaire cubain et prépare la &lt;a href="https://fr.wikipedia.org/wiki/Guerre_d%27ind%C3%A9pendance_cubaine" title=" Wikipedia"&gt;guerre d’indépendance&lt;/a&gt;. Débarqué à Cuba avec les insurgés, il est tué au combat à Dos Ríos le 19 mai 1895. Il est considéré à Cuba comme le héros national et « l’Apôtre » de l’indépendance.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/freire-mini.webp</t>
-        </is>
-      </c>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/marti-mini.webp</t>
+        </is>
+      </c>
+      <c r="I62" s="1"/>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ethique ; politique</t>
+          <t xml:space="preserve">politique ; esthetique</t>
         </is>
       </c>
       <c r="K62" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Humanisme ; Marxisme ; Théologie de la libération</t>
+          <t xml:space="preserve">Anticolonialisme ; Humanisme</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">pédagogue brésilien, auteur de Pédagogie des opprimés, penseur de l’éducation comme pratique de la liberté.</t>
+          <t xml:space="preserve">poète et penseur de l’indépendance cubaine, auteur de « Notre Amérique », héros national de Cuba.</t>
         </is>
       </c>
       <c r="N62" s="1" t="inlineStr">
@@ -4992,56 +4990,56 @@
         </is>
       </c>
       <c r="O62" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brésilienne</t>
+          <t xml:space="preserve">Cubaine</t>
         </is>
       </c>
     </row>
     <row r="63" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1">
-        <v>1882</v>
+        <v>1921</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1959</t>
+          <t xml:space="preserve">1997</t>
         </is>
       </c>
       <c r="C63" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1882 – 1959</t>
+          <t xml:space="preserve">1921 – 1997</t>
         </is>
       </c>
       <c r="D63" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">José VASCONCELOS</t>
+          <t xml:space="preserve">Paulo FREIRE</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jos%C3%A9_Vasconcelos" title=" Wikipedia"&gt;José VASCONCELOS&lt;/a&gt; est un philosophe, écrivain et homme politique mexicain, l’un des grands éducateurs de l’Amérique latine. Né à Oaxaca, avocat, il fonde en 1909 avec Antonio Caso et Alfonso Reyes l’Ateneo de la Juventud, cercle de jeunes intellectuels qui rejette le positivisme officiel du régime de Porfirio Díaz. Il prend part à la &lt;a href="https://fr.wikipedia.org/wiki/R%C3%A9volution_mexicaine" title=" Wikipedia"&gt;révolution mexicaine&lt;/a&gt; aux côtés de Francisco Madero. Recteur de l’université nationale en 1920, il lui donne sa devise, toujours en usage : « Par ma race parlera l’esprit. »&lt;/p&gt; &lt;p&gt;Ministre de l’Éducation de 1921 à 1924, il mène une véritable croisade pour instruire le peuple : écoles rurales, missions culturelles dans les villages, bibliothèques, éditions populaires des grands classiques. Il commande aussi aux peintres &lt;a href="https://fr.wikipedia.org/wiki/Diego_Rivera" title=" Wikipedia"&gt;Diego Rivera&lt;/a&gt; et José Clemente Orozco les fresques murales qui racontent l’histoire du Mexique sur les murs des bâtiments publics. Il est surnommé le « maître de la jeunesse d’Amérique ».&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;La Race cosmique&lt;/em&gt; (1925), il prophétise que l’Amérique latine, terre de tous les mélanges, verra naître une « cinquième race », synthèse de toutes les autres, porteuse d’une civilisation de l’amour et de la beauté. Sa philosophie, un « monisme esthétique », voit dans l’émotion esthétique la forme la plus haute de connaissance. Battu en 1929 dans une élection présidentielle qu’il juge truquée, il s’exile, puis évolue vers un conservatisme catholique, au point de manifester en 1940 des sympathies pour l’Allemagne nazie. Il meurt à Mexico en 1959.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Paulo_Freire" title=" Wikipedia"&gt;Paulo FREIRE&lt;/a&gt; est un pédagogue et philosophe brésilien, l’un des penseurs de l’éducation les plus lus au monde. Né à Recife, dans le Nordeste, il connaît la faim pendant la crise des années 1930, ce qui le marque pour toute sa vie. Formé au droit et à la philosophie, lecteur de Marx comme des penseurs chrétiens, il se consacre à l’&lt;a href="https://fr.wikipedia.org/wiki/Alphab%C3%A9tisation" title=" Wikipedia"&gt;alphabétisation&lt;/a&gt; des adultes pauvres. En 1963, à Angicos, sa méthode permet à 300 travailleurs agricoles d’apprendre à lire et à écrire en une quarantaine d’heures.&lt;/p&gt; &lt;p&gt;Sa méthode part des « mots générateurs » tirés de la vie des apprenants, comme la brique, la terre ou le salaire, et fait de la lecture une prise de conscience : apprendre à lire le mot, c’est apprendre à lire le monde. Après le coup d’État militaire de 1964, il est emprisonné puis contraint à un exil de seize ans. Au Chili, il écrit &lt;a href="https://fr.wikipedia.org/wiki/P%C3%A9dagogie_des_opprim%C3%A9s" title=" Wikipedia"&gt;&lt;em&gt;Pédagogie des opprimés&lt;/em&gt;&lt;/a&gt; (1968), où il critique l’éducation « bancaire », qui dépose des savoirs dans des élèves passifs comme on remplit un coffre, et lui oppose une éducation par le dialogue, où maître et élèves cherchent ensemble.&lt;/p&gt; &lt;p&gt;« Personne n’éduque autrui, personne ne s’éduque seul, les hommes s’éduquent ensemble par l’intermédiaire du monde. » L’éducation n’est jamais neutre : elle maintient l’oppression ou aide les opprimés à s’en libérer, sans devenir à leur tour oppresseurs. Rentré au Brésil en 1980, il dirige l’éducation de la ville de São Paulo. Son œuvre est à l’origine de la &lt;a href="https://fr.wikipedia.org/wiki/P%C3%A9dagogie_critique" title=" Wikipedia"&gt;pédagogie critique&lt;/a&gt;, et il a été proclamé en 2012 patron de l’éducation brésilienne.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/vasconcelos-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/freire-mini.webp</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">esthetique ; politique</t>
+          <t xml:space="preserve">ethique ; politique</t>
         </is>
       </c>
       <c r="K63" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monisme ; Spiritualisme</t>
+          <t xml:space="preserve">Humanisme ; Marxisme ; Théologie de la libération</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe et ministre mexicain de l’Éducation, auteur de La Race cosmique, penseur du métissage.</t>
+          <t xml:space="preserve">pédagogue brésilien, auteur de Pédagogie des opprimés, penseur de l’éducation comme pratique de la liberté.</t>
         </is>
       </c>
       <c r="N63" s="1" t="inlineStr">
@@ -5050,66 +5048,61 @@
         </is>
       </c>
       <c r="O63" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mexicaine</t>
+          <t xml:space="preserve">Brésilienne</t>
         </is>
       </c>
     </row>
     <row r="64" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1">
-        <v>1907</v>
+        <v>1882</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1972</t>
+          <t xml:space="preserve">1959</t>
         </is>
       </c>
       <c r="C64" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1907 – 1972</t>
+          <t xml:space="preserve">1882 – 1959</t>
         </is>
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abraham Joshua HESCHEL</t>
+          <t xml:space="preserve">José VASCONCELOS</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Abraham_Joshua_Heschel" title=" Wikipedia"&gt;Abraham Joshua HESCHEL&lt;/a&gt; est un rabbin, théologien et philosophe juif, l’une des grandes voix religieuses du XXe siècle. Né à Varsovie dans une illustre famille du &lt;a href="https://fr.wikipedia.org/wiki/Hassidisme" title=" Wikipedia"&gt;hassidisme&lt;/a&gt;, il étudie la philosophie à Berlin, où il soutient une thèse sur les prophètes d’Israël. Expulsé d’Allemagne vers la Pologne en 1938, il parvient à quitter Varsovie quelques semaines avant l’invasion allemande et gagne Londres, puis les États-Unis. Sa mère et ses sœurs sont assassinées pendant la Shoah. Il enseigne à partir de 1946 au Séminaire théologique juif de New York.&lt;/p&gt; &lt;p&gt;Pour Heschel, la religion commence par l’« étonnement radical » devant le monde, qui précède toute réflexion. Contre l’idée d’un Dieu impassible des philosophes, il parle du « pathos divin » : le Dieu des prophètes est concerné par le sort des hommes et souffre de l’injustice. La question n’est pas seulement de savoir si l’homme cherche Dieu, mais de comprendre que &lt;em&gt;Dieu est en quête de l’homme&lt;/em&gt;, titre de son livre de 1955. Dans &lt;em&gt;Les Bâtisseurs du temps&lt;/em&gt; (1951), il présente le &lt;a href="https://fr.wikipedia.org/wiki/Shabbat" title=" Wikipedia"&gt;shabbat&lt;/a&gt; comme « une cathédrale dans le temps » : le judaïsme sanctifie des moments plutôt que des lieux. Il consacre aussi un grand livre aux prophètes, témoins de la passion de Dieu pour la justice.&lt;/p&gt; &lt;p&gt;Sa foi le conduit à l’action. En 1965, il marche de Selma à Montgomery aux côtés de Martin Luther King et dira : « J’avais l’impression que mes jambes priaient. » Il s’oppose à la guerre du Vietnam et contribue au dialogue entre juifs et chrétiens lors du concile Vatican II. Il meurt à New York en 1972.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jos%C3%A9_Vasconcelos" title=" Wikipedia"&gt;José VASCONCELOS&lt;/a&gt; est un philosophe, écrivain et homme politique mexicain, l’un des grands éducateurs de l’Amérique latine. Né à Oaxaca, avocat, il fonde en 1909 avec Antonio Caso et Alfonso Reyes l’Ateneo de la Juventud, cercle de jeunes intellectuels qui rejette le positivisme officiel du régime de Porfirio Díaz. Il prend part à la &lt;a href="https://fr.wikipedia.org/wiki/R%C3%A9volution_mexicaine" title=" Wikipedia"&gt;révolution mexicaine&lt;/a&gt; aux côtés de Francisco Madero. Recteur de l’université nationale en 1920, il lui donne sa devise, toujours en usage : « Par ma race parlera l’esprit. »&lt;/p&gt; &lt;p&gt;Ministre de l’Éducation de 1921 à 1924, il mène une véritable croisade pour instruire le peuple : écoles rurales, missions culturelles dans les villages, bibliothèques, éditions populaires des grands classiques. Il commande aussi aux peintres &lt;a href="https://fr.wikipedia.org/wiki/Diego_Rivera" title=" Wikipedia"&gt;Diego Rivera&lt;/a&gt; et José Clemente Orozco les fresques murales qui racontent l’histoire du Mexique sur les murs des bâtiments publics. Il est surnommé le « maître de la jeunesse d’Amérique ».&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;La Race cosmique&lt;/em&gt; (1925), il prophétise que l’Amérique latine, terre de tous les mélanges, verra naître une « cinquième race », synthèse de toutes les autres, porteuse d’une civilisation de l’amour et de la beauté. Sa philosophie, un « monisme esthétique », voit dans l’émotion esthétique la forme la plus haute de connaissance. Battu en 1929 dans une élection présidentielle qu’il juge truquée, il s’exile, puis évolue vers un conservatisme catholique, au point de manifester en 1940 des sympathies pour l’Allemagne nazie. Il meurt à Mexico en 1959.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/heschel-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/vasconcelos-mini.webp</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">spiritualite ; ethique</t>
+          <t xml:space="preserve">esthetique ; politique</t>
         </is>
       </c>
       <c r="K64" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existentialisme ; Mysticisme ; Hassidisme</t>
+          <t xml:space="preserve">Monisme ; Spiritualisme</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rabbin et philosophe juif, penseur du « pathos divin » et du shabbat, militant des droits civiques.</t>
-        </is>
-      </c>
-      <c r="M64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">juive</t>
+          <t xml:space="preserve">philosophe et ministre mexicain de l’Éducation, auteur de La Race cosmique, penseur du métissage.</t>
         </is>
       </c>
       <c r="N64" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">occident</t>
+          <t xml:space="preserve">sud</t>
         </is>
       </c>
       <c r="O64" s="1">
@@ -5117,57 +5110,62 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Américaine</t>
+          <t xml:space="preserve">Mexicaine</t>
         </is>
       </c>
     </row>
     <row r="65" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1">
-        <v>1914</v>
+        <v>1907</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1998</t>
+          <t xml:space="preserve">1972</t>
         </is>
       </c>
       <c r="C65" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1914 – 1998</t>
+          <t xml:space="preserve">1907 – 1972</t>
         </is>
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Octavio PAZ</t>
+          <t xml:space="preserve">Abraham Joshua HESCHEL</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Octavio_Paz" title=" Wikipedia"&gt;Octavio PAZ&lt;/a&gt; est un poète, essayiste et diplomate mexicain, prix Nobel de littérature en 1990. Né à Mexico dans une famille marquée par la révolution, son père ayant été le représentant d’Emiliano Zapata aux États-Unis, il soutient les républicains pendant la guerre d’Espagne, puis rompt avec le communisme après l’assassinat de Trotski. Diplomate à Paris après la guerre, il y fréquente les surréalistes et André Breton.&lt;/p&gt; &lt;p&gt;Dans &lt;a href="https://fr.wikipedia.org/wiki/Le_Labyrinthe_de_la_solitude" title=" Wikipedia"&gt;&lt;em&gt;Le Labyrinthe de la solitude&lt;/em&gt;&lt;/a&gt; (1950), il interroge l’identité mexicaine : derrière les masques de la politesse et la violence des fêtes se cache une solitude née de l’histoire, celle d’un peuple issu de la conquête, qui a renié à la fois son passé indien et son passé espagnol. Il y évoque la figure de la &lt;a href="https://fr.wikipedia.org/wiki/La_Malinche" title=" Wikipedia"&gt;Malinche&lt;/a&gt;, compagne indienne de Cortés, symbole ambigu de l’origine métisse du pays. Mais cette solitude est aussi celle de l’homme moderne, et la poésie, l’amour et la fête sont des moyens de la dépasser. Dans &lt;em&gt;L’Arc et la Lyre&lt;/em&gt; (1956), il fait de la poésie une expérience de communion qui révèle l’homme à lui-même.&lt;/p&gt; &lt;p&gt;Ambassadeur du Mexique en Inde de 1962 à 1968, il découvre les philosophies et l’art de l’Orient, qui nourrissent sa poésie. Il démissionne après le &lt;a href="https://fr.wikipedia.org/wiki/Massacre_de_Tlatelolco" title=" Wikipedia"&gt;massacre de Tlatelolco&lt;/a&gt;, où des centaines d’étudiants sont tués par l’armée en 1968. Critique des totalitarismes de droite comme de gauche, il fonde la revue &lt;em&gt;Vuelta&lt;/em&gt; et consacre un grand livre à la poétesse et penseuse Juana Inés de la Cruz. Il meurt à Mexico en 1998, à quatre-vingt-quatre ans.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Abraham_Joshua_Heschel" title=" Wikipedia"&gt;Abraham Joshua HESCHEL&lt;/a&gt; est un rabbin, théologien et philosophe juif, l’une des grandes voix religieuses du XXe siècle. Né à Varsovie dans une illustre famille du &lt;a href="https://fr.wikipedia.org/wiki/Hassidisme" title=" Wikipedia"&gt;hassidisme&lt;/a&gt;, il étudie la philosophie à Berlin, où il soutient une thèse sur les prophètes d’Israël. Expulsé d’Allemagne vers la Pologne en 1938, il parvient à quitter Varsovie quelques semaines avant l’invasion allemande et gagne Londres, puis les États-Unis. Sa mère et ses sœurs sont assassinées pendant la Shoah. Il enseigne à partir de 1946 au Séminaire théologique juif de New York.&lt;/p&gt; &lt;p&gt;Pour Heschel, la religion commence par l’« étonnement radical » devant le monde, qui précède toute réflexion. Contre l’idée d’un Dieu impassible des philosophes, il parle du « pathos divin » : le Dieu des prophètes est concerné par le sort des hommes et souffre de l’injustice. La question n’est pas seulement de savoir si l’homme cherche Dieu, mais de comprendre que &lt;em&gt;Dieu est en quête de l’homme&lt;/em&gt;, titre de son livre de 1955. Dans &lt;em&gt;Les Bâtisseurs du temps&lt;/em&gt; (1951), il présente le &lt;a href="https://fr.wikipedia.org/wiki/Shabbat" title=" Wikipedia"&gt;shabbat&lt;/a&gt; comme « une cathédrale dans le temps » : le judaïsme sanctifie des moments plutôt que des lieux. Il consacre aussi un grand livre aux prophètes, témoins de la passion de Dieu pour la justice.&lt;/p&gt; &lt;p&gt;Sa foi le conduit à l’action. En 1965, il marche de Selma à Montgomery aux côtés de Martin Luther King et dira : « J’avais l’impression que mes jambes priaient. » Il s’oppose à la guerre du Vietnam et contribue au dialogue entre juifs et chrétiens lors du concile Vatican II. Il meurt à New York en 1972.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/paz-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/heschel-mini.webp</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">esthetique ; politique</t>
+          <t xml:space="preserve">spiritualite ; ethique</t>
         </is>
       </c>
       <c r="K65" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Humanisme</t>
+          <t xml:space="preserve">Existentialisme ; Mysticisme ; Hassidisme</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">poète et essayiste mexicain, prix Nobel 1990, auteur du Labyrinthe de la solitude.</t>
+          <t xml:space="preserve">rabbin et philosophe juif, penseur du « pathos divin » et du shabbat, militant des droits civiques.</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
         </is>
       </c>
       <c r="N65" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">sud</t>
+          <t xml:space="preserve">occident</t>
         </is>
       </c>
       <c r="O65" s="1">
@@ -5175,52 +5173,52 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mexicaine</t>
+          <t xml:space="preserve">Américaine</t>
         </is>
       </c>
     </row>
     <row r="66" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1">
-        <v>1871</v>
+        <v>1914</v>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1917</t>
+          <t xml:space="preserve">1998</t>
         </is>
       </c>
       <c r="C66" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1871 – 1917</t>
+          <t xml:space="preserve">1914 – 1998</t>
         </is>
       </c>
       <c r="D66" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">José Enrique RODÓ</t>
+          <t xml:space="preserve">Octavio PAZ</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jos%C3%A9_Enrique_Rod%C3%B3" title=" Wikipedia"&gt;José Enrique RODÓ&lt;/a&gt; est un écrivain et essayiste uruguayen, l’un des grands maîtres à penser de l’Amérique latine au début du XXe siècle. Né à Montevideo, il doit interrompre ses études après la ruine de sa famille, se forme largement seul et devient professeur de littérature à l’université de Montevideo, puis député. Correspondant de &lt;a href="https://fr.wikipedia.org/wiki/Rub%C3%A9n_Dar%C3%ADo" title=" Wikipedia"&gt;Rubén Darío&lt;/a&gt;, il est le principal théoricien du modernisme, le grand mouvement de renouvellement de la littérature hispano-américaine.&lt;/p&gt; &lt;p&gt;Son essai &lt;em&gt;Ariel&lt;/em&gt; (1900), écrit deux ans après la victoire des États-Unis sur l’Espagne à Cuba, prend la forme d’un dernier cours donné par un vieux maître, Prospero, à ses élèves. Empruntant les personnages de &lt;em&gt;La Tempête&lt;/em&gt; de Shakespeare, il oppose Ariel, l’esprit, la beauté, le désintéressement, à Caliban, la matière, l’utilité, les appétits. Il met en garde la jeunesse latino-américaine contre l’utilitarisme et la « nordomanie », la fascination pour le modèle des États-Unis, puissant mais tourné vers le seul profit.&lt;/p&gt; &lt;p&gt;Rodó invite les jeunes à cultiver toutes les facultés de l’esprit, à préserver un temps libre pour la pensée et la beauté, et à construire une démocratie qui élève chacun au lieu de niveler par le bas. Le livre connut un immense succès et inspira tout un courant, l’« arielisme ». Plus tard, des penseurs comme Roberto Fernández Retamar ont renversé le symbole en faisant de Caliban la figure du colonisé. Dans &lt;em&gt;Motifs de Protée&lt;/em&gt; (1909), il médite sur la transformation continuelle de soi. Rodó meurt à Palerme en 1917, au cours d’un voyage en Europe.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Octavio_Paz" title=" Wikipedia"&gt;Octavio PAZ&lt;/a&gt; est un poète, essayiste et diplomate mexicain, prix Nobel de littérature en 1990. Né à Mexico dans une famille marquée par la révolution, son père ayant été le représentant d’Emiliano Zapata aux États-Unis, il soutient les républicains pendant la guerre d’Espagne, puis rompt avec le communisme après l’assassinat de Trotski. Diplomate à Paris après la guerre, il y fréquente les surréalistes et André Breton.&lt;/p&gt; &lt;p&gt;Dans &lt;a href="https://fr.wikipedia.org/wiki/Le_Labyrinthe_de_la_solitude" title=" Wikipedia"&gt;&lt;em&gt;Le Labyrinthe de la solitude&lt;/em&gt;&lt;/a&gt; (1950), il interroge l’identité mexicaine : derrière les masques de la politesse et la violence des fêtes se cache une solitude née de l’histoire, celle d’un peuple issu de la conquête, qui a renié à la fois son passé indien et son passé espagnol. Il y évoque la figure de la &lt;a href="https://fr.wikipedia.org/wiki/La_Malinche" title=" Wikipedia"&gt;Malinche&lt;/a&gt;, compagne indienne de Cortés, symbole ambigu de l’origine métisse du pays. Mais cette solitude est aussi celle de l’homme moderne, et la poésie, l’amour et la fête sont des moyens de la dépasser. Dans &lt;em&gt;L’Arc et la Lyre&lt;/em&gt; (1956), il fait de la poésie une expérience de communion qui révèle l’homme à lui-même.&lt;/p&gt; &lt;p&gt;Ambassadeur du Mexique en Inde de 1962 à 1968, il découvre les philosophies et l’art de l’Orient, qui nourrissent sa poésie. Il démissionne après le &lt;a href="https://fr.wikipedia.org/wiki/Massacre_de_Tlatelolco" title=" Wikipedia"&gt;massacre de Tlatelolco&lt;/a&gt;, où des centaines d’étudiants sont tués par l’armée en 1968. Critique des totalitarismes de droite comme de gauche, il fonde la revue &lt;em&gt;Vuelta&lt;/em&gt; et consacre un grand livre à la poétesse et penseuse Juana Inés de la Cruz. Il meurt à Mexico en 1998, à quatre-vingt-quatre ans.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/rodo-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/paz-mini.webp</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">esthetique ; ethique</t>
+          <t xml:space="preserve">esthetique ; politique</t>
         </is>
       </c>
       <c r="K66" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Humanisme ; Spiritualisme</t>
+          <t xml:space="preserve">Humanisme</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">essayiste uruguayen, auteur d’Ariel, maître à penser de la jeunesse latino-américaine.</t>
+          <t xml:space="preserve">poète et essayiste mexicain, prix Nobel 1990, auteur du Labyrinthe de la solitude.</t>
         </is>
       </c>
       <c r="N66" s="1" t="inlineStr">
@@ -5233,52 +5231,52 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uruguayenne</t>
+          <t xml:space="preserve">Mexicaine</t>
         </is>
       </c>
     </row>
     <row r="67" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1">
-        <v>1922</v>
+        <v>1871</v>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1979</t>
+          <t xml:space="preserve">1917</t>
         </is>
       </c>
       <c r="C67" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1922 – 1979</t>
+          <t xml:space="preserve">1871 – 1917</t>
         </is>
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rodolfo KUSCH</t>
+          <t xml:space="preserve">José Enrique RODÓ</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://es.wikipedia.org/wiki/Rodolfo_Kusch" title=" Wikipedia (es)"&gt;Rodolfo KUSCH&lt;/a&gt; est un philosophe et anthropologue argentin qui a cherché à fonder une philosophie à partir de la pensée indigène et populaire de l’Amérique. Né à Buenos Aires de parents allemands, il étudie la philosophie à l’université de Buenos Aires, enseigne l’esthétique et écrit aussi pour le théâtre, notamment sur le tango. Persécuté pour ses sympathies péronistes après 1955, il part pour la Bolivie et le Pérou, puis s’installe dans le nord-ouest de l’Argentine, à Maimará, dans la province de Jujuy.&lt;/p&gt; &lt;p&gt;Au contact des communautés &lt;a href="https://fr.wikipedia.org/wiki/Quechuas" title=" Wikipedia"&gt;quechuas&lt;/a&gt; et &lt;a href="https://fr.wikipedia.org/wiki/Aymaras" title=" Wikipedia"&gt;aymaras&lt;/a&gt; des Andes, il mène de longues enquêtes de terrain, dont il tire &lt;em&gt;L’Amérique profonde&lt;/em&gt; (1962) et &lt;em&gt;La Pensée indigène et populaire en Amérique&lt;/em&gt; (1970). Il y oppose deux attitudes. Celle de l’Occident, l’« être », qui veut dominer le monde, le transformer et accumuler. Et celle de l’Amérique indienne, l’« être là » ou le simple « se tenir » (en espagnol &lt;em&gt;estar&lt;/em&gt;), qui accepte l’incertitude du monde, ses forces et ses menaces, et cherche à vivre en équilibre avec lui.&lt;/p&gt; &lt;p&gt;Pour Kusch, les classes moyennes des villes, qui se veulent européennes, vivent dans la peur de cette « Amérique profonde » qu’elles refoulent. Penser en Amérique, c’est accepter cette part indienne et populaire au lieu de la mépriser. Son œuvre, longtemps marginale, a nourri la &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_la_lib%C3%A9ration" title=" Wikipedia"&gt;philosophie de la libération&lt;/a&gt; et les pensées décoloniales latino-américaines, et elle est aujourd’hui redécouverte. Il parle même de « phagocytose » : la culture populaire finirait par absorber ce que la modernité importée croit lui imposer. Il meurt en 1979 à Maimará, à cinquante-sept ans.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jos%C3%A9_Enrique_Rod%C3%B3" title=" Wikipedia"&gt;José Enrique RODÓ&lt;/a&gt; est un écrivain et essayiste uruguayen, l’un des grands maîtres à penser de l’Amérique latine au début du XXe siècle. Né à Montevideo, il doit interrompre ses études après la ruine de sa famille, se forme largement seul et devient professeur de littérature à l’université de Montevideo, puis député. Correspondant de &lt;a href="https://fr.wikipedia.org/wiki/Rub%C3%A9n_Dar%C3%ADo" title=" Wikipedia"&gt;Rubén Darío&lt;/a&gt;, il est le principal théoricien du modernisme, le grand mouvement de renouvellement de la littérature hispano-américaine.&lt;/p&gt; &lt;p&gt;Son essai &lt;em&gt;Ariel&lt;/em&gt; (1900), écrit deux ans après la victoire des États-Unis sur l’Espagne à Cuba, prend la forme d’un dernier cours donné par un vieux maître, Prospero, à ses élèves. Empruntant les personnages de &lt;em&gt;La Tempête&lt;/em&gt; de Shakespeare, il oppose Ariel, l’esprit, la beauté, le désintéressement, à Caliban, la matière, l’utilité, les appétits. Il met en garde la jeunesse latino-américaine contre l’utilitarisme et la « nordomanie », la fascination pour le modèle des États-Unis, puissant mais tourné vers le seul profit.&lt;/p&gt; &lt;p&gt;Rodó invite les jeunes à cultiver toutes les facultés de l’esprit, à préserver un temps libre pour la pensée et la beauté, et à construire une démocratie qui élève chacun au lieu de niveler par le bas. Le livre connut un immense succès et inspira tout un courant, l’« arielisme ». Plus tard, des penseurs comme Roberto Fernández Retamar ont renversé le symbole en faisant de Caliban la figure du colonisé. Dans &lt;em&gt;Motifs de Protée&lt;/em&gt; (1909), il médite sur la transformation continuelle de soi. Rodó meurt à Palerme en 1917, au cours d’un voyage en Europe.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/kusch-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/rodo-mini.webp</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">metaphysique ; epistemologie</t>
+          <t xml:space="preserve">esthetique ; ethique</t>
         </is>
       </c>
       <c r="K67" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buen Vivir (cosmovision andine) ; Philosophie de la libération</t>
+          <t xml:space="preserve">Humanisme ; Spiritualisme</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe et anthropologue argentin, penseur de l’« Amérique profonde » et de la pensée indigène et populaire.</t>
+          <t xml:space="preserve">essayiste uruguayen, auteur d’Ariel, maître à penser de la jeunesse latino-américaine.</t>
         </is>
       </c>
       <c r="N67" s="1" t="inlineStr">
@@ -5291,52 +5289,52 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Argentine</t>
+          <t xml:space="preserve">Uruguayenne</t>
         </is>
       </c>
     </row>
     <row r="68" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1">
-        <v>1925</v>
+        <v>1922</v>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1974</t>
+          <t xml:space="preserve">1979</t>
         </is>
       </c>
       <c r="C68" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1925 – 1974</t>
+          <t xml:space="preserve">1922 – 1979</t>
         </is>
       </c>
       <c r="D68" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Augusto SALAZAR BONDY</t>
+          <t xml:space="preserve">Rodolfo KUSCH</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://es.wikipedia.org/wiki/Augusto_Salazar_Bondy" title=" Wikipedia (es)"&gt;Augusto SALAZAR BONDY&lt;/a&gt; est un philosophe et éducateur péruvien, l’une des figures fondatrices de la philosophie latino-américaine de la libération. Né à Lima, frère cadet de l’écrivain Sebastián Salazar Bondy, il étudie à l’université San Marcos, puis au Mexique auprès de José Gaos et de Leopoldo Zea, et à Paris, où il suit les cours de Jean Wahl, Jean Hyppolite et Gaston Bachelard. Professeur d’éthique à San Marcos, il écrit une grande histoire des idées au Pérou contemporain.&lt;/p&gt; &lt;p&gt;En 1968, il publie &lt;em&gt;Existe-t-il une philosophie de notre Amérique ?&lt;/em&gt;, qui provoque un vif débat avec Leopoldo Zea. Sa réponse est dure : jusqu’ici, il n’existe pas de philosophie latino-américaine authentique, mais seulement des imitations des courants européens, adoptés tour à tour sans être vraiment pensés. Ce n’est pas un manque de talent : c’est la conséquence de la domination et du sous-développement, qui produisent une culture dépendante et « aliénée », incapable de se penser elle-même.&lt;/p&gt; &lt;p&gt;Une philosophie authentique ne pourra naître qu’en prenant pour objet cette situation de domination, et en contribuant à la transformer. La philosophie devient ainsi une tâche de libération, comme le développera la &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_la_lib%C3%A9ration" title=" Wikipedia"&gt;philosophie de la libération&lt;/a&gt;. Engagé dans la réforme de l’éducation sous le gouvernement péruvien de la fin des années 1960, il défend une école qui forme des personnes libres et critiques. Il meurt prématurément à Lima en 1974, à quarante-huit ans. Ses idées ont notamment inspiré Enrique Dussel.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://es.wikipedia.org/wiki/Rodolfo_Kusch" title=" Wikipedia (es)"&gt;Rodolfo KUSCH&lt;/a&gt; est un philosophe et anthropologue argentin qui a cherché à fonder une philosophie à partir de la pensée indigène et populaire de l’Amérique. Né à Buenos Aires de parents allemands, il étudie la philosophie à l’université de Buenos Aires, enseigne l’esthétique et écrit aussi pour le théâtre, notamment sur le tango. Persécuté pour ses sympathies péronistes après 1955, il part pour la Bolivie et le Pérou, puis s’installe dans le nord-ouest de l’Argentine, à Maimará, dans la province de Jujuy.&lt;/p&gt; &lt;p&gt;Au contact des communautés &lt;a href="https://fr.wikipedia.org/wiki/Quechuas" title=" Wikipedia"&gt;quechuas&lt;/a&gt; et &lt;a href="https://fr.wikipedia.org/wiki/Aymaras" title=" Wikipedia"&gt;aymaras&lt;/a&gt; des Andes, il mène de longues enquêtes de terrain, dont il tire &lt;em&gt;L’Amérique profonde&lt;/em&gt; (1962) et &lt;em&gt;La Pensée indigène et populaire en Amérique&lt;/em&gt; (1970). Il y oppose deux attitudes. Celle de l’Occident, l’« être », qui veut dominer le monde, le transformer et accumuler. Et celle de l’Amérique indienne, l’« être là » ou le simple « se tenir » (en espagnol &lt;em&gt;estar&lt;/em&gt;), qui accepte l’incertitude du monde, ses forces et ses menaces, et cherche à vivre en équilibre avec lui.&lt;/p&gt; &lt;p&gt;Pour Kusch, les classes moyennes des villes, qui se veulent européennes, vivent dans la peur de cette « Amérique profonde » qu’elles refoulent. Penser en Amérique, c’est accepter cette part indienne et populaire au lieu de la mépriser. Son œuvre, longtemps marginale, a nourri la &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_la_lib%C3%A9ration" title=" Wikipedia"&gt;philosophie de la libération&lt;/a&gt; et les pensées décoloniales latino-américaines, et elle est aujourd’hui redécouverte. Il parle même de « phagocytose » : la culture populaire finirait par absorber ce que la modernité importée croit lui imposer. Il meurt en 1979 à Maimará, à cinquante-sept ans.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/salazarbondy-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/kusch-mini.webp</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">politique ; ethique</t>
+          <t xml:space="preserve">metaphysique ; epistemologie</t>
         </is>
       </c>
       <c r="K68" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiers-mondisme ; Philosophie de la libération</t>
+          <t xml:space="preserve">Buen Vivir (cosmovision andine) ; Philosophie de la libération</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe péruvien, auteur d’Existe-t-il une philosophie de notre Amérique ?, penseur de la domination.</t>
+          <t xml:space="preserve">philosophe et anthropologue argentin, penseur de l’« Amérique profonde » et de la pensée indigène et populaire.</t>
         </is>
       </c>
       <c r="N68" s="1" t="inlineStr">
@@ -5349,52 +5347,52 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Péruvienne</t>
+          <t xml:space="preserve">Argentine</t>
         </is>
       </c>
     </row>
     <row r="69" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1">
-        <v>1839</v>
+        <v>1925</v>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1903</t>
+          <t xml:space="preserve">1974</t>
         </is>
       </c>
       <c r="C69" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1839 – 1903</t>
+          <t xml:space="preserve">1925 – 1974</t>
         </is>
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eugenio María de HOSTOS</t>
+          <t xml:space="preserve">Augusto SALAZAR BONDY</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Eugenio_Mar%C3%ADa_de_Hostos" title=" Wikipedia (en)"&gt;Eugenio María de HOSTOS&lt;/a&gt; est un philosophe, éducateur, sociologue et écrivain de &lt;a href="https://fr.wikipedia.org/wiki/Porto_Rico" title=" Wikipedia"&gt;Porto Rico&lt;/a&gt;, surnommé « le Grand Citoyen des Amériques ». Né à Mayagüez dans une famille aisée, il fait ses études en Espagne, où il étudie le droit et la philosophie à Madrid et publie en 1863 un roman, &lt;em&gt;Le Pèlerinage de Bayoán&lt;/em&gt;, qui évoque déjà le destin des Antilles. Déçu que la République espagnole refuse l’autonomie de Porto Rico, il quitte l’Espagne en 1869 pour se consacrer à l’indépendance des colonies antillaises.&lt;/p&gt; &lt;p&gt;Il rêve d’une Confédération des Antilles, réunissant Porto Rico, Cuba et la République dominicaine, et parcourt pour la défendre les États-Unis, le Pérou, le Chili, l’Argentine, le Brésil et le Venezuela. Partout, il fonde ou réforme des écoles. En République dominicaine, il crée en 1880 la première école normale, qui forme des instituteurs à une pédagogie scientifique et laïque. Au Chili, il plaide pour que les femmes aient accès à l’enseignement supérieur et aux professions savantes.&lt;/p&gt; &lt;p&gt;Sa &lt;em&gt;Morale sociale&lt;/em&gt; (1888), inspirée du &lt;a href="https://fr.wikipedia.org/wiki/Positivisme" title=" Wikipedia"&gt;positivisme&lt;/a&gt;, fonde les devoirs de l’individu non sur la religion, mais sur la raison et sur les liens qui l’unissent à la famille, à la société et à l’humanité ; l’éducation doit former des consciences libres et responsables. Après la guerre de 1898, qui fait passer Porto Rico sous domination américaine, il milite pour que l’île puisse décider elle-même de son avenir. Il laisse aussi un traité de sociologie, l’un des premiers d’Amérique latine. Il meurt en exil à Saint-Domingue en 1903.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://es.wikipedia.org/wiki/Augusto_Salazar_Bondy" title=" Wikipedia (es)"&gt;Augusto SALAZAR BONDY&lt;/a&gt; est un philosophe et éducateur péruvien, l’une des figures fondatrices de la philosophie latino-américaine de la libération. Né à Lima, frère cadet de l’écrivain Sebastián Salazar Bondy, il étudie à l’université San Marcos, puis au Mexique auprès de José Gaos et de Leopoldo Zea, et à Paris, où il suit les cours de Jean Wahl, Jean Hyppolite et Gaston Bachelard. Professeur d’éthique à San Marcos, il écrit une grande histoire des idées au Pérou contemporain.&lt;/p&gt; &lt;p&gt;En 1968, il publie &lt;em&gt;Existe-t-il une philosophie de notre Amérique ?&lt;/em&gt;, qui provoque un vif débat avec Leopoldo Zea. Sa réponse est dure : jusqu’ici, il n’existe pas de philosophie latino-américaine authentique, mais seulement des imitations des courants européens, adoptés tour à tour sans être vraiment pensés. Ce n’est pas un manque de talent : c’est la conséquence de la domination et du sous-développement, qui produisent une culture dépendante et « aliénée », incapable de se penser elle-même.&lt;/p&gt; &lt;p&gt;Une philosophie authentique ne pourra naître qu’en prenant pour objet cette situation de domination, et en contribuant à la transformer. La philosophie devient ainsi une tâche de libération, comme le développera la &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_la_lib%C3%A9ration" title=" Wikipedia"&gt;philosophie de la libération&lt;/a&gt;. Engagé dans la réforme de l’éducation sous le gouvernement péruvien de la fin des années 1960, il défend une école qui forme des personnes libres et critiques. Il meurt prématurément à Lima en 1974, à quarante-huit ans. Ses idées ont notamment inspiré Enrique Dussel.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/hostos-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/salazarbondy-mini.webp</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ethique ; politique</t>
+          <t xml:space="preserve">politique ; ethique</t>
         </is>
       </c>
       <c r="K69" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Positivisme</t>
+          <t xml:space="preserve">Tiers-mondisme ; Philosophie de la libération</t>
         </is>
       </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">éducateur et penseur portoricain, apôtre d’une confédération des Antilles et d’une morale sociale laïque.</t>
+          <t xml:space="preserve">philosophe péruvien, auteur d’Existe-t-il une philosophie de notre Amérique ?, penseur de la domination.</t>
         </is>
       </c>
       <c r="N69" s="1" t="inlineStr">
@@ -5407,52 +5405,52 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portoricaine</t>
+          <t xml:space="preserve">Péruvienne</t>
         </is>
       </c>
     </row>
     <row r="70" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1">
-        <v>1925</v>
+        <v>1839</v>
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2008</t>
+          <t xml:space="preserve">1903</t>
         </is>
       </c>
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1925 – 2008</t>
+          <t xml:space="preserve">1839 – 1903</t>
         </is>
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Orlando FALS BORDA</t>
+          <t xml:space="preserve">Eugenio María de HOSTOS</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Orlando_Fals_Borda" title=" Wikipedia (en)"&gt;Orlando FALS BORDA&lt;/a&gt; est un sociologue colombien, l’un des grands penseurs latino-américains des sciences sociales et le fondateur de la « recherche-action participative ». Né à Barranquilla, sur la côte caraïbe, formé aux États-Unis, il fonde en 1959 à l’Université nationale de Colombie, avec le prêtre Camilo Torres, l’une des premières facultés de sociologie d’Amérique latine. Son livre &lt;em&gt;La Violence en Colombie&lt;/em&gt; (1962), écrit avec Germán Guzmán et Eduardo Umaña, étudie pour la première fois la guerre civile qui ravage les campagnes.&lt;/p&gt; &lt;p&gt;Déçu par une sociologie qui observe les pauvres de l’extérieur sans rien changer à leur sort, il quitte l’université dans les années 1970 pour travailler avec les paysans et les communautés de la côte caraïbe. Il y développe la &lt;a href="https://fr.wikipedia.org/wiki/Recherche-action" title=" Wikipedia"&gt;recherche-action&lt;/a&gt; participative : le chercheur ne doit pas monopoliser le savoir ni imposer sa technique, mais travailler avec les communautés comme avec des partenaires et des co-chercheurs, recueillir leurs savoirs, leur mémoire et leurs récits, et partager les résultats sous une forme que tous peuvent comprendre.&lt;/p&gt; &lt;p&gt;La science n’est pas, selon lui, une affaire d’experts neutres : elle doit servir la transformation de la société et la libération des opprimés. Il parle d’une « subversion positive » qui conteste l’ordre injuste pour en construire un meilleur. Ses idées se sont répandues dans le monde entier, en éducation, en santé et en développement. Il participe aussi à l’Assemblée constituante qui rédige la Constitution colombienne de 1991. Il meurt à Bogotá en 2008.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Eugenio_Mar%C3%ADa_de_Hostos" title=" Wikipedia (en)"&gt;Eugenio María de HOSTOS&lt;/a&gt; est un philosophe, éducateur, sociologue et écrivain de &lt;a href="https://fr.wikipedia.org/wiki/Porto_Rico" title=" Wikipedia"&gt;Porto Rico&lt;/a&gt;, surnommé « le Grand Citoyen des Amériques ». Né à Mayagüez dans une famille aisée, il fait ses études en Espagne, où il étudie le droit et la philosophie à Madrid et publie en 1863 un roman, &lt;em&gt;Le Pèlerinage de Bayoán&lt;/em&gt;, qui évoque déjà le destin des Antilles. Déçu que la République espagnole refuse l’autonomie de Porto Rico, il quitte l’Espagne en 1869 pour se consacrer à l’indépendance des colonies antillaises.&lt;/p&gt; &lt;p&gt;Il rêve d’une Confédération des Antilles, réunissant Porto Rico, Cuba et la République dominicaine, et parcourt pour la défendre les États-Unis, le Pérou, le Chili, l’Argentine, le Brésil et le Venezuela. Partout, il fonde ou réforme des écoles. En République dominicaine, il crée en 1880 la première école normale, qui forme des instituteurs à une pédagogie scientifique et laïque. Au Chili, il plaide pour que les femmes aient accès à l’enseignement supérieur et aux professions savantes.&lt;/p&gt; &lt;p&gt;Sa &lt;em&gt;Morale sociale&lt;/em&gt; (1888), inspirée du &lt;a href="https://fr.wikipedia.org/wiki/Positivisme" title=" Wikipedia"&gt;positivisme&lt;/a&gt;, fonde les devoirs de l’individu non sur la religion, mais sur la raison et sur les liens qui l’unissent à la famille, à la société et à l’humanité ; l’éducation doit former des consciences libres et responsables. Après la guerre de 1898, qui fait passer Porto Rico sous domination américaine, il milite pour que l’île puisse décider elle-même de son avenir. Il laisse aussi un traité de sociologie, l’un des premiers d’Amérique latine. Il meurt en exil à Saint-Domingue en 1903.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/falsborda-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/hostos-mini.webp</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">epistemologie ; politique</t>
+          <t xml:space="preserve">ethique ; politique</t>
         </is>
       </c>
       <c r="K70" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiers-mondisme</t>
+          <t xml:space="preserve">Positivisme</t>
         </is>
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sociologue colombien, fondateur de la recherche-action participative, penseur d’un savoir construit avec le peuple.</t>
+          <t xml:space="preserve">éducateur et penseur portoricain, apôtre d’une confédération des Antilles et d’une morale sociale laïque.</t>
         </is>
       </c>
       <c r="N70" s="1" t="inlineStr">
@@ -5465,62 +5463,57 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Colombienne</t>
+          <t xml:space="preserve">Portoricaine</t>
         </is>
       </c>
     </row>
     <row r="71" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1">
-        <v>1928</v>
+        <v>1925</v>
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2021</t>
+          <t xml:space="preserve">2008</t>
         </is>
       </c>
       <c r="C71" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1928 – 2021</t>
+          <t xml:space="preserve">1925 – 2008</t>
         </is>
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Humberto MATURANA</t>
+          <t xml:space="preserve">Orlando FALS BORDA</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Humberto_Maturana" title=" Wikipedia"&gt;Humberto MATURANA&lt;/a&gt; est un biologiste et philosophe chilien, l’un des penseurs les plus originaux de la biologie de la connaissance. Né à Santiago, il étudie la médecine et la biologie au Chili, puis en Angleterre et à Harvard. Au Massachusetts Institute of Technology, il participe en 1959 à une étude devenue célèbre sur ce que l’œil de la grenouille transmet à son cerveau, qui montre que la perception n’est pas une simple copie du monde extérieur. Il fonde ensuite à l’université du Chili un laboratoire d’« épistémologie expérimentale ».&lt;/p&gt; &lt;p&gt;Avec son élève Francisco Varela, il propose au début des années 1970 le concept d’&lt;a href="https://fr.wikipedia.org/wiki/Autopo%C3%AF%C3%A8se" title=" Wikipedia"&gt;autopoïèse&lt;/a&gt;, du grec « se produire soi-même » : un être vivant est un système qui produit et renouvelle sans cesse ses propres composants, et maintient ainsi sa propre organisation. La cellule en est le modèle. Le vivant n’est donc pas défini par ce qu’il contient, mais par cette manière de s’entretenir lui-même, en échange constant avec son milieu.&lt;/p&gt; &lt;p&gt;Il en tire une théorie de la connaissance : « Tout ce qui est dit est dit par un observateur. » Connaître n’est pas refléter un monde tout fait, mais une activité du vivant, qui fait émerger un monde à travers son action. Dans &lt;em&gt;L’Arbre de la connaissance&lt;/em&gt; (1984), écrit avec Varela, il montre aussi que le langage et la société naissent de la coordination entre les êtres, et que l’amour, l’acceptation de l’autre, est le fondement biologique de la vie sociale. Ses idées ont nourri le &lt;a href="https://fr.wikipedia.org/wiki/Constructivisme_%28%C3%A9pist%C3%A9mologie%29" title=" Wikipedia"&gt;constructivisme&lt;/a&gt;, la thérapie familiale et la théorie des systèmes sociaux de &lt;a href="https://fr.wikipedia.org/wiki/Niklas_Luhmann" title=" Wikipedia"&gt;Niklas Luhmann&lt;/a&gt;. Il meurt à Santiago en 2021.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Orlando_Fals_Borda" title=" Wikipedia (en)"&gt;Orlando FALS BORDA&lt;/a&gt; est un sociologue colombien, l’un des grands penseurs latino-américains des sciences sociales et le fondateur de la « recherche-action participative ». Né à Barranquilla, sur la côte caraïbe, formé aux États-Unis, il fonde en 1959 à l’Université nationale de Colombie, avec le prêtre Camilo Torres, l’une des premières facultés de sociologie d’Amérique latine. Son livre &lt;em&gt;La Violence en Colombie&lt;/em&gt; (1962), écrit avec Germán Guzmán et Eduardo Umaña, étudie pour la première fois la guerre civile qui ravage les campagnes.&lt;/p&gt; &lt;p&gt;Déçu par une sociologie qui observe les pauvres de l’extérieur sans rien changer à leur sort, il quitte l’université dans les années 1970 pour travailler avec les paysans et les communautés de la côte caraïbe. Il y développe la &lt;a href="https://fr.wikipedia.org/wiki/Recherche-action" title=" Wikipedia"&gt;recherche-action&lt;/a&gt; participative : le chercheur ne doit pas monopoliser le savoir ni imposer sa technique, mais travailler avec les communautés comme avec des partenaires et des co-chercheurs, recueillir leurs savoirs, leur mémoire et leurs récits, et partager les résultats sous une forme que tous peuvent comprendre.&lt;/p&gt; &lt;p&gt;La science n’est pas, selon lui, une affaire d’experts neutres : elle doit servir la transformation de la société et la libération des opprimés. Il parle d’une « subversion positive » qui conteste l’ordre injuste pour en construire un meilleur. Ses idées se sont répandues dans le monde entier, en éducation, en santé et en développement. Il participe aussi à l’Assemblée constituante qui rédige la Constitution colombienne de 1991. Il meurt à Bogotá en 2008.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/maturana-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/falsborda-mini.webp</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">epistemologie ; metaphysique</t>
+          <t xml:space="preserve">epistemologie ; politique</t>
         </is>
       </c>
       <c r="K71" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Constructivisme</t>
+          <t xml:space="preserve">Tiers-mondisme</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">biologiste et philosophe chilien, inventeur avec Varela de l’autopoïèse, penseur de la connaissance comme fait biologique.</t>
-        </is>
-      </c>
-      <c r="M71" t="inlineStr">
+          <t xml:space="preserve">sociologue colombien, fondateur de la recherche-action participative, penseur d’un savoir construit avec le peuple.</t>
+        </is>
+      </c>
+      <c r="N71" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">sud</t>
-        </is>
-      </c>
-      <c r="N71" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
         </is>
       </c>
       <c r="O71" s="1">
@@ -5528,37 +5521,37 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chilienne</t>
+          <t xml:space="preserve">Colombienne</t>
         </is>
       </c>
     </row>
     <row r="72" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1">
-        <v>1946</v>
+        <v>1928</v>
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2001</t>
+          <t xml:space="preserve">2021</t>
         </is>
       </c>
       <c r="C72" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1946 – 2001</t>
+          <t xml:space="preserve">1928 – 2021</t>
         </is>
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Francisco VARELA</t>
+          <t xml:space="preserve">Humberto MATURANA</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Francisco_Varela" title=" Wikipedia"&gt;Francisco VARELA&lt;/a&gt; est un biologiste, neuroscientifique et philosophe chilien, l’un des fondateurs des sciences cognitives « incarnées ». Né à Talcahuano, élève d’Humberto Maturana, il soutient une thèse de biologie à Harvard, puis invente avec son maître le concept d’&lt;a href="https://fr.wikipedia.org/wiki/Autopo%C3%AF%C3%A8se" title=" Wikipedia"&gt;autopoïèse&lt;/a&gt;, qui définit le vivant par sa capacité à se produire lui-même. Après le coup d’État de Pinochet en 1973, il doit s’exiler aux États-Unis. Il s’installe en France en 1986 et dirige jusqu’à sa mort une équipe de recherche au CNRS, à Paris.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;L’Inscription corporelle de l’esprit&lt;/em&gt; (1991), écrit avec Evan Thompson et Eleanor Rosch, il critique l’idée que l’esprit serait un ordinateur qui traite des représentations d’un monde extérieur déjà donné. Il propose à la place l’« &lt;a href="https://fr.wikipedia.org/wiki/%C3%89naction" title=" Wikipedia"&gt;énaction&lt;/a&gt; » : la cognition est une action incarnée, par laquelle un être vivant fait émerger son monde à travers son corps, ses sens et ses gestes. Il fonde aussi la « neurophénoménologie », qui veut unir les mesures du cerveau et la description rigoureuse de l’expérience vécue, à la manière de Husserl et de Merleau-Ponty.&lt;/p&gt; &lt;p&gt;Pratiquant du bouddhisme tibétain depuis les années 1970, il voit dans la méditation une méthode précise pour explorer l’expérience. En 1987, il cofonde le &lt;a href="https://fr.wikipedia.org/wiki/Mind_and_Life_Institute" title=" Wikipedia"&gt;Mind and Life Institute&lt;/a&gt;, qui organise des rencontres entre scientifiques et le dalaï-lama. Il est l’un des inspirateurs de l’idée d’un esprit « incarné », aujourd’hui centrale en &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_l%27esprit" title=" Wikipedia"&gt;philosophie de l’esprit&lt;/a&gt;. Il meurt à Paris en 2001, à cinquante-quatre ans, d’une maladie du foie.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Humberto_Maturana" title=" Wikipedia"&gt;Humberto MATURANA&lt;/a&gt; est un biologiste et philosophe chilien, l’un des penseurs les plus originaux de la biologie de la connaissance. Né à Santiago, il étudie la médecine et la biologie au Chili, puis en Angleterre et à Harvard. Au Massachusetts Institute of Technology, il participe en 1959 à une étude devenue célèbre sur ce que l’œil de la grenouille transmet à son cerveau, qui montre que la perception n’est pas une simple copie du monde extérieur. Il fonde ensuite à l’université du Chili un laboratoire d’« épistémologie expérimentale ».&lt;/p&gt; &lt;p&gt;Avec son élève Francisco Varela, il propose au début des années 1970 le concept d’&lt;a href="https://fr.wikipedia.org/wiki/Autopo%C3%AF%C3%A8se" title=" Wikipedia"&gt;autopoïèse&lt;/a&gt;, du grec « se produire soi-même » : un être vivant est un système qui produit et renouvelle sans cesse ses propres composants, et maintient ainsi sa propre organisation. La cellule en est le modèle. Le vivant n’est donc pas défini par ce qu’il contient, mais par cette manière de s’entretenir lui-même, en échange constant avec son milieu.&lt;/p&gt; &lt;p&gt;Il en tire une théorie de la connaissance : « Tout ce qui est dit est dit par un observateur. » Connaître n’est pas refléter un monde tout fait, mais une activité du vivant, qui fait émerger un monde à travers son action. Dans &lt;em&gt;L’Arbre de la connaissance&lt;/em&gt; (1984), écrit avec Varela, il montre aussi que le langage et la société naissent de la coordination entre les êtres, et que l’amour, l’acceptation de l’autre, est le fondement biologique de la vie sociale. Ses idées ont nourri le &lt;a href="https://fr.wikipedia.org/wiki/Constructivisme_%28%C3%A9pist%C3%A9mologie%29" title=" Wikipedia"&gt;constructivisme&lt;/a&gt;, la thérapie familiale et la théorie des systèmes sociaux de &lt;a href="https://fr.wikipedia.org/wiki/Niklas_Luhmann" title=" Wikipedia"&gt;Niklas Luhmann&lt;/a&gt;. Il meurt à Santiago en 2021.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/varela-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/maturana-mini.webp</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -5568,12 +5561,12 @@
       </c>
       <c r="K72" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Constructivisme ; Phénoménologie</t>
+          <t xml:space="preserve">Constructivisme</t>
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">neurobiologiste et philosophe chilien, penseur de l’énaction et du dialogue entre sciences cognitives et bouddhisme.</t>
+          <t xml:space="preserve">biologiste et philosophe chilien, inventeur avec Varela de l’autopoïèse, penseur de la connaissance comme fait biologique.</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -5597,46 +5590,46 @@
     </row>
     <row r="73" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1">
-        <v>1868</v>
+        <v>1946</v>
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1963</t>
+          <t xml:space="preserve">2001</t>
         </is>
       </c>
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1868 – 1963</t>
+          <t xml:space="preserve">1946 – 2001</t>
         </is>
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">W. E. B. DU BOIS</t>
+          <t xml:space="preserve">Francisco VARELA</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/W._E._B._Du_Bois" title=" Wikipedia"&gt;W. E. B. DU BOIS&lt;/a&gt; (William Edward Burghardt Du Bois) est un sociologue, historien et militant africain-américain, l’un des plus grands penseurs américains du XXe siècle. Né en 1868 dans le Massachusetts, il étudie à Fisk, à Berlin, puis à Harvard, où il devient en 1895 le premier Africain-Américain à obtenir un doctorat. Son étude &lt;em&gt;The Philadelphia Negro&lt;/em&gt; (1899) est l’une des premières grandes enquêtes de sociologie empirique aux États-Unis.&lt;/p&gt; &lt;p&gt;Dans &lt;a href="https://fr.wikipedia.org/wiki/Les_%C3%82mes_du_peuple_noir" title=" Wikipedia"&gt;&lt;em&gt;Les Âmes du peuple noir&lt;/em&gt;&lt;/a&gt; (1903), il affirme que « le problème du XXe siècle est le problème de la ligne de couleur ». Il y décrit la « double conscience » des Noirs américains : le sentiment de se voir toujours à travers les yeux d’un monde qui les méprise, d’être à la fois américain et noir, « deux âmes, deux pensées, deux combats inconciliables dans un seul corps sombre ». Dans &lt;em&gt;Black Reconstruction&lt;/em&gt; (1935), il réhabilitera le rôle des anciens esclaves dans l’histoire américaine d’après la guerre de Sécession. Il y critique aussi Booker T. Washington, qui conseillait aux Noirs d’accepter la ségrégation en échange du progrès économique.&lt;/p&gt; &lt;p&gt;En 1909, il est l’un des fondateurs de la &lt;a href="https://fr.wikipedia.org/wiki/National_Association_for_the_Advancement_of_Colored_People" title=" Wikipedia"&gt;NAACP&lt;/a&gt;, la grande organisation de défense des droits civiques, dont il dirige la revue &lt;em&gt;The Crisis&lt;/em&gt;. Il organise plusieurs congrès panafricains et devient le « père du &lt;a href="https://fr.wikipedia.org/wiki/Panafricanisme" title=" Wikipedia"&gt;panafricanisme&lt;/a&gt; ». Proche du socialisme, persécuté pendant le maccarthysme, il s’installe à la fin de sa vie au &lt;a href="https://fr.wikipedia.org/wiki/Ghana" title=" Wikipedia"&gt;Ghana&lt;/a&gt;, à l’invitation de Kwame Nkrumah, et y meurt en 1963, à la veille de la marche sur Washington de Martin Luther King.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Francisco_Varela" title=" Wikipedia"&gt;Francisco VARELA&lt;/a&gt; est un biologiste, neuroscientifique et philosophe chilien, l’un des fondateurs des sciences cognitives « incarnées ». Né à Talcahuano, élève d’Humberto Maturana, il soutient une thèse de biologie à Harvard, puis invente avec son maître le concept d’&lt;a href="https://fr.wikipedia.org/wiki/Autopo%C3%AF%C3%A8se" title=" Wikipedia"&gt;autopoïèse&lt;/a&gt;, qui définit le vivant par sa capacité à se produire lui-même. Après le coup d’État de Pinochet en 1973, il doit s’exiler aux États-Unis. Il s’installe en France en 1986 et dirige jusqu’à sa mort une équipe de recherche au CNRS, à Paris.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;L’Inscription corporelle de l’esprit&lt;/em&gt; (1991), écrit avec Evan Thompson et Eleanor Rosch, il critique l’idée que l’esprit serait un ordinateur qui traite des représentations d’un monde extérieur déjà donné. Il propose à la place l’« &lt;a href="https://fr.wikipedia.org/wiki/%C3%89naction" title=" Wikipedia"&gt;énaction&lt;/a&gt; » : la cognition est une action incarnée, par laquelle un être vivant fait émerger son monde à travers son corps, ses sens et ses gestes. Il fonde aussi la « neurophénoménologie », qui veut unir les mesures du cerveau et la description rigoureuse de l’expérience vécue, à la manière de Husserl et de Merleau-Ponty.&lt;/p&gt; &lt;p&gt;Pratiquant du bouddhisme tibétain depuis les années 1970, il voit dans la méditation une méthode précise pour explorer l’expérience. En 1987, il cofonde le &lt;a href="https://fr.wikipedia.org/wiki/Mind_and_Life_Institute" title=" Wikipedia"&gt;Mind and Life Institute&lt;/a&gt;, qui organise des rencontres entre scientifiques et le dalaï-lama. Il est l’un des inspirateurs de l’idée d’un esprit « incarné », aujourd’hui centrale en &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_l%27esprit" title=" Wikipedia"&gt;philosophie de l’esprit&lt;/a&gt;. Il meurt à Paris en 2001, à cinquante-quatre ans, d’une maladie du foie.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/dubois-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/varela-mini.webp</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">politique ; ethique</t>
+          <t xml:space="preserve">epistemologie ; metaphysique</t>
         </is>
       </c>
       <c r="K73" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pan-africanisme</t>
+          <t xml:space="preserve">Constructivisme ; Phénoménologie</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sociologue et militant africain-américain, penseur de la « double conscience » et père du panafricanisme.</t>
+          <t xml:space="preserve">neurobiologiste et philosophe chilien, penseur de l’énaction et du dialogue entre sciences cognitives et bouddhisme.</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -5650,69 +5643,74 @@
         </is>
       </c>
       <c r="O73" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Américaine</t>
+          <t xml:space="preserve">Chilienne</t>
         </is>
       </c>
     </row>
     <row r="74" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="1">
-        <v>1928</v>
+        <v>1868</v>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024</t>
+          <t xml:space="preserve">1963</t>
         </is>
       </c>
       <c r="C74" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1928 – 2024</t>
+          <t xml:space="preserve">1868 – 1963</t>
         </is>
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gustavo GUTIÉRREZ</t>
+          <t xml:space="preserve">W. E. B. DU BOIS</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Gustavo_Guti%C3%A9rrez_Merino" title=" Wikipedia"&gt;Gustavo GUTIÉRREZ&lt;/a&gt; est un prêtre et théologien péruvien, considéré comme le père de la &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9ologie_de_la_lib%C3%A9ration" title=" Wikipedia"&gt;théologie de la libération&lt;/a&gt;. Né à Lima en 1928 dans un milieu modeste, il souffre adolescent d’une ostéomyélite qui le cloue longtemps au lit ; il lit alors beaucoup et commence des études de médecine pour devenir psychiatre. À vingt-quatre ans, il choisit la prêtrise et part étudier la philosophie et la psychologie à Louvain, puis la théologie à Lyon.&lt;/p&gt; &lt;p&gt;Ordonné prêtre en 1959, il devient vicaire dans un quartier pauvre de Lima, tout en enseignant à l’université catholique, et repense toute sa théologie au contact de ce peuple. En 1971, il publie &lt;em&gt;Théologie de la libération&lt;/em&gt;, traduit dans une vingtaine de langues. La pauvreté, écrit-il, n’est pas une fatalité mais le fruit d’injustices, et elle est contraire à la volonté de Dieu. La théologie est une « réflexion critique sur la pratique à la lumière de la Parole » : elle vient en second, après l’engagement aux côtés des pauvres. Le salut ne se joue pas seulement dans l’au-delà ; il touche toute l’existence, et la libération sociale et politique en fait partie, sans s’y réduire. Dans &lt;em&gt;Boire à son propre puits&lt;/em&gt; (1983), il montre que cet engagement est aussi une spiritualité, une manière de suivre le Christ.&lt;/p&gt; &lt;p&gt;Ses positions lui valent la méfiance de Rome dans les années 1980, sans condamnation. Entré chez les Dominicains en 1998, il enseigne dans de nombreuses universités d’Europe et des États-Unis. Le pape François le reçoit en 2013, signe de la réhabilitation de son œuvre, et l’« option préférentielle pour les pauvres » est devenue un principe de l’enseignement de l’Église. Il meurt à Lima en 2024, à quatre-vingt-seize ans.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/W._E._B._Du_Bois" title=" Wikipedia"&gt;W. E. B. DU BOIS&lt;/a&gt; (William Edward Burghardt Du Bois) est un sociologue, historien et militant africain-américain, l’un des plus grands penseurs américains du XXe siècle. Né en 1868 dans le Massachusetts, il étudie à Fisk, à Berlin, puis à Harvard, où il devient en 1895 le premier Africain-Américain à obtenir un doctorat. Son étude &lt;em&gt;The Philadelphia Negro&lt;/em&gt; (1899) est l’une des premières grandes enquêtes de sociologie empirique aux États-Unis.&lt;/p&gt; &lt;p&gt;Dans &lt;a href="https://fr.wikipedia.org/wiki/Les_%C3%82mes_du_peuple_noir" title=" Wikipedia"&gt;&lt;em&gt;Les Âmes du peuple noir&lt;/em&gt;&lt;/a&gt; (1903), il affirme que « le problème du XXe siècle est le problème de la ligne de couleur ». Il y décrit la « double conscience » des Noirs américains : le sentiment de se voir toujours à travers les yeux d’un monde qui les méprise, d’être à la fois américain et noir, « deux âmes, deux pensées, deux combats inconciliables dans un seul corps sombre ». Dans &lt;em&gt;Black Reconstruction&lt;/em&gt; (1935), il réhabilitera le rôle des anciens esclaves dans l’histoire américaine d’après la guerre de Sécession. Il y critique aussi Booker T. Washington, qui conseillait aux Noirs d’accepter la ségrégation en échange du progrès économique.&lt;/p&gt; &lt;p&gt;En 1909, il est l’un des fondateurs de la &lt;a href="https://fr.wikipedia.org/wiki/National_Association_for_the_Advancement_of_Colored_People" title=" Wikipedia"&gt;NAACP&lt;/a&gt;, la grande organisation de défense des droits civiques, dont il dirige la revue &lt;em&gt;The Crisis&lt;/em&gt;. Il organise plusieurs congrès panafricains et devient le « père du &lt;a href="https://fr.wikipedia.org/wiki/Panafricanisme" title=" Wikipedia"&gt;panafricanisme&lt;/a&gt; ». Proche du socialisme, persécuté pendant le maccarthysme, il s’installe à la fin de sa vie au &lt;a href="https://fr.wikipedia.org/wiki/Ghana" title=" Wikipedia"&gt;Ghana&lt;/a&gt;, à l’invitation de Kwame Nkrumah, et y meurt en 1963, à la veille de la marche sur Washington de Martin Luther King.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/ggutierrez-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/dubois-mini.webp</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">spiritualite ; politique</t>
+          <t xml:space="preserve">politique ; ethique</t>
         </is>
       </c>
       <c r="K74" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Théologie de la libération</t>
+          <t xml:space="preserve">Pan-africanisme</t>
         </is>
       </c>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">prêtre et théologien péruvien, père de la théologie de la libération et de l’« option préférentielle pour les pauvres ».</t>
+          <t xml:space="preserve">sociologue et militant africain-américain, penseur de la « double conscience » et père du panafricanisme.</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
         </is>
       </c>
       <c r="N74" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">sud</t>
+          <t xml:space="preserve">occident</t>
         </is>
       </c>
       <c r="O74" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Péruvienne</t>
+          <t xml:space="preserve">Américaine</t>
         </is>
       </c>
     </row>
@@ -5722,42 +5720,42 @@
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2018</t>
+          <t xml:space="preserve">2024</t>
         </is>
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1928 – 2018</t>
+          <t xml:space="preserve">1928 – 2024</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aníbal QUIJANO</t>
+          <t xml:space="preserve">Gustavo GUTIÉRREZ</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/An%C3%ADbal_Quijano" title=" Wikipedia"&gt;Aníbal QUIJANO&lt;/a&gt; est un sociologue péruvien, l’un des grands penseurs latino-américains du XXe siècle et le fondateur de la pensée décoloniale. Né en 1928 à Yanama, dans les Andes péruviennes, il étudie à l’université de San Marcos, à Lima, où il enseigne ensuite la sociologie. Dans les années 1960 et 1970, il participe aux travaux de la &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9orie_de_la_d%C3%A9pendance" title=" Wikipedia"&gt;théorie de la dépendance&lt;/a&gt;, qui explique le sous-développement de l’Amérique latine par sa place subordonnée dans l’économie mondiale, et étudie la condition des populations indiennes et métisses des villes.&lt;/p&gt; &lt;p&gt;En 1992, pour le cinquième centenaire de l’arrivée de Christophe Colomb, il publie l’article « Colonialité et modernité/rationalité », qui forge la notion de « colonialité du pouvoir ». La conquête de l’Amérique a donné naissance à la fois au capitalisme mondial et à une idée nouvelle, celle de « race », qui a permis de classer les peuples en supérieurs et inférieurs et de distribuer entre eux le travail : le salariat pour les Européens, le servage pour les Indiens, l’esclavage pour les Africains. Cette classification a survécu à l’indépendance des colonies : elle structure encore les rapports sociaux, le savoir et la manière dont chacun se perçoit. Quijano critique aussi l’« eurocentrisme », qui fait de l’histoire européenne le modèle de l’histoire universelle.&lt;/p&gt; &lt;p&gt;Professeur à l’université de Binghamton, aux États-Unis, il anime le &lt;a href="https://fr.wikipedia.org/wiki/Groupe_modernit%C3%A9/colonialit%C3%A9" title=" Wikipedia"&gt;groupe « modernité/colonialité »&lt;/a&gt; avec Walter Mignolo et Enrique Dussel. La philosophe argentine &lt;a href="https://fr.wikipedia.org/wiki/Mar%C3%ADa_Lugones" title=" Wikipedia"&gt;María Lugones&lt;/a&gt; a prolongé son concept dans celui de « colonialité du genre ». Il meurt à Lima en 2018.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Gustavo_Guti%C3%A9rrez_Merino" title=" Wikipedia"&gt;Gustavo GUTIÉRREZ&lt;/a&gt; est un prêtre et théologien péruvien, considéré comme le père de la &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9ologie_de_la_lib%C3%A9ration" title=" Wikipedia"&gt;théologie de la libération&lt;/a&gt;. Né à Lima en 1928 dans un milieu modeste, il souffre adolescent d’une ostéomyélite qui le cloue longtemps au lit ; il lit alors beaucoup et commence des études de médecine pour devenir psychiatre. À vingt-quatre ans, il choisit la prêtrise et part étudier la philosophie et la psychologie à Louvain, puis la théologie à Lyon.&lt;/p&gt; &lt;p&gt;Ordonné prêtre en 1959, il devient vicaire dans un quartier pauvre de Lima, tout en enseignant à l’université catholique, et repense toute sa théologie au contact de ce peuple. En 1971, il publie &lt;em&gt;Théologie de la libération&lt;/em&gt;, traduit dans une vingtaine de langues. La pauvreté, écrit-il, n’est pas une fatalité mais le fruit d’injustices, et elle est contraire à la volonté de Dieu. La théologie est une « réflexion critique sur la pratique à la lumière de la Parole » : elle vient en second, après l’engagement aux côtés des pauvres. Le salut ne se joue pas seulement dans l’au-delà ; il touche toute l’existence, et la libération sociale et politique en fait partie, sans s’y réduire. Dans &lt;em&gt;Boire à son propre puits&lt;/em&gt; (1983), il montre que cet engagement est aussi une spiritualité, une manière de suivre le Christ.&lt;/p&gt; &lt;p&gt;Ses positions lui valent la méfiance de Rome dans les années 1980, sans condamnation. Entré chez les Dominicains en 1998, il enseigne dans de nombreuses universités d’Europe et des États-Unis. Le pape François le reçoit en 2013, signe de la réhabilitation de son œuvre, et l’« option préférentielle pour les pauvres » est devenue un principe de l’enseignement de l’Église. Il meurt à Lima en 2024, à quatre-vingt-seize ans.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/quijano-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/ggutierrez-mini.webp</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">politique ; epistemologie</t>
+          <t xml:space="preserve">spiritualite ; politique</t>
         </is>
       </c>
       <c r="K75" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pensée décoloniale</t>
+          <t xml:space="preserve">Théologie de la libération</t>
         </is>
       </c>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sociologue péruvien, inventeur de la « colonialité du pouvoir » et fondateur de la pensée décoloniale.</t>
+          <t xml:space="preserve">prêtre et théologien péruvien, père de la théologie de la libération et de l’« option préférentielle pour les pauvres ».</t>
         </is>
       </c>
       <c r="N75" s="1" t="inlineStr">
@@ -5765,7 +5763,9 @@
           <t xml:space="preserve">sud</t>
         </is>
       </c>
-      <c r="O75" s="1"/>
+      <c r="O75" s="1">
+        <v>2</v>
+      </c>
       <c r="P75" t="inlineStr">
         <is>
           <t xml:space="preserve">Péruvienne</t>
@@ -6147,16 +6147,16 @@
     <hyperlink ref="H41" r:id="rId26" display="https://www.laphilo.fr/pho/mrothbard-mini.webp"/>
     <hyperlink ref="H42" r:id="rId27" display="https://www.laphilo.fr/pho/ewiesel-mini.webp"/>
     <hyperlink ref="H43" r:id="rId28" display="https://www.laphilo.fr/pho/abracken-mini.webp"/>
-    <hyperlink ref="E44" r:id="rId29" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Richard_Rorty&quot; title=&quot; Wikipedia&quot;&gt;Richard RORTY&lt;/a&gt; était un  philosophe américain, figure majeure du  &lt;a href=&quot;https://www.youtube.com/watch?v=lfx4Jag1ic4&quot;  title=&quot;Le pragmatisme : définition, exemples par le savoir partagé&quot;&gt;pragmatisme&lt;/a&gt; et du postmodernisme, il a remis en cause les fondements de la philosophie occidentale et proposé une &lt;a href=&quot;https://laviedesidees.fr/Rorty-Pragmatism-Anti-Authoritarianism&quot; title=&quot; a bas l'autorité par laviedesidees&quot;&gt;vision radicale&lt;/a&gt;  de la vérité, de la culture et de la société. Il rejette l'idée que la vérité soit une correspondance entre le langage et la réalité. Pour lui, la vérité est simplement ce qui est utile ou avantageux à croire dans une communauté donnée et il propose d'abandonner la quête de fondements absolus de la connaissance, jugée vaine. &lt;/p&gt; &lt;p&gt; Inspiré par Wittgenstein et Davidson, il considère le langage non pas comme un miroir de la réalité, mais comme un ensemble d'outils pour résoudre des problèmes pratiques.  Les vocabularies que nous utilisons sont historiquement et culturellement contingents, non pas &quot;vrais&quot; ou &quot;faux&quot;. &lt;/p&gt; &lt;p&gt; Dans ces oeuvres principales , on trouve  &lt;a href=&quot;https://www.youtube.com/watch?v=MgU0dXZ3umM&quot; title=&quot;L’ironiste libéral chez Rorty : Contingence, ironie et solidarité par Darina Metreveli&quot;&gt;&quot; Contingence, ironie et solidarité &quot;&lt;/a&gt; (1989) ou il décrit l'ironiste comme quelqu'un qui doute de ses propres croyances tout en œuvrant pour une société plus juste. Dans &quot; Achieving Our Country&quot; (1998),  il y appelle la gauche américaine à abandonner le &quot;culturalisme&quot; pour se recentrer sur les inégalités économiques et sociales. Cet ouvrage est souvent cité pour avoir anticipé les crises politiques du XXIe siècle. &lt;/p&gt; &lt;p&gt;  Ses thèses sur la contingence de la vérité sont souvent invoquées pour analyser l'ère de la &quot;post-vérité&quot;. Son insistance sur la conversation comme fondement du lien social influence la philosophie politique contemporaine. Il  a bouleversé la philosophie en démystifiant ses prétentions à la vérité absolue. Son œuvre, à la fois provocante et humaniste, invite à remplacer la quête métaphysique par un engagement en faveur d'une société plus juste et plus inclusive. &lt;/p&gt; "/>
-    <hyperlink ref="E46" r:id="rId30" display="&lt;p&gt;&lt;a href=&quot;https://en.wikipedia.org/wiki/Charles_Parsons_(philosopher)&quot;  title=&quot; Wikipedia&quot;&gt;Charles Dacre PARSONS&lt;/a&gt; était un philosophe américain connu pour ses travaux en philosophie des mathématiques et en philosophie de Kant. Il a enseigné à Columbia puis à Harvard, où il est devenu professeur émérite. Il s’est formé à Harvard, avec une thèse dirigée par Willard Van Orman Quine, ce qui le place au croisement de la logique, de la philosophie analytique et des fondements des mathématiques. Son parcours intellectuel a été marqué très tôt par la rigueur mathématique, puisqu’il avait d’abord étudié les mathématiques avant de se tourner vers la philosophie. &lt;/p&gt; &lt;p&gt; Son apport principal concerne la philosophie des mathématiques, domaine dans lequel il a travaillé sur la nature des objets mathématiques, la logique, la preuve et l’interprétation constructive des mathématiques prédicatives. Il a aussi beaucoup écrit sur Frege, Gödel, Hilbert et Quine, en lisant ces auteurs à la fois comme philosophes et comme figures majeures des fondements. &lt;/p&gt; &lt;p&gt; Il n’était pas seulement un spécialiste de logique ; il a aussi produit des travaux importants sur Kant, montrant comment les questions de connaissance, d’expérience et de structure de l’esprit se relient aux mathématiques. Cette double compétence, en philosophie des mathématiques et en histoire de la philosophie, explique pourquoi il est souvent vu comme un auteur à la fois technique et très large dans ses intérêts.&lt;/p&gt; &lt;p&gt; Son influence est restée forte dans le monde anglophone, au point d’être décrit comme l’un des philosophes des mathématiques les plus importants de sa génération. En plus de ses livres et articles, il a aussi contribué à l’édition de textes posthumes de Gödel, ce qui a renforcé son rôle dans l’étude contemporaine des fondements des mathématiques. &lt;/p&gt; &#10;&#10;&#10;"/>
-    <hyperlink ref="I46" r:id="rId31" display="https://www.laphilo.fr/photo/cparsons.webp"/>
-    <hyperlink ref="H48" r:id="rId32" display="https://www.laphilo.fr/pho/dihde-mini.webp"/>
-    <hyperlink ref="E50" r:id="rId33" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Edward_Sa%C3%AFd&quot;  title=&quot; Wikipedia&quot;&gt;Edward SAÏD&lt;/a&gt; était un intellectuel palestinien-américain, critique littéraire et professeur de littérature anglaise et comparée à l’université Columbia de New York. D’origine palestinienne et né à Jérusalem, il a grandi entre l’Égypte, les États-Unis et l’Europe, une expérience de déplacement qui a profondément marqué sa pensée sur l’identité, la colonisation et l’altérité.  &lt;/p&gt; &lt;p&gt; Sa contribution la plus célèbre est l’essai &lt;a href=&quot;https://www.youtube.com/watch?v=Ne4WRykmjhA&quot; title=&quot;Edward Said  Orientalisme par HD Doc&quot;&gt;L’Orientalisme : &lt;/a&gt;  L’Orient créé par l’Occident* (1978), considéré comme le texte fondateur des postcolonial studies. Dans cet ouvrage, Saïd montre que l’« Orient » n’est pas une réalité objective mais une invention de l’Occident : un discours façonné par des siècles de domination coloniale pour mieux contrôler et représenter l’Autre. &lt;/p&gt; &lt;p&gt; Pour lui, l’orientalisme est à la fois un savoir et un outil de pouvoir : il ne s’agit pas seulement de décrire l’Orient, mais de le hiérarchiser, de l’essentialiser et de le rendre  &lt;a href=&quot;https://www.youtube.com/watch?v=QBj-yWLnayM&quot; title=&quot;Edward Said writings on Orientalism par Middle East Eye&quot;&gt; inférieur à l’Occident. &lt;/a&gt; Il analyse quatre thèses principales : la domination politique et culturelle de l’Orient par l’Occident, la dépréciation de la langue arabe, la diabolisation de l’arabe et de l’islam, et la défense de la cause palestinienne. &lt;/p&gt; &lt;p&gt; Sa pensée articule critique littéraire, histoire, philosophie et sciences politiques, en s’inspirant notamment de Michel Foucault (discours–pouvoir) et de Jacques Derrida (déconstruction). Il montre que la violence du colonialisme n’est pas seulement matérielle (conquête, pillage), mais aussi épistémique : une violence de la raison qui classe, essentialise et dévalue les « Autres » de l’Occident. &lt;/p&gt; &lt;p&gt;  Intéressé par &lt;a href=&quot;https://www.lesclesdumoyenorient.com/Edward-W-Said-1935-2003.html&quot; title=&quot;Edward Said par lesclesdumoyenorient&quot;&gt; l’engagement politique, &lt;/a&gt; il a aussi défendu la cause palestinienne et la légitimité des revendications d’autodétermination du peuple palestinien, tout en reconnaissance du droit à une patrie juive. Il rejetait le repli identitaire et prônait une vision universelle qui défend les différences et les droits, tissant des liens entre classicisme et excentricité, histoire et actualité. &lt;/p&gt;  &lt;audio controls title=&quot;Edward Said, une conscience morale par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/12360-08.12.2017-ITEMA_21518070-2017C19327S0342-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;  &#10;&#10;&#10;"/>
-    <hyperlink ref="H50" r:id="rId34" display="https://laphilo.fr/pho/esaid-mini.webp"/>
-    <hyperlink ref="H51" r:id="rId35" display="https://www.laphilo.fr/pho/rmadams-mini.webp"/>
-    <hyperlink ref="E52" r:id="rId36" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Robert_Nozick&quot;  title=&quot; Wikipedia&quot;&gt;Robert NOZICK&lt;/a&gt; était un philosophe américain connu pour &lt;a href=&quot;https://www.youtube.com/watch?v=Q-t3cpFAk4o&quot;  title=&quot; Libertarianisme par Vadim Media&quot;&gt; son libertarianisme &lt;/a&gt; et sa critique des théories égalitaristes comme celle de John Rawls. Professeur à Harvard, il a marqué la philosophie politique, morale et épistémologique par son œuvre principale, Anarchie, État et utopie (1974), qui défend un  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Minarchisme&quot;  title=&quot; Minarchisme par Wikipédia&quot;&gt; Etat Minimal. &lt;/a&gt; &lt;/p&gt; &lt;p&gt; Il argue que seul l'État minimal, ou &quot;État gardien de nuit&quot;, est légitime, car il se limite à protéger les individus contre la force, la fraude et le vol, sans redistribuer les richesses. Il rejette l'anarcho-capitalisme en montrant, via des agences de protection privée, comment un État dominant émerge naturellement pour monopoliser la coercition légitime, justifié par le droit naturel à la personne. &lt;/p&gt; &lt;p&gt; Contrairement à la justice distributive de Rawls, il propose une théorie de l'entitlement : une acquisition initiale juste et des transferts volontaires rendent la distribution légitime, sans besoin d'égalisation par l'État. Toute intervention redistributive viole les droits individuels, traitant les personnes comme des moyens plutôt que des fins, en écho à Kant. &lt;/p&gt; &lt;p&gt; Dans Anarchie, État et utopie, Il réfute l'utilitarisme via l'expérience de pensée de la &lt;a href=&quot;https://www.youtube.com/watch?v=2FVwXaNWPQ0&quot;  title=&quot; La machine à expérience par Monsieur Phi&quot;&gt;&quot;machine à expérience&quot; :&lt;/a&gt;  même si elle offre un bonheur parfait et indistinguable de la réalité, les gens préfèrent vivre des actions réelles et façonner leur identité plutôt que des simulations. Cela prouve que le bonheur n'est pas le seul bien suprême. &lt;/p&gt; &lt;p&gt; Plus tard, dans Explications philosophiques (1981), il développe une théorie du suivi (tracking theory) en épistémologie, où la connaissance repose sur des conditionnels contrefactuels fiables, contournant le scepticisme sans justification traditionnelle. Son anti-coercitivisme intellectuel invite à une philosophie ouverte, non imposée. &lt;/p&gt; &#10;&lt;audio controls title=&quot;Qui a peur des Libertariens par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10467-14.06.2022-ITEMA_23058436-2022C12410S0165-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt;&lt;/audio&gt;&#10;"/>
-    <hyperlink ref="H58" r:id="rId37" display="https://www.laphilo.fr/pho/imyoung-mini.webp"/>
-    <hyperlink ref="H59" r:id="rId38" display="https://www.laphilo.fr/pho/bhooks-mini.webp"/>
+    <hyperlink ref="E45" r:id="rId29" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Richard_Rorty&quot; title=&quot; Wikipedia&quot;&gt;Richard RORTY&lt;/a&gt; était un  philosophe américain, figure majeure du  &lt;a href=&quot;https://www.youtube.com/watch?v=lfx4Jag1ic4&quot;  title=&quot;Le pragmatisme : définition, exemples par le savoir partagé&quot;&gt;pragmatisme&lt;/a&gt; et du postmodernisme, il a remis en cause les fondements de la philosophie occidentale et proposé une &lt;a href=&quot;https://laviedesidees.fr/Rorty-Pragmatism-Anti-Authoritarianism&quot; title=&quot; a bas l'autorité par laviedesidees&quot;&gt;vision radicale&lt;/a&gt;  de la vérité, de la culture et de la société. Il rejette l'idée que la vérité soit une correspondance entre le langage et la réalité. Pour lui, la vérité est simplement ce qui est utile ou avantageux à croire dans une communauté donnée et il propose d'abandonner la quête de fondements absolus de la connaissance, jugée vaine. &lt;/p&gt; &lt;p&gt; Inspiré par Wittgenstein et Davidson, il considère le langage non pas comme un miroir de la réalité, mais comme un ensemble d'outils pour résoudre des problèmes pratiques.  Les vocabularies que nous utilisons sont historiquement et culturellement contingents, non pas &quot;vrais&quot; ou &quot;faux&quot;. &lt;/p&gt; &lt;p&gt; Dans ces oeuvres principales , on trouve  &lt;a href=&quot;https://www.youtube.com/watch?v=MgU0dXZ3umM&quot; title=&quot;L’ironiste libéral chez Rorty : Contingence, ironie et solidarité par Darina Metreveli&quot;&gt;&quot; Contingence, ironie et solidarité &quot;&lt;/a&gt; (1989) ou il décrit l'ironiste comme quelqu'un qui doute de ses propres croyances tout en œuvrant pour une société plus juste. Dans &quot; Achieving Our Country&quot; (1998),  il y appelle la gauche américaine à abandonner le &quot;culturalisme&quot; pour se recentrer sur les inégalités économiques et sociales. Cet ouvrage est souvent cité pour avoir anticipé les crises politiques du XXIe siècle. &lt;/p&gt; &lt;p&gt;  Ses thèses sur la contingence de la vérité sont souvent invoquées pour analyser l'ère de la &quot;post-vérité&quot;. Son insistance sur la conversation comme fondement du lien social influence la philosophie politique contemporaine. Il  a bouleversé la philosophie en démystifiant ses prétentions à la vérité absolue. Son œuvre, à la fois provocante et humaniste, invite à remplacer la quête métaphysique par un engagement en faveur d'une société plus juste et plus inclusive. &lt;/p&gt; "/>
+    <hyperlink ref="E47" r:id="rId30" display="&lt;p&gt;&lt;a href=&quot;https://en.wikipedia.org/wiki/Charles_Parsons_(philosopher)&quot;  title=&quot; Wikipedia&quot;&gt;Charles Dacre PARSONS&lt;/a&gt; était un philosophe américain connu pour ses travaux en philosophie des mathématiques et en philosophie de Kant. Il a enseigné à Columbia puis à Harvard, où il est devenu professeur émérite. Il s’est formé à Harvard, avec une thèse dirigée par Willard Van Orman Quine, ce qui le place au croisement de la logique, de la philosophie analytique et des fondements des mathématiques. Son parcours intellectuel a été marqué très tôt par la rigueur mathématique, puisqu’il avait d’abord étudié les mathématiques avant de se tourner vers la philosophie. &lt;/p&gt; &lt;p&gt; Son apport principal concerne la philosophie des mathématiques, domaine dans lequel il a travaillé sur la nature des objets mathématiques, la logique, la preuve et l’interprétation constructive des mathématiques prédicatives. Il a aussi beaucoup écrit sur Frege, Gödel, Hilbert et Quine, en lisant ces auteurs à la fois comme philosophes et comme figures majeures des fondements. &lt;/p&gt; &lt;p&gt; Il n’était pas seulement un spécialiste de logique ; il a aussi produit des travaux importants sur Kant, montrant comment les questions de connaissance, d’expérience et de structure de l’esprit se relient aux mathématiques. Cette double compétence, en philosophie des mathématiques et en histoire de la philosophie, explique pourquoi il est souvent vu comme un auteur à la fois technique et très large dans ses intérêts.&lt;/p&gt; &lt;p&gt; Son influence est restée forte dans le monde anglophone, au point d’être décrit comme l’un des philosophes des mathématiques les plus importants de sa génération. En plus de ses livres et articles, il a aussi contribué à l’édition de textes posthumes de Gödel, ce qui a renforcé son rôle dans l’étude contemporaine des fondements des mathématiques. &lt;/p&gt; &#10;&#10;&#10;"/>
+    <hyperlink ref="I47" r:id="rId31" display="https://www.laphilo.fr/photo/cparsons.webp"/>
+    <hyperlink ref="H49" r:id="rId32" display="https://www.laphilo.fr/pho/dihde-mini.webp"/>
+    <hyperlink ref="E51" r:id="rId33" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Edward_Sa%C3%AFd&quot;  title=&quot; Wikipedia&quot;&gt;Edward SAÏD&lt;/a&gt; était un intellectuel palestinien-américain, critique littéraire et professeur de littérature anglaise et comparée à l’université Columbia de New York. D’origine palestinienne et né à Jérusalem, il a grandi entre l’Égypte, les États-Unis et l’Europe, une expérience de déplacement qui a profondément marqué sa pensée sur l’identité, la colonisation et l’altérité.  &lt;/p&gt; &lt;p&gt; Sa contribution la plus célèbre est l’essai &lt;a href=&quot;https://www.youtube.com/watch?v=Ne4WRykmjhA&quot; title=&quot;Edward Said  Orientalisme par HD Doc&quot;&gt;L’Orientalisme : &lt;/a&gt;  L’Orient créé par l’Occident* (1978), considéré comme le texte fondateur des postcolonial studies. Dans cet ouvrage, Saïd montre que l’« Orient » n’est pas une réalité objective mais une invention de l’Occident : un discours façonné par des siècles de domination coloniale pour mieux contrôler et représenter l’Autre. &lt;/p&gt; &lt;p&gt; Pour lui, l’orientalisme est à la fois un savoir et un outil de pouvoir : il ne s’agit pas seulement de décrire l’Orient, mais de le hiérarchiser, de l’essentialiser et de le rendre  &lt;a href=&quot;https://www.youtube.com/watch?v=QBj-yWLnayM&quot; title=&quot;Edward Said writings on Orientalism par Middle East Eye&quot;&gt; inférieur à l’Occident. &lt;/a&gt; Il analyse quatre thèses principales : la domination politique et culturelle de l’Orient par l’Occident, la dépréciation de la langue arabe, la diabolisation de l’arabe et de l’islam, et la défense de la cause palestinienne. &lt;/p&gt; &lt;p&gt; Sa pensée articule critique littéraire, histoire, philosophie et sciences politiques, en s’inspirant notamment de Michel Foucault (discours–pouvoir) et de Jacques Derrida (déconstruction). Il montre que la violence du colonialisme n’est pas seulement matérielle (conquête, pillage), mais aussi épistémique : une violence de la raison qui classe, essentialise et dévalue les « Autres » de l’Occident. &lt;/p&gt; &lt;p&gt;  Intéressé par &lt;a href=&quot;https://www.lesclesdumoyenorient.com/Edward-W-Said-1935-2003.html&quot; title=&quot;Edward Said par lesclesdumoyenorient&quot;&gt; l’engagement politique, &lt;/a&gt; il a aussi défendu la cause palestinienne et la légitimité des revendications d’autodétermination du peuple palestinien, tout en reconnaissance du droit à une patrie juive. Il rejetait le repli identitaire et prônait une vision universelle qui défend les différences et les droits, tissant des liens entre classicisme et excentricité, histoire et actualité. &lt;/p&gt;  &lt;audio controls title=&quot;Edward Said, une conscience morale par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/12360-08.12.2017-ITEMA_21518070-2017C19327S0342-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;  &#10;&#10;&#10;"/>
+    <hyperlink ref="H51" r:id="rId34" display="https://laphilo.fr/pho/esaid-mini.webp"/>
+    <hyperlink ref="H52" r:id="rId35" display="https://www.laphilo.fr/pho/rmadams-mini.webp"/>
+    <hyperlink ref="E53" r:id="rId36" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Robert_Nozick&quot;  title=&quot; Wikipedia&quot;&gt;Robert NOZICK&lt;/a&gt; était un philosophe américain connu pour &lt;a href=&quot;https://www.youtube.com/watch?v=Q-t3cpFAk4o&quot;  title=&quot; Libertarianisme par Vadim Media&quot;&gt; son libertarianisme &lt;/a&gt; et sa critique des théories égalitaristes comme celle de John Rawls. Professeur à Harvard, il a marqué la philosophie politique, morale et épistémologique par son œuvre principale, Anarchie, État et utopie (1974), qui défend un  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Minarchisme&quot;  title=&quot; Minarchisme par Wikipédia&quot;&gt; Etat Minimal. &lt;/a&gt; &lt;/p&gt; &lt;p&gt; Il argue que seul l'État minimal, ou &quot;État gardien de nuit&quot;, est légitime, car il se limite à protéger les individus contre la force, la fraude et le vol, sans redistribuer les richesses. Il rejette l'anarcho-capitalisme en montrant, via des agences de protection privée, comment un État dominant émerge naturellement pour monopoliser la coercition légitime, justifié par le droit naturel à la personne. &lt;/p&gt; &lt;p&gt; Contrairement à la justice distributive de Rawls, il propose une théorie de l'entitlement : une acquisition initiale juste et des transferts volontaires rendent la distribution légitime, sans besoin d'égalisation par l'État. Toute intervention redistributive viole les droits individuels, traitant les personnes comme des moyens plutôt que des fins, en écho à Kant. &lt;/p&gt; &lt;p&gt; Dans Anarchie, État et utopie, Il réfute l'utilitarisme via l'expérience de pensée de la &lt;a href=&quot;https://www.youtube.com/watch?v=2FVwXaNWPQ0&quot;  title=&quot; La machine à expérience par Monsieur Phi&quot;&gt;&quot;machine à expérience&quot; :&lt;/a&gt;  même si elle offre un bonheur parfait et indistinguable de la réalité, les gens préfèrent vivre des actions réelles et façonner leur identité plutôt que des simulations. Cela prouve que le bonheur n'est pas le seul bien suprême. &lt;/p&gt; &lt;p&gt; Plus tard, dans Explications philosophiques (1981), il développe une théorie du suivi (tracking theory) en épistémologie, où la connaissance repose sur des conditionnels contrefactuels fiables, contournant le scepticisme sans justification traditionnelle. Son anti-coercitivisme intellectuel invite à une philosophie ouverte, non imposée. &lt;/p&gt; &#10;&lt;audio controls title=&quot;Qui a peur des Libertariens par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10467-14.06.2022-ITEMA_23058436-2022C12410S0165-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt;&lt;/audio&gt;&#10;"/>
+    <hyperlink ref="H59" r:id="rId37" display="https://www.laphilo.fr/pho/imyoung-mini.webp"/>
+    <hyperlink ref="H60" r:id="rId38" display="https://www.laphilo.fr/pho/bhooks-mini.webp"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Fiches — 7 fiches modifiées : Newton DA COSTA, Marilena CHAUI, PRODICOS de Céos, HIPPIAS d'Élis, LIE Zi, Viola CORDOVA et 1 autre(s) ; 5 images
Publié depuis l'éditeur des fiches.
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-americains.xlsx
+++ b/data/frise-philosophes-americains.xlsx
@@ -4087,941 +4087,937 @@
         <v>51</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7" t="n">
+    <row r="43" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1">
+        <v>1929</v>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1929 – 2024</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Newton DA COSTA</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Newton_da_Costa" title=" Wikipedia (en)"&gt;Newton DA COSTA&lt;/a&gt; est un logicien et philosophe brésilien, l’un des fondateurs de la &lt;a href="https://fr.wikipedia.org/wiki/Logique_paraconsistante" title=" Wikipedia"&gt;logique paraconsistante&lt;/a&gt;. Né à Curitiba, il étudie d’abord le génie civil puis les mathématiques, et enseigne à l’université fédérale du Paraná, puis à l’université de São Paulo et à l’université fédérale de Santa Catarina.&lt;/p&gt; &lt;p&gt;Dans la logique classique, une seule contradiction suffit à tout prouver : si l’on admet à la fois une proposition et sa négation, on peut en déduire n’importe quoi. C’est le principe d’« explosion ». Dès sa thèse de 1963, il construit des systèmes logiques, appelés « calculs C », où l’on peut admettre certaines contradictions sans que toute la théorie s’effondre. Le nom de « paraconsistance » leur est donné en 1976 par le philosophe péruvien Francisco Miró Quesada. Ces logiques permettent de raisonner rigoureusement sur des informations contradictoires, comme celles d’une base de données, d’un témoignage ou d’une théorie scientifique en crise.&lt;/p&gt; &lt;p&gt;Il &lt;a href="https://www.youtube.com/watch?v=Zo-o_fHnfkA" title="Newton da Costa sobre a leitura par Fábio Salgado de Carvalho"&gt;étend ces travaux &lt;/a&gt;à la théorie des ensembles et à la philosophie des sciences. Avec Steven French, il développe la notion de « quasi-vérité » : une théorie scientifique peut être partiellement vraie et utile sans être entièrement exacte. Avec Francisco Antônio Dória, il montre en 1991 que certaines questions de la théorie du chaos sont indécidables : aucun calcul ne peut y répondre. Membre de nombreuses académies, il a formé une importante école de logique au Brésil et en Amérique latine. Il meurt en 2024 à Florianópolis.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LXOUyxZNuL8</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Newton da Costa, o maior pensador brasileiro" par Verve Científica</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/dacosta-mini.webp</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">logique ; epistemologie</t>
+        </is>
+      </c>
+      <c r="K43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Logique paraconsistante</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">logicien brésilien, l’un des fondateurs des logiques paraconsistantes.</t>
+        </is>
+      </c>
+      <c r="N43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brésilienne</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="7" t="n">
         <v>1930</v>
       </c>
-      <c r="B43" s="7" t="s">
+      <c r="B44" s="7" t="s">
         <v>322</v>
       </c>
-      <c r="C43" s="7" t="s">
+      <c r="C44" s="7" t="s">
         <v>367</v>
       </c>
-      <c r="D43" s="8" t="s">
+      <c r="D44" s="8" t="s">
         <v>368</v>
       </c>
-      <c r="E43" s="11" t="s">
+      <c r="E44" s="11" t="s">
         <v>369</v>
       </c>
-      <c r="F43" s="7" t="s">
+      <c r="F44" s="7" t="s">
         <v>370</v>
       </c>
-      <c r="G43" s="9" t="s">
+      <c r="G44" s="9" t="s">
         <v>371</v>
       </c>
-      <c r="H43" s="10" t="s">
+      <c r="H44" s="10" t="s">
         <v>372</v>
       </c>
-      <c r="I43" s="9"/>
-      <c r="J43" s="2" t="s">
+      <c r="I44" s="9"/>
+      <c r="J44" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="K43" s="2" t="s">
+      <c r="K44" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="L43" s="2" t="s">
+      <c r="L44" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="N43" s="1" t="s">
+      <c r="N44" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="1">
+    <row r="45" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1">
         <v>1930</v>
       </c>
-      <c r="B44" s="1" t="inlineStr">
+      <c r="B45" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">2018</t>
         </is>
       </c>
-      <c r="C44" s="1" t="inlineStr">
+      <c r="C45" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">1930 – 2018</t>
         </is>
       </c>
-      <c r="D44" s="1" t="inlineStr">
+      <c r="D45" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Aníbal QUIJANO</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/An%C3%ADbal_Quijano" title=" Wikipedia"&gt;Aníbal QUIJANO&lt;/a&gt; est un sociologue péruvien, l’un des grands penseurs latino-américains du XXe siècle et le fondateur de la pensée décoloniale. Né en 1928 à Yanama, dans les Andes péruviennes, il étudie à l’université de San Marcos, à Lima, où il enseigne ensuite la sociologie. Dans les années 1960 et 1970, il participe aux travaux de la &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9orie_de_la_d%C3%A9pendance" title=" Wikipedia"&gt;théorie de la dépendance&lt;/a&gt;, qui explique le sous-développement de l’Amérique latine par sa place subordonnée dans l’économie mondiale, et étudie la condition des populations indiennes et métisses des villes.&lt;/p&gt; &lt;p&gt;En 1992, pour le cinquième centenaire de l’arrivée de Christophe Colomb, il publie l’article « Colonialité et modernité/rationalité », qui forge la notion de « colonialité du pouvoir ». La conquête de l’Amérique a donné naissance à la fois au capitalisme mondial et à une idée nouvelle, celle de « race », qui a permis de classer les peuples en supérieurs et inférieurs et de distribuer entre eux le travail : le salariat pour les Européens, le servage pour les Indiens, l’esclavage pour les Africains. Cette classification a survécu à l’indépendance des colonies : elle structure encore les rapports sociaux, le savoir et la manière dont chacun se perçoit. Quijano critique aussi l’« eurocentrisme », qui fait de l’histoire européenne le modèle de l’histoire universelle.&lt;/p&gt; &lt;p&gt;Professeur à l’université de Binghamton, aux États-Unis, il anime le &lt;a href="https://fr.wikipedia.org/wiki/Groupe_modernit%C3%A9/colonialit%C3%A9" title=" Wikipedia"&gt;groupe « modernité/colonialité »&lt;/a&gt; avec Walter Mignolo et Enrique Dussel. La philosophe argentine &lt;a href="https://fr.wikipedia.org/wiki/Mar%C3%ADa_Lugones" title=" Wikipedia"&gt;María Lugones&lt;/a&gt; a prolongé son concept dans celui de « colonialité du genre ». Il meurt à Lima en 2018.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t xml:space="preserve">aibG8RehlTE</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t xml:space="preserve">"Aníbal Quijano - Colonialidad del Poder" par Filo Errante</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/quijano-mini.webp</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
+      <c r="J45" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">politique ; epistemologie</t>
         </is>
       </c>
-      <c r="K44" s="1" t="inlineStr">
+      <c r="K45" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Pensée décoloniale</t>
         </is>
       </c>
-      <c r="L44" s="2" t="inlineStr">
+      <c r="L45" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">sociologue péruvien, inventeur de la « colonialité du pouvoir » et fondateur de la pensée décoloniale.</t>
         </is>
       </c>
-      <c r="N44" s="1" t="inlineStr">
+      <c r="N45" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">sud</t>
         </is>
       </c>
-      <c r="O44" s="1"/>
-      <c r="P44" t="inlineStr">
+      <c r="O45" s="1"/>
+      <c r="P45" t="inlineStr">
         <is>
           <t xml:space="preserve">Péruvienne</t>
         </is>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7" t="n">
+    <row r="46" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="7" t="n">
         <v>1931</v>
       </c>
-      <c r="B45" s="7" t="s">
+      <c r="B46" s="7" t="s">
         <v>374</v>
       </c>
-      <c r="C45" s="7" t="s">
+      <c r="C46" s="7" t="s">
         <v>375</v>
       </c>
-      <c r="D45" s="8" t="s">
+      <c r="D46" s="8" t="s">
         <v>376</v>
       </c>
-      <c r="E45" s="10" t="inlineStr">
+      <c r="E46" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Richard_Rorty" title=" Wikipedia"&gt;Richard RORTY&lt;/a&gt; était un  philosophe américain, figure majeure du  &lt;a href="https://www.youtube.com/watch?v=lfx4Jag1ic4"  title="Le pragmatisme : définition, exemples par le savoir partagé"&gt;pragmatisme&lt;/a&gt; et du postmodernisme, il a remis en cause les fondements de la philosophie occidentale et proposé une &lt;a href="https://laviedesidees.fr/Rorty-Pragmatism-Anti-Authoritarianism" title=" a bas l'autorité par laviedesidees"&gt;vision radicale&lt;/a&gt;  de la vérité, de la culture et de la société. Il rejette l'idée que la vérité soit une correspondance entre le langage et la réalité. Pour lui, la vérité est simplement ce qui est utile ou avantageux à croire dans une communauté donnée et il propose d'abandonner la quête de fondements absolus de la connaissance, jugée vaine. &lt;/p&gt; &lt;p&gt; Inspiré par Wittgenstein et Davidson, il considère le langage non pas comme un miroir de la réalité, mais comme un ensemble d'outils pour résoudre des problèmes pratiques.  Les vocabularies que nous utilisons sont historiquement et culturellement contingents, non pas "vrais" ou "faux". &lt;/p&gt; &lt;p&gt; Dans ces oeuvres principales, on trouve  &lt;a href="https://www.youtube.com/watch?v=MgU0dXZ3umM" title="L’ironiste libéral chez Rorty : Contingence, ironie et solidarité par Darina Metreveli"&gt;" Contingence, ironie et solidarité "&lt;/a&gt; (1989) ou il décrit l'ironiste comme quelqu'un qui doute de ses propres croyances tout en œuvrant pour une société plus juste. Dans " Achieving Our Country" (1998),  il y appelle la gauche américaine à abandonner le "culturalisme" pour se recentrer sur les inégalités économiques et sociales. Cet ouvrage est souvent cité pour avoir anticipé les crises politiques du XXIe siècle. &lt;/p&gt; &lt;p&gt;  Ses thèses sur la contingence de la vérité sont souvent invoquées pour analyser l'ère de la "post-vérité". Son insistance sur la conversation comme fondement du lien social influence la philosophie politique contemporaine. Il  a bouleversé la philosophie en démystifiant ses prétentions à la vérité absolue. Son œuvre, à la fois provocante et humaniste, invite à remplacer la quête métaphysique par un engagement en faveur d'une société plus juste et plus inclusive. &lt;/p&gt; </t>
         </is>
       </c>
-      <c r="F45" s="7" t="s">
+      <c r="F46" s="7" t="s">
         <v>378</v>
       </c>
-      <c r="G45" s="9" t="s">
+      <c r="G46" s="9" t="s">
         <v>379</v>
       </c>
-      <c r="H45" s="9" t="s">
+      <c r="H46" s="9" t="s">
         <v>380</v>
       </c>
-      <c r="I45" s="9"/>
-      <c r="J45" s="2" t="s">
+      <c r="I46" s="9"/>
+      <c r="J46" s="2" t="s">
         <v>381</v>
       </c>
-      <c r="K45" s="2" t="s">
+      <c r="K46" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="L45" s="2" t="s">
+      <c r="L46" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="N45" s="1" t="s">
+      <c r="N46" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="293.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="1" t="n">
+    <row r="47" customFormat="false" ht="293.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="n">
         <v>1932</v>
       </c>
-      <c r="B46" s="1" t="n">
+      <c r="B47" s="1" t="n">
         <v>2025</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="C47" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="D47" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/John_Searle"  title=" Wikipedia"&gt;John SEARLE&lt;/a&gt; était un philosophe américain  connu pour ses travaux influents dans plusieurs domaines, notamment la philosophie du langage, la philosophie de l'esprit et la philosophie sociale. Il  a développé et systématisé la théorie des &lt;a href="https://www.youtube.com/watch?v=pIbkpLfrD6A" title="
 La théorie des actes de langage (2) - John Searle par Heraut du Mont Parnasse"&gt;actes de langage&lt;/a&gt; car, pour lui, parler une langue, ce n'est pas seulement émettre des sons ou des suites de symboles, mais accomplir des actions. &lt;/p&gt; &lt;p&gt; Défenseur du "naturalisme biologique" en philosophie de l'esprit. Il s'oppose au dualisme cartésien tout en refusant le matérialisme réducteur qui nierait l'existence de &lt;a href="https://www.youtube.com/watch?v=EriAhi0mj7w" title=" Conscience et matière grise par TEDx Talks"&gt;la conscience&lt;/a&gt; ou la réduirirait à de simples phénomènes physiques. Pour lui, les états mentaux (douleur, croyances, désirs, conscience) sont des phénomènes  &lt;a href="https://www.youtube.com/watch?v=Bq2bfSzkTfU"  title="John Searle - Une personne peut-elle être une âme ? par Closer To Truth"&gt;biologiques réels&lt;/a&gt;, causés par des processus neuronaux du cerveau, mais ils ne sont pas réductibles à ces processus au sens où ils émergent à un niveau supérieur et possèdent des propriétés irréductibles.&lt;/p&gt; &lt;p&gt; L'une des ses contributions les plus célèbres est son argument de la &lt;a href="https://www.youtube.com/watch?v=P5DtwDr9YEc" title=" La Chambre chinoise par Ian et frank"&gt;Chambre Chinoise&lt;/a&gt;. Cet argument vise à réfuter la thèse de l'IA forte (position selon laquelle un ordinateur programmé de manière appropriée n'est pas seulement un outil pour l'étude de l'esprit, mais qu'il est véritablement un esprit, capable de comprendre et de posséder d'autres états cognitifs) opposé à l'IA faible (position selon laquelle les ordinateurs sont des outils utiles pour étudier l'esprit, mais qu'ils ne sont pas eux-mêmes des esprits). &lt;/p&gt; &lt;p&gt; Dans son ouvrage &lt;a href="https://labo.nonmarchand.org/pmwiki/uploads/Textes/JohnSearleLaConstructionDeLaRealiteSociale/JohnSearle_LaConstructionDeLaRealiteSociale.pdf"  title=" La construction e la réalité sociale par nonmarchand"&gt;"La Construction de la Réalité Sociale"&lt;/a&gt;, il étend sa théorie des actes de langage et de l'intentionnalité pour expliquer comment nous construisons des faits institutionnels et sociaux. Il distingue les "Faits bruts" qui existent indépendamment de toute institution humaine (par exemple, la montagne Everest) des "Faits institutionnels" qui n'existent qu'en vertu d'institutions humaines et de l'accord collectif (par exemple, l'argent, le mariage, la propriété). &lt;/p&gt; 
 </t>
         </is>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="F47" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="G47" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="H46" s="2" t="s">
+      <c r="H47" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="I46" s="1"/>
-      <c r="J46" s="2" t="s">
+      <c r="I47" s="1"/>
+      <c r="J47" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="K46" s="1" t="s">
+      <c r="K47" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="L46" s="2" t="s">
+      <c r="L47" s="2" t="s">
         <v>391</v>
-      </c>
-      <c r="N46" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="P46" s="1" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="171.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="n">
-        <v>1933</v>
-      </c>
-      <c r="B47" s="7" t="s">
-        <v>322</v>
-      </c>
-      <c r="C47" s="7" t="s">
-        <v>393</v>
-      </c>
-      <c r="D47" s="8" t="s">
-        <v>394</v>
-      </c>
-      <c r="E47" s="13" t="s">
-        <v>395</v>
-      </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OvpUxJQRAbw</t>
-        </is>
-      </c>
-      <c r="G47" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"Charles Parsons Intuition and Reason | HUSSERL to GODEL | Mark van Atten" par The Van Leer Jerusalem Institute - מכון ון ליר בירושלים</t>
-        </is>
-      </c>
-      <c r="H47" s="9" t="s">
-        <v>396</v>
-      </c>
-      <c r="I47" s="10" t="s">
-        <v>397</v>
-      </c>
-      <c r="J47" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="K47" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="L47" s="2" t="s">
-        <v>399</v>
       </c>
       <c r="N47" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="48" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P47" s="1" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="171.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="n">
+        <v>1933</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="D48" s="8" t="s">
+        <v>394</v>
+      </c>
+      <c r="E48" s="13" t="s">
+        <v>395</v>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OvpUxJQRAbw</t>
+        </is>
+      </c>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Charles Parsons Intuition and Reason | HUSSERL to GODEL | Mark van Atten" par The Van Leer Jerusalem Institute - מכון ון ליר בירושלים</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="s">
+        <v>396</v>
+      </c>
+      <c r="I48" s="10" t="s">
+        <v>397</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="L48" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="N48" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="7" t="n">
         <v>1934</v>
       </c>
-      <c r="B48" s="7" t="s">
+      <c r="B49" s="7" t="s">
         <v>400</v>
       </c>
-      <c r="C48" s="7" t="s">
+      <c r="C49" s="7" t="s">
         <v>401</v>
       </c>
-      <c r="D48" s="8" t="s">
+      <c r="D49" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="E48" s="9" t="inlineStr">
+      <c r="E49" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Enrique_Dussel"  title=" Wikipedia"&gt;Enrique DUSSEL&lt;/a&gt; était un philosophe argentin majeurs de la décolonialité et de la philosophie latino-américaine de la liberation.  Jeune intellectuel engagé dans les mouvements étudiants et opposé aux régimes autoritaires, il a été persécuté en Argentine avant de s’exiler au Mexique en 1975, où il a poursuivi sa carrière académique et développé sa pensée. Il élabore une &lt;a href="https://www.youtube.com/watch?v=QGPosp7lYlM" title="Enrique Dussel and the Philosophy of Liberation – Decolonizing Thought par Darina Metreveli"&gt;philosophie de la libération &lt;/a&gt; qui remet en question l’ontologie monologique de la modernité et introduit une approche éthique et alteritaire inspirée par Levinas, souvent décrite sous le nom d’analectique ou de dialectique positive. &lt;/p&gt; &lt;p&gt; Pionnier du décolonialisme latino-américain, il contribue à la construction des cadres Modernité/Colonialité et à l’idée d’une transmodernité, articulant critique de la modernité et invitation à repenser les rapports Nord-Sud et centre-périphérie. &lt;/p&gt; &lt;p&gt; Ses oeuvres majeures : &lt;a href="https://www.youtube.com/watch?v=nXNyqKCrKLY" title="Enrique Dussel, métaphysicien de la libération - Emmanuel Lévine par lundimatin"&gt;"Méthode pour une philosophie de la libération" &lt;/a&gt; paru en  1974 et "Filosofía ética latinoamericana" (période majeure)  posent les bases d’une philosophie enracinée dans les expériences des peuples opprimés et des contextes colonisés. &lt;/p&gt; &lt;p&gt; Il est reconnu dans les &lt;a href="https://lestempsquirestent.org/fr/numeros/numero-7/enrique-dussel-un-philosophe-indispensable-pour-decoloniser-la-theologie-politique" title="Enrique Dussel,
 un philosophe indispensable pour décoloniser la théologie politique par les temps qui restent"&gt;milieux décoloniaux &lt;/a&gt; et philosophie de la libération, mais demeure moins connu du grand public français, bien que des traductions et des analyses apparaissent et stimulent l’intérêt académique en France. Son travail nourrit le courant décolonial qui met en évidence l’interdépendance entre modernité et colonialité depuis 1492 et propose des axes pour une pensée transmoderne, dépassant les cadres classiques de la philosophie occidentale. &lt;/p&gt; </t>
         </is>
       </c>
-      <c r="F48" s="7" t="s">
+      <c r="F49" s="7" t="s">
         <v>404</v>
       </c>
-      <c r="G48" s="9" t="s">
+      <c r="G49" s="9" t="s">
         <v>405</v>
       </c>
-      <c r="H48" s="9" t="s">
+      <c r="H49" s="9" t="s">
         <v>406</v>
-      </c>
-      <c r="I48" s="9"/>
-      <c r="J48" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiers-mondisme ; Théologie de la libération ; Philosophie de la libération ; Pensée décoloniale</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="N48" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="O48" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="P48" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="240.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7" t="n">
-        <v>1934</v>
-      </c>
-      <c r="B49" s="7" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C49" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="D49" s="8" t="s">
-        <v>409</v>
-      </c>
-      <c r="E49" s="11" t="s">
-        <v>410</v>
-      </c>
-      <c r="F49" s="7" t="s">
-        <v>411</v>
-      </c>
-      <c r="G49" s="9" t="s">
-        <v>412</v>
-      </c>
-      <c r="H49" s="10" t="s">
-        <v>413</v>
       </c>
       <c r="I49" s="9"/>
       <c r="J49" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tiers-mondisme ; Théologie de la libération ; Philosophie de la libération ; Pensée décoloniale</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="N49" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O49" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="P49" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="240.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="7" t="n">
+        <v>1934</v>
+      </c>
+      <c r="B50" s="7" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="E50" s="11" t="s">
+        <v>410</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="G50" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="H50" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="I50" s="9"/>
+      <c r="J50" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="K49" s="2" t="s">
+      <c r="K50" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="L49" s="2" t="s">
+      <c r="L50" s="2" t="s">
         <v>415</v>
-      </c>
-      <c r="N49" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="240.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="1" t="n">
-        <v>1934</v>
-      </c>
-      <c r="B50" s="1" t="n">
-        <v>2019</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>417</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>418</v>
-      </c>
-      <c r="F50" s="1" t="s">
-        <v>419</v>
-      </c>
-      <c r="G50" s="15" t="s">
-        <v>420</v>
-      </c>
-      <c r="H50" s="2" t="s">
-        <v>421</v>
-      </c>
-      <c r="I50" s="1"/>
-      <c r="J50" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="K50" s="1" t="s">
-        <v>390</v>
-      </c>
-      <c r="L50" s="2" t="s">
-        <v>422</v>
-      </c>
-      <c r="M50" s="1" t="s">
-        <v>423</v>
       </c>
       <c r="N50" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="P50" s="1" t="s">
+    </row>
+    <row r="51" customFormat="false" ht="240.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1" t="n">
+        <v>1934</v>
+      </c>
+      <c r="B51" s="1" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="G51" s="15" t="s">
+        <v>420</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="I51" s="1"/>
+      <c r="J51" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="K51" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="L51" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="M51" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="N51" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="P51" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="XFC50" s="0"/>
-      <c r="XFD50" s="0"/>
-    </row>
-    <row r="51" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="16" t="n">
+      <c r="XFC51" s="0"/>
+      <c r="XFD51" s="0"/>
+    </row>
+    <row r="52" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="16" t="n">
         <v>1935</v>
       </c>
-      <c r="B51" s="16" t="n">
+      <c r="B52" s="16" t="n">
         <v>2003</v>
       </c>
-      <c r="C51" s="16" t="s">
+      <c r="C52" s="16" t="s">
         <v>425</v>
       </c>
-      <c r="D51" s="17" t="s">
+      <c r="D52" s="17" t="s">
         <v>426</v>
       </c>
-      <c r="E51" s="13" t="s">
+      <c r="E52" s="13" t="s">
         <v>427</v>
       </c>
-      <c r="F51" s="16" t="s">
+      <c r="F52" s="16" t="s">
         <v>428</v>
       </c>
-      <c r="G51" s="18" t="s">
+      <c r="G52" s="18" t="s">
         <v>429</v>
       </c>
-      <c r="H51" s="10" t="s">
+      <c r="H52" s="10" t="s">
         <v>430</v>
       </c>
-      <c r="I51" s="18"/>
-      <c r="J51" s="2" t="s">
+      <c r="I52" s="18"/>
+      <c r="J52" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="K51" s="2" t="s">
+      <c r="K52" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="L51" s="14" t="s">
+      <c r="L52" s="14" t="s">
         <v>432</v>
       </c>
-      <c r="M51" s="14" t="s">
+      <c r="M52" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="N51" s="14" t="s">
+      <c r="N52" s="14" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="7" t="n">
+    <row r="53" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="7" t="n">
         <v>1937</v>
       </c>
-      <c r="B52" s="7" t="s">
+      <c r="B53" s="7" t="s">
         <v>322</v>
       </c>
-      <c r="C52" s="7" t="s">
+      <c r="C53" s="7" t="s">
         <v>433</v>
       </c>
-      <c r="D52" s="8" t="s">
+      <c r="D53" s="8" t="s">
         <v>434</v>
       </c>
-      <c r="E52" s="11" t="s">
+      <c r="E53" s="11" t="s">
         <v>435</v>
       </c>
-      <c r="F52" s="7" t="s">
+      <c r="F53" s="7" t="s">
         <v>436</v>
       </c>
-      <c r="G52" s="9" t="s">
+      <c r="G53" s="9" t="s">
         <v>437</v>
       </c>
-      <c r="H52" s="10" t="s">
+      <c r="H53" s="10" t="s">
         <v>438</v>
-      </c>
-      <c r="I52" s="9"/>
-      <c r="J52" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="K52" s="2" t="s">
-        <v>439</v>
-      </c>
-      <c r="L52" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="N52" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="167.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7" t="n">
-        <v>1938</v>
-      </c>
-      <c r="B53" s="7" t="n">
-        <v>2002</v>
-      </c>
-      <c r="C53" s="7" t="s">
-        <v>441</v>
-      </c>
-      <c r="D53" s="8" t="s">
-        <v>442</v>
-      </c>
-      <c r="E53" s="13" t="s">
-        <v>443</v>
-      </c>
-      <c r="F53" s="7" t="s">
-        <v>444</v>
-      </c>
-      <c r="G53" s="9" t="s">
-        <v>445</v>
-      </c>
-      <c r="H53" s="10" t="s">
-        <v>446</v>
       </c>
       <c r="I53" s="9"/>
       <c r="J53" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="K53" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Libéralisme ; Minarchisme ; Déontologisme</t>
-        </is>
+        <v>127</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>439</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="M53" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="N53" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="N53" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="167.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="n">
         <v>1938</v>
       </c>
-      <c r="B54" s="7" t="s">
-        <v>449</v>
+      <c r="B54" s="7" t="n">
+        <v>2002</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>450</v>
+        <v>441</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>451</v>
-      </c>
-      <c r="E54" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Tom_Regan"  title=" Wikipedia"&gt;Tom REGAN&lt;/a&gt; était un philosophe américain   &lt;a href="https://www.youtube.com/watch?v=hgVMf3q4Vh4"  title=" Les animaux aussi ont une valeur. Valeur inhérente &amp; respect. - Tom Regan - Pensées antispécistes par The Critical Vegan"&gt;antispéciste &lt;/a&gt; influent dans le domaine de l'éthique animale, considéré comme un pionnier de la théorie des droits des animaux sur une base déontologique. Né à Pittsburgh, il enseigne de 1967 à 2001 à l’université d’État de Caroline du Nord. Il développe une approche abolitionniste opposée à l'utilitarisme de Peter Singer, arguant que les mammifères normaux d'un an ou plus sont des "sujets-d'une-vie" dotés d'une valeur inhérente, méritant des droits moraux fondamentaux indépendamment de leur utilité. Inspiré par Kant mais étendu aux non-humains, il définit ces sujets comme des êtres conscients pour qui leur vie importe intrinsèquement, justifiant l'interdiction absolue de l'exploitation. &lt;/p&gt; &lt;p&gt; Ses Œuvres principales sont : "The Case for Animal Rights" paru en 1983, traduit en français comme  &lt;a href="http://tomregan.free.fr/" title=" Les animaux aussi ont une valeur. Valeur inhérente &amp; respect. - Tom Regan - Les Droits des animaux par Tom Regan"&gt;"Les Droits des animaux" &lt;/a&gt; en 2013 : son magnum opus, salué comme un classique moderne critiquant Descartes et plaidant pour le "principe de respect" envers tout sujet-d'une-vie. "All That Dwell Therein" paru en  1982 : recueil d'essais sur le végétarisme et l'éthique animale. &lt;/p&gt; &lt;p&gt; Ses idées ont profondément marqué le mouvement des droits des animaux, influençant débats sur végétarisme, anti-vivisection et critique de l'environnementalisme indirect, tout en étant cité par des penseurs comme Derrida ou dans des ouvrages comme ceux de Jean-Baptiste Jeangène Vilmer. Dans &lt;em&gt;Empty Cages&lt;/em&gt; (2004), destiné au grand public, il résume son combat : il ne s’agit pas d’agrandir les cages, mais de les vider. &lt;/p&gt; </t>
-        </is>
+        <v>442</v>
+      </c>
+      <c r="E54" s="13" t="s">
+        <v>443</v>
       </c>
       <c r="F54" s="7" t="s">
-        <v>453</v>
+        <v>444</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>454</v>
-      </c>
-      <c r="H54" s="9" t="s">
-        <v>455</v>
+        <v>445</v>
+      </c>
+      <c r="H54" s="10" t="s">
+        <v>446</v>
       </c>
       <c r="I54" s="9"/>
       <c r="J54" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Libéralisme ; Minarchisme ; Déontologisme</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="M54" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="N54" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="7" t="n">
+        <v>1938</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>449</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="D55" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Tom_Regan"  title=" Wikipedia"&gt;Tom REGAN&lt;/a&gt; était un philosophe américain   &lt;a href="https://www.youtube.com/watch?v=hgVMf3q4Vh4"  title=" Les animaux aussi ont une valeur. Valeur inhérente &amp; respect. - Tom Regan - Pensées antispécistes par The Critical Vegan"&gt;antispéciste &lt;/a&gt; influent dans le domaine de l'éthique animale, considéré comme un pionnier de la théorie des droits des animaux sur une base déontologique. Né à Pittsburgh, il enseigne de 1967 à 2001 à l’université d’État de Caroline du Nord. Il développe une approche abolitionniste opposée à l'utilitarisme de Peter Singer, arguant que les mammifères normaux d'un an ou plus sont des "sujets-d'une-vie" dotés d'une valeur inhérente, méritant des droits moraux fondamentaux indépendamment de leur utilité. Inspiré par Kant mais étendu aux non-humains, il définit ces sujets comme des êtres conscients pour qui leur vie importe intrinsèquement, justifiant l'interdiction absolue de l'exploitation. &lt;/p&gt; &lt;p&gt; Ses Œuvres principales sont : "The Case for Animal Rights" paru en 1983, traduit en français comme  &lt;a href="http://tomregan.free.fr/" title=" Les animaux aussi ont une valeur. Valeur inhérente &amp; respect. - Tom Regan - Les Droits des animaux par Tom Regan"&gt;"Les Droits des animaux" &lt;/a&gt; en 2013 : son magnum opus, salué comme un classique moderne critiquant Descartes et plaidant pour le "principe de respect" envers tout sujet-d'une-vie. "All That Dwell Therein" paru en  1982 : recueil d'essais sur le végétarisme et l'éthique animale. &lt;/p&gt; &lt;p&gt; Ses idées ont profondément marqué le mouvement des droits des animaux, influençant débats sur végétarisme, anti-vivisection et critique de l'environnementalisme indirect, tout en étant cité par des penseurs comme Derrida ou dans des ouvrages comme ceux de Jean-Baptiste Jeangène Vilmer. Dans &lt;em&gt;Empty Cages&lt;/em&gt; (2004), destiné au grand public, il résume son combat : il ne s’agit pas d’agrandir les cages, mais de les vider. &lt;/p&gt; </t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="s">
+        <v>453</v>
+      </c>
+      <c r="G55" s="9" t="s">
+        <v>454</v>
+      </c>
+      <c r="H55" s="9" t="s">
+        <v>455</v>
+      </c>
+      <c r="I55" s="9"/>
+      <c r="J55" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="K54" s="2" t="s">
+      <c r="K55" s="2" t="s">
         <v>456</v>
       </c>
-      <c r="L54" s="2" t="s">
+      <c r="L55" s="2" t="s">
         <v>457</v>
-      </c>
-      <c r="N54" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="1" t="n">
-        <v>1940</v>
-      </c>
-      <c r="B55" s="1" t="n">
-        <v>2022</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>458</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Saul_Kripke"  title=" Wikipedia"&gt;Saul KRIPKE&lt;/a&gt; était un philosophe américain de la tradition analytique connu pour ses apports décisifs en logique modale, en métaphysique et en philosophie du langage. Très jeune, il révolutionne la logique en introduisant la sémantique des mondes possibles, aujourd’hui appelée &lt;a href="https://www.youtube.com/watch?v=_sIgAdvhruU"title="Qui est Saul Kripke ? par Monsieur Phi"&gt;"cadres de Kripke"&lt;/a&gt;, qui permet de formaliser la modalité (le nécessaire et le possible) de façon rigoureuse. &lt;/p&gt; &lt;p&gt; Son œuvre la plus influente est "Naming and Necessity", où il critique la conception descriptiviste des noms défendue par Frege et Russell. Selon lui, un  &lt;a href="https://www.youtube.com/watch?v=d7-8Avem7EE" title="Saul Kripke, La logique des noms propres. par Jtgrandtour"&gt; nom propre&lt;/a&gt; n’équivaut pas à une description mais fonctionne comme un « désignateur rigide » : il désigne le même individu dans tous les mondes possibles. Cette idée bouleverse la philosophie du langage et entraîne une redéfinition de la notion de référence.&lt;/p&gt; &lt;p&gt;  Il montre également qu’il existe des vérités nécessaires découvertes empiriquement : par exemple, l’identité « l’eau est H₂O » est nécessaire, mais nous ne l’avons apprise qu’a posteriori. Ce concept de nécessité a posteriori a marqué un tournant dans la métaphysique contemporaine. À l’inverse, il identifie la possibilité de certaines vérités contingentes connues a priori, ce qui remet en cause des distinctions classiques entre connaissance et modalité. &lt;/p&gt; &lt;p&gt; Il s’oppose au physicalisme en arguant que l’on peut concevoir un monde où tous les états cérébraux existent sans que la conscience subjective "le qualia" ne soit présente. Cette critique alimente encore aujourd’hui les débats sur la nature de la conscience. Son ouvrage "Wittgenstein on Rules and Private Language" propose une lecture radicale de Wittgenstein, selon laquelle toute règle est sujette à un scepticisme profond sur son application. Bien que controversée, cette interprétation a largement stimulé les discussions en philosophie du langage et en épistémologie. &lt;/p&gt; &lt;p&gt; Connu aussi pour son ouvrage " On two Paradoxes of Knowledge" et son  &lt;a href="https://www.youtube.com/watch?v=AzaUSC--2G0"  title="Le Paradoxe de l'Examen selon Saul Kripke par Silogic"&gt;"paradoxe de l'examen"&lt;/a&gt;. &lt;/p&gt; </t>
-        </is>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>461</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>462</v>
-      </c>
-      <c r="H55" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="J55" s="2" t="s">
-        <v>464</v>
-      </c>
-      <c r="K55" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="L55" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="M55" s="1" t="s">
-        <v>176</v>
       </c>
       <c r="N55" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="P55" s="1" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="7" t="n">
-        <v>1941</v>
-      </c>
-      <c r="B56" s="7" t="s">
-        <v>467</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>468</v>
-      </c>
-      <c r="D56" s="8" t="s">
-        <v>469</v>
-      </c>
-      <c r="E56" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/David_Lewis_(philosophe)"  title=" Wikipedia"&gt;David LEWIS&lt;/a&gt; était un philosophe américain connu pour sa théorie du  réalisme modal, selon laquelle il existe un nombre infini de mondes possibles concrets et causalement isolés les uns des autres. Son ouvrage majeur   &lt;a href="https://www.youtube.com/watch?v=-QlqLDLifuc" title="David Lewis - "De la pluralité des mondes" - De quoi parle ce livre ? par Philosophie 21"&gt;"On the Plurality of Worlds"&lt;/a&gt;  sortie en 1986, expose cette position révolutionnaire : pour lui, chaque monde possible existe aussi réellement que notre monde actuel, et sert à comprendre la modalité, c'est-à-dire ce qui pourrait être ou ce qui doit être. &lt;/p&gt; &lt;p&gt; Il a également proposé la théorie des contreparties en logique modale : au lieu de supposer que les personnes ou objets existent dans plusieurs mondes possibles, il affirme que chaque individu de notre monde a des « contreparties » dans les autres mondes possibles qui partagent certaines caractéristiques mais ne sont pas identiques à lui. Cette approche constitue une alternative à la logique modale traditionnelle, notamment celle de Saul Kripke. &lt;/p&gt; &lt;p&gt; Sa métaphysique est marquée par une conception atomiste (pointilliste) : la réalité n’est qu’une vaste mosaïque de faits locaux, chaque fait étant centré sur un « point » ayant des propriétés intrinsèques. Ce point de vue s’inspire de David Hume, d’où le nom « survenance humienne », refusant les liens nécessaires entre les faits et privilégiant une juxtaposition de qualités locales. &lt;/p&gt; &lt;p&gt; Il  a beaucoup écrit sur la philosophie du langage, la philosophie de l’esprit, l’épistémologie, la logique philosophique et la philosophie des mathématiques. Son premier grand ouvrage, "Convention" de 1969, analyse les conventions sociales à l’aide de la théorie des jeux, en montrant leur caractère arbitraire et leur diffusion par la connaissance commune et le précédent. Il s a marqué durablement la philosophie analytique.  &lt;a href="https://www.youtube.com/watch?v=g3jQwDP_Lyc" title="David Lewis - "David Lewis Speaks at La Trobe University par TimeSparrow"&gt;"Ses théories&lt;/a&gt; sont incontournables dans les débats sur les mondes possibles, la modalité, la causalité, la convention sociale, et l’atomisme métaphysique. Ses ouvrages, tels que Counterfactuals et Philosophical Papers, restent des références dans l’analyse logique et conceptuelle contemporaine. &lt;/p&gt; &lt;audio controls title=" On dit de David Lewis que c'est le plus grand métaphysicien qu’on ait vu depuis Leibniz par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/18292-28.02.2019-ITEMA_21995453-0.mp3" type="audio/mpeg" align="center"&gt;&lt;/audio&gt;  </t>
-        </is>
-      </c>
-      <c r="F56" s="7" t="s">
-        <v>471</v>
-      </c>
-      <c r="G56" s="9" t="s">
-        <v>472</v>
-      </c>
-      <c r="H56" s="9" t="s">
-        <v>473</v>
-      </c>
-      <c r="I56" s="9"/>
+    </row>
+    <row r="56" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="n">
+        <v>1940</v>
+      </c>
+      <c r="B56" s="1" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Saul_Kripke"  title=" Wikipedia"&gt;Saul KRIPKE&lt;/a&gt; était un philosophe américain de la tradition analytique connu pour ses apports décisifs en logique modale, en métaphysique et en philosophie du langage. Très jeune, il révolutionne la logique en introduisant la sémantique des mondes possibles, aujourd’hui appelée &lt;a href="https://www.youtube.com/watch?v=_sIgAdvhruU"title="Qui est Saul Kripke ? par Monsieur Phi"&gt;"cadres de Kripke"&lt;/a&gt;, qui permet de formaliser la modalité (le nécessaire et le possible) de façon rigoureuse. &lt;/p&gt; &lt;p&gt; Son œuvre la plus influente est "Naming and Necessity", où il critique la conception descriptiviste des noms défendue par Frege et Russell. Selon lui, un  &lt;a href="https://www.youtube.com/watch?v=d7-8Avem7EE" title="Saul Kripke, La logique des noms propres. par Jtgrandtour"&gt; nom propre&lt;/a&gt; n’équivaut pas à une description mais fonctionne comme un « désignateur rigide » : il désigne le même individu dans tous les mondes possibles. Cette idée bouleverse la philosophie du langage et entraîne une redéfinition de la notion de référence.&lt;/p&gt; &lt;p&gt;  Il montre également qu’il existe des vérités nécessaires découvertes empiriquement : par exemple, l’identité « l’eau est H₂O » est nécessaire, mais nous ne l’avons apprise qu’a posteriori. Ce concept de nécessité a posteriori a marqué un tournant dans la métaphysique contemporaine. À l’inverse, il identifie la possibilité de certaines vérités contingentes connues a priori, ce qui remet en cause des distinctions classiques entre connaissance et modalité. &lt;/p&gt; &lt;p&gt; Il s’oppose au physicalisme en arguant que l’on peut concevoir un monde où tous les états cérébraux existent sans que la conscience subjective "le qualia" ne soit présente. Cette critique alimente encore aujourd’hui les débats sur la nature de la conscience. Son ouvrage "Wittgenstein on Rules and Private Language" propose une lecture radicale de Wittgenstein, selon laquelle toute règle est sujette à un scepticisme profond sur son application. Bien que controversée, cette interprétation a largement stimulé les discussions en philosophie du langage et en épistémologie. &lt;/p&gt; &lt;p&gt; Connu aussi pour son ouvrage " On two Paradoxes of Knowledge" et son  &lt;a href="https://www.youtube.com/watch?v=AzaUSC--2G0"  title="Le Paradoxe de l'Examen selon Saul Kripke par Silogic"&gt;"paradoxe de l'examen"&lt;/a&gt;. &lt;/p&gt; </t>
+        </is>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>463</v>
+      </c>
       <c r="J56" s="2" t="s">
-        <v>474</v>
-      </c>
-      <c r="K56" s="2" t="s">
-        <v>475</v>
+        <v>464</v>
+      </c>
+      <c r="K56" s="1" t="s">
+        <v>465</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>476</v>
+        <v>466</v>
+      </c>
+      <c r="M56" s="1" t="s">
+        <v>176</v>
       </c>
       <c r="N56" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="57" customFormat="false" ht="332.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P56" s="1" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="n">
+        <v>1941</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>468</v>
+      </c>
+      <c r="D57" s="8" t="s">
+        <v>469</v>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/David_Lewis_(philosophe)"  title=" Wikipedia"&gt;David LEWIS&lt;/a&gt; était un philosophe américain connu pour sa théorie du  réalisme modal, selon laquelle il existe un nombre infini de mondes possibles concrets et causalement isolés les uns des autres. Son ouvrage majeur   &lt;a href="https://www.youtube.com/watch?v=-QlqLDLifuc" title="David Lewis - "De la pluralité des mondes" - De quoi parle ce livre ? par Philosophie 21"&gt;"On the Plurality of Worlds"&lt;/a&gt;  sortie en 1986, expose cette position révolutionnaire : pour lui, chaque monde possible existe aussi réellement que notre monde actuel, et sert à comprendre la modalité, c'est-à-dire ce qui pourrait être ou ce qui doit être. &lt;/p&gt; &lt;p&gt; Il a également proposé la théorie des contreparties en logique modale : au lieu de supposer que les personnes ou objets existent dans plusieurs mondes possibles, il affirme que chaque individu de notre monde a des « contreparties » dans les autres mondes possibles qui partagent certaines caractéristiques mais ne sont pas identiques à lui. Cette approche constitue une alternative à la logique modale traditionnelle, notamment celle de Saul Kripke. &lt;/p&gt; &lt;p&gt; Sa métaphysique est marquée par une conception atomiste (pointilliste) : la réalité n’est qu’une vaste mosaïque de faits locaux, chaque fait étant centré sur un « point » ayant des propriétés intrinsèques. Ce point de vue s’inspire de David Hume, d’où le nom « survenance humienne », refusant les liens nécessaires entre les faits et privilégiant une juxtaposition de qualités locales. &lt;/p&gt; &lt;p&gt; Il  a beaucoup écrit sur la philosophie du langage, la philosophie de l’esprit, l’épistémologie, la logique philosophique et la philosophie des mathématiques. Son premier grand ouvrage, "Convention" de 1969, analyse les conventions sociales à l’aide de la théorie des jeux, en montrant leur caractère arbitraire et leur diffusion par la connaissance commune et le précédent. Il s a marqué durablement la philosophie analytique.  &lt;a href="https://www.youtube.com/watch?v=g3jQwDP_Lyc" title="David Lewis - "David Lewis Speaks at La Trobe University par TimeSparrow"&gt;"Ses théories&lt;/a&gt; sont incontournables dans les débats sur les mondes possibles, la modalité, la causalité, la convention sociale, et l’atomisme métaphysique. Ses ouvrages, tels que Counterfactuals et Philosophical Papers, restent des références dans l’analyse logique et conceptuelle contemporaine. &lt;/p&gt; &lt;audio controls title=" On dit de David Lewis que c'est le plus grand métaphysicien qu’on ait vu depuis Leibniz par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/18292-28.02.2019-ITEMA_21995453-0.mp3" type="audio/mpeg" align="center"&gt;&lt;/audio&gt;  </t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="s">
+        <v>471</v>
+      </c>
+      <c r="G57" s="9" t="s">
+        <v>472</v>
+      </c>
+      <c r="H57" s="9" t="s">
+        <v>473</v>
+      </c>
+      <c r="I57" s="9"/>
+      <c r="J57" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="L57" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="N57" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="332.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="7" t="n">
         <v>1942</v>
       </c>
-      <c r="B57" s="7" t="s">
+      <c r="B58" s="7" t="s">
         <v>322</v>
       </c>
-      <c r="C57" s="7" t="s">
+      <c r="C58" s="7" t="s">
         <v>477</v>
       </c>
-      <c r="D57" s="8" t="s">
+      <c r="D58" s="8" t="s">
         <v>478</v>
       </c>
-      <c r="E57" s="9" t="inlineStr">
+      <c r="E58" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Daniel_Dennett"  style="color:#6A142A"  title=" Wikipedia"&gt;Daniel DENNETT&lt;/a&gt; était un  philosophe américain, figure importante et  influente de la philosophie de l'esprit, de la biologie et des sciences cognitives. Ses travaux se caractérisent par une volonté d'intégrer les découvertes scientifiques (biologie évolutionniste, neurosciences, intelligence artificielle) à la réflexion philosophique, souvent pour démanteler des intuitions traditionnelles qu'il juge erronées. &lt;/p&gt; &lt;p&gt; La Théorie de l'Esprit comme &lt;a href="https://www.youtube.com/watch?v=LKJJpvdqkFA" style="color:#88A1E9" title="Cette histoire va vous retourner le cerveau. | "Où suis-je" de Daniel Dennett par Monsieur Phi"&gt;"Position Intentionnelle"&lt;/a&gt; est sa contribution majeure. Il propose que pour prédire et expliquer le comportement d'un système (qu'il s'agisse d'un humain, d'un animal, d'un ordinateur ou même d'un thermostat), nous pouvons adopter trois "stances" : &lt;/p&gt; &lt;p&gt;La stance physique : On décrit le système par sa physique et sa chimie. Très difficile pour des systèmes complexes. &lt;/p&gt; &lt;p&gt;La stance du design : On considère le système comme conçu pour une fonction spécifique (ex: "ce thermostat est fait pour réguler la température"). &lt;/p&gt; &lt;p&gt;La stance intentionnelle : On traite le système comme s'il avait des croyances, des désirs et une rationalité. C'est une stratégie de prédiction extrêmement efficace, même si les croyances et désirs ne sont pas "réels" au sens littéral. Pour lui, avoir des croyances, c'est être un système dont le comportement peut être prédit avec succès par la stance intentionnelle. &lt;/p&gt; &lt;p&gt; Il est un matérialiste farouche et  rejette l'idée d'un &lt;a href="https://www.nonfiction.fr/article-1116-daniel_dennett_est_il_le_diable_.htm" title="Daniel Dennett est-il le diable ? par nonfiction"&gt;"théâtre cartésien"&lt;/a&gt;, un endroit dans le cerveau où tout se réunirait pour être "vu" par un &lt;a href="https://www.youtube.com/watch?v=0It9fwSj6xM"  title="Le moi comme illusion (Daniel Dennett, la conscience expliquée 4) par Philosophie Analytique"&gt;"spectateur" (le soi)&lt;/a&gt;. Pour lui, c'est une illusion.
 Il défend plutôt un modèle de "espace de travail global" : la conscience émerge de processus cérébraux parallèles et compétitifs. Une information devient "consciente" lorsqu'elle gagne une compétition pour être diffusée à grande échelle dans le cerveau, rendant ainsi disponible pour d'autres systèmes (mémoire, langage, prise de décision). Il n'y a pas de "centre" unique. &lt;/p&gt; &lt;p&gt; Il  considère que l'idée de la sélection naturelle de Darwin est "l'idée la plus dangereuse de tous les temps" car elle a un pouvoir explicatif immense, bien au-delà de la biologie. Il l'étend à d'autres domaines grâce au concept de "mèmes" (introduit par Richard Dawkins).
 Les mèmes sont des unités de culture (idées, mélodies, modes, concepts) qui se répliquent, mutent et sont sélectionnées dans le "payage" des esprits humains. Le langage,&lt;a href="https://www.youtube.com/shorts/bG3YBavy29Y" title="Cette histoire va vous retourner le cerveau | Daniel Dennett par StopCroyance"&gt; la religion&lt;/a&gt;, la morale peuvent être analysés comme des produits d'un processus darwinien. &lt;/p&gt; &lt;p&gt; Il défend une forme de libre arbitre qu'il estime compatible avec le déterminisme scientifique (le fait que l'univers soit régi par des lois causales). Pour lui, le libre arbitre n'est pas une "causalité magique" qui échapperait aux lois de la nature.  C'est la capacité d'un agent complexe (comme un être humain) à se projeter dans le futur, à évaluer les conséquences de ses actes et à agir en fonction de ses raisons. Ce libre arbitre est le produit de l'évolution et de la culture. Il est réel et précieux, même s'il n'est pas "libre" au sens d'une exemption des lois de la physique. &lt;/p&gt; &lt;audio controls title=" "Daniel Dennett, le penseur qui a révolutionné la philosophie des sciences et de l’esprit" par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/24419-10.05.2024-ITEMA_23737219-2024C51851S0131-21.mp3" type="audio/mpeg" align="center"&gt;&lt;/audio&gt; </t>
         </is>
       </c>
-      <c r="F57" s="7" t="s">
+      <c r="F58" s="7" t="s">
         <v>480</v>
       </c>
-      <c r="G57" s="9" t="s">
+      <c r="G58" s="9" t="s">
         <v>481</v>
       </c>
-      <c r="H57" s="9" t="s">
+      <c r="H58" s="9" t="s">
         <v>482</v>
       </c>
-      <c r="I57" s="9"/>
-      <c r="J57" s="2" t="s">
+      <c r="I58" s="9"/>
+      <c r="J58" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="K57" s="2" t="s">
+      <c r="K58" s="2" t="s">
         <v>483</v>
       </c>
-      <c r="L57" s="2" t="s">
+      <c r="L58" s="2" t="s">
         <v>484</v>
       </c>
-      <c r="N57" s="1" t="s">
+      <c r="N58" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="207" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="7" t="n">
+    <row r="59" customFormat="false" ht="207" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="7" t="n">
         <v>1943</v>
       </c>
-      <c r="B58" s="7" t="s">
+      <c r="B59" s="7" t="s">
         <v>449</v>
       </c>
-      <c r="C58" s="7" t="s">
+      <c r="C59" s="7" t="s">
         <v>485</v>
       </c>
-      <c r="D58" s="8" t="inlineStr">
+      <c r="D59" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Marilyn MCCORD-ADAMS</t>
         </is>
       </c>
-      <c r="E58" s="11" t="inlineStr">
+      <c r="E59" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Marilyn_McCord_Adams" title=" Wikipedia"&gt;Marilyn McCORD ADAMS&lt;/a&gt; était une philosophe américaine et une théologienne anglicane, reconnue pour son travail en philosophie de la religion et en philosophie médiévale. Elle a aussi été ordonnée prêtre épiscopalienne, ce qui donnait à sa réflexion philosophique une forte dimension spirituelle et pastorale. Elle a étudié à l’Université de l’Illinois puis à Cornell, où elle a obtenu son doctorat en philosophie en 1967. Sa carrière universitaire l’a menée à Michigan, UCLA, Yale, Oxford et elle a été la première femme, ainsi que la première Américaine, à occuper la chaire Regius de divinité à Oxford. &lt;/p&gt; &lt;p&gt;  &lt;a href="https://senate.universityofcalifornia.edu/in-memoriam/files/marilyn-adams.html" title="Marilyn Adans par university of california"&gt;Son apport le plus célèbre &lt;/a&gt; concerne l’étude de Guillaume d’Ockham, à qui elle a consacré une grande étude en deux volumes qui a beaucoup compté dans les recherches sur la théologie médiévale. Elle a aussi travaillé sur l’eucharistie, le christologie et d’autres auteurs médiévaux comme Thomas d’Aquin, Gilles de Rome et Duns Scot. &lt;/p&gt; &lt;p&gt; En  &lt;a href="https://www.youtube.com/watch?v=nFRGDG__ELM" title="Marilyn Adans par Real Atheology"&gt;philosophie de la religion, &lt;/a&gt; elle est connue pour ses analyses du mal extrême, qu’elle appelait les horrendous evils. Son idée centrale est qu’une théologie sérieuse doit prendre au sérieux les souffrances qui semblent détruire toute possibilité de sens, et montrer comment elles peuvent malgré tout être intégrées dans une vision de la bonté divine. &lt;/p&gt; &lt;p&gt; Son œuvre a eu une influence durable parce qu’elle relie la rigueur philosophique, l’érudition médiévale et l’expérience religieuse vécue. Elle reste une figure majeure pour comprendre à la fois la philosophie analytique de la religion et la redécouverte moderne de la pensée médiévale. &lt;/p&gt; 
 </t>
         </is>
       </c>
-      <c r="F58" s="7" t="s">
+      <c r="F59" s="7" t="s">
         <v>488</v>
       </c>
-      <c r="G58" s="9" t="s">
+      <c r="G59" s="9" t="s">
         <v>489</v>
       </c>
-      <c r="H58" s="9" t="s">
+      <c r="H59" s="9" t="s">
         <v>490</v>
       </c>
-      <c r="I58" s="9"/>
-      <c r="J58" s="2" t="s">
+      <c r="I59" s="9"/>
+      <c r="J59" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="K58" s="2" t="s">
+      <c r="K59" s="2" t="s">
         <v>475</v>
       </c>
-      <c r="L58" s="2" t="s">
+      <c r="L59" s="2" t="s">
         <v>491</v>
       </c>
-      <c r="M58" s="1" t="s">
+      <c r="M59" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N58" s="1" t="s">
+      <c r="N59" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="1" t="n">
+    <row r="60" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1" t="n">
         <v>1949</v>
       </c>
-      <c r="B59" s="1" t="n">
+      <c r="B60" s="1" t="n">
         <v>2006</v>
       </c>
-      <c r="C59" s="1" t="s">
+      <c r="C60" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="D59" s="1" t="s">
+      <c r="D60" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="E59" s="14" t="inlineStr">
+      <c r="E60" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Iris_Marion_Young" title=" Wikipedia"&gt;Iris Marion YOUNG&lt;/a&gt; était une philosophe politique américaine majeure, figure centrale du féminisme contemporain et de la théorie de la justice. Professeure à l'Université de Chicago, elle articule phénoménologie existentialiste, marxisme, théorie critique et postmodernisme pour repenser l'oppression, la domination et la démocratie au-delà des approches universalistes traditionnelles. &lt;/p&gt; &lt;p&gt; Sa contribution la plus célèbre est sa théorie des &lt;a href="https://www.youtube.com/watch?v=KyOut8zqJRI" title="les cinq visages de l’oppression par Eliot Goodine"&gt; cinq visages de l'oppression,&lt;/a&gt;  qu'elle développe dans Justice and the Politics of Difference (1990) ou elle développe également une,&lt;a href="https://www.persee.fr/doc/phlou_0035-3841_2018_num_116_4_8681" title="le féminisme phénoménologique par persée"&gt; phénoménologie féministe &lt;/a&gt; du corps, notamment dans son essai célèbre « Throwing Like a Girl » (1980). Elle y décrit comment les femmes vivent leur corps comme limité, fragmenté et constamment surveillé, ce qui produit une « immanence » sociale qui entrave leur capacité d'action et d'autodétermination. Le corps n'est pas seulement biologique mais politique, façonné par les normes sociales et les rapports de pouvoir. &lt;/p&gt; &lt;p&gt; Elle défend une conception de la justice fondée sur l'inclusion différenciée plutôt que sur l'universalisme abstrait. Pour Young, une société juste doit reconnaître les différences de groupe (genre, race, classe, sexualité) et créer des espaces où chacun puisse participer à la vie démocratique sans être forcé d'abandonner son identité particulière. Elle propose aussi le concept de responsabilité sociale diffuse, selon lequel tous les membres d'une société sont responsables des injustice structurelles, pas seulement les auteurs directs. &lt;/p&gt; &lt;p&gt; Elle évite tout essentialisme en conceptualisant « les femmes » comme un groupe social sériel, au sens de Sartre : un groupe dont les membres ne partagent pas une essence commune mais sont reliés par des conditions sociales similaires et des rapports de pouvoir. Cette approche permet un féminisme pluriel, Alliant diverses luttes (racisme, homophobie, validisme, écologie) dans des coalitions contre les rapports de domination. &lt;/p&gt; 
 </t>
         </is>
       </c>
-      <c r="F59" s="1" t="s">
+      <c r="F60" s="1" t="s">
         <v>495</v>
       </c>
-      <c r="G59" s="2" t="s">
+      <c r="G60" s="2" t="s">
         <v>496</v>
       </c>
-      <c r="H59" s="2" t="s">
+      <c r="H60" s="2" t="s">
         <v>497</v>
       </c>
-      <c r="J59" s="2" t="s">
+      <c r="J60" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="K59" s="2" t="s">
+      <c r="K60" s="2" t="s">
         <v>498</v>
       </c>
-      <c r="L59" s="2" t="s">
+      <c r="L60" s="2" t="s">
         <v>499</v>
       </c>
-      <c r="M59" s="1" t="s">
+      <c r="M60" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N59" s="1" t="s">
+      <c r="N60" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="1" t="n">
+    <row r="61" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="n">
         <v>1952</v>
       </c>
-      <c r="B60" s="1" t="n">
+      <c r="B61" s="1" t="n">
         <v>2021</v>
       </c>
-      <c r="C60" s="1" t="s">
+      <c r="C61" s="1" t="s">
         <v>500</v>
       </c>
-      <c r="D60" s="1" t="s">
+      <c r="D61" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Bell_hooks"  title=" Wikipedia"&gt;Bell HOOKS&lt;/a&gt;, de son vrai nom Gloria Jean Watkins, est une autrice, professeure et militante féministe afro-américaine. Née dans le Kentucky, dans le Sud ségrégationniste, elle prit le nom de son arrière-grand-mère, qu'elle écrivait en minuscules pour que l'attention se porte sur ses idées plutôt que sur sa personne.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Ne suis-je pas une femme ?&lt;/em&gt; (1981), elle montre que les femmes noires ont été oubliées à la fois par le mouvement féministe, dominé par des femmes blanches de classe moyenne, et par le mouvement pour les droits civiques, dominé par des hommes. Elle  &lt;a href="https://www.youtube.com/watch?v=pCwMdHBSQgM" title=" bell hooks, un féminisme anticapitaliste et intersectionnel par META "&gt;développe l'idée &lt;/a&gt; que le sexisme, le racisme et l'exploitation économique forment un même système de domination, qu'elle appelle le « patriarcat capitaliste suprémaciste blanc ».&lt;/p&gt; &lt;p&gt;Ses idées ont profondément influencé ce que l'on appelle aujourd'hui l'intersectionnalité, c'est-à-dire l'étude de la manière dont différentes formes de discrimination se croisent et se renforcent. Elle écrivait dans un style simple et direct, refusant le jargon universitaire, pour que ses livres soient lus au-delà des cercles savants. Elle a aussi consacré plusieurs ouvrages à l'amour, qu'elle considérait comme une force politique capable de transformer la société.&lt;/p&gt; &lt;p&gt;Elle a écrit une quarantaine de livres, sur le féminisme, l'amour, les médias, la culture populaire et l'éducation. Dans &lt;em&gt;Apprendre à transgresser&lt;/em&gt; (1994), inspirée par Paulo Freire, elle défend une pédagogie de la liberté où l'enseignement devient une pratique d'émancipation. Pour elle, le féminisme n'est pas une guerre contre les hommes mais un mouvement pour mettre fin à toute forme de domination, porté par une « éthique de l'amour ».&lt;/p&gt;    &lt;audio controls title="Lire bell hooks aujourd’hui par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/23875-15.11.2023-ITEMA_23552434-2023C49162S0319-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;  
 </t>
         </is>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="F61" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="G60" s="2" t="s">
+      <c r="G61" s="2" t="s">
         <v>504</v>
       </c>
-      <c r="H60" s="2" t="s">
+      <c r="H61" s="2" t="s">
         <v>505</v>
       </c>
-      <c r="I60" s="1"/>
-      <c r="J60" s="2" t="s">
+      <c r="I61" s="1"/>
+      <c r="J61" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="K60" s="1" t="inlineStr">
+      <c r="K61" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Féminisme ; Wokisme</t>
         </is>
       </c>
-      <c r="L60" s="2" t="s">
+      <c r="L61" s="2" t="s">
         <v>507</v>
       </c>
-      <c r="M60" s="1" t="s">
+      <c r="M61" s="1" t="s">
         <v>508</v>
       </c>
-      <c r="N60" s="1" t="s">
+      <c r="N61" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="O60" s="1" t="n">
+      <c r="O61" s="1" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="293.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="0">
+    <row r="62" customFormat="false" ht="293.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="0">
         <v>1535</v>
       </c>
-      <c r="B61" s="0" t="inlineStr">
+      <c r="B62" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">1616</t>
         </is>
       </c>
-      <c r="C61" s="0" t="inlineStr">
+      <c r="C62" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">vers 1535 – vers 1616</t>
         </is>
       </c>
-      <c r="D61" s="0" t="inlineStr">
+      <c r="D62" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Felipe GUAMÁN POMA de Ayala</t>
         </is>
       </c>
-      <c r="E61" s="0" t="inlineStr">
+      <c r="E62" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Felipe_Guam%C3%A1n_Poma_de_Ayala" title=" Wikipedia"&gt;Felipe GUAMÁN POMA de Ayala&lt;/a&gt; est un noble andin de langue quechua, auteur de l’un des documents les plus extraordinaires de l’époque coloniale. Né dans la province de Lucanas, au Pérou, peu après la conquête espagnole, il descend par sa mère d’une lignée liée aux souverains de l’&lt;a href="https://fr.wikipedia.org/wiki/Empire_inca" title=" Wikipedia"&gt;Empire inca&lt;/a&gt;. Élevé parmi les Espagnols, il apprend leur langue, se fait chrétien et travaille comme interprète auprès d’un prêtre chargé d’extirper les « idolâtries », puis auprès de juges de Huamanga, avant d’être dépouillé de ses terres et banni vers 1600.&lt;/p&gt; &lt;p&gt;Il parcourt alors les Andes pendant des années et rédige, vers 1615, une lettre de près de 1 200 pages adressée au roi d’Espagne Philippe III : la &lt;em&gt;Nouvelle Chronique et bon gouvernement&lt;/em&gt;. Ses quelque 400 dessins à la plume racontent l’histoire des Incas, le calendrier, les travaux des champs, puis les abus des colons : prêtres, corregidors et propriétaires qui exploitent, volent et maltraitent les Indiens. Il y décrit un « monde à l’envers » (&lt;em&gt;mundo al revés&lt;/em&gt;), où l’ordre juste a été renversé par la conquête.&lt;/p&gt; &lt;p&gt;Il ne réclame pas le départ des Espagnols, mais un « bon gouvernement » : que les Andins se gouvernent eux-mêmes sous l’autorité lointaine du roi, et que les colons qui abusent soient chassés des villages. Il défend aussi la valeur de la civilisation andine, qui connaissait selon lui la justice et un ordre moral bien avant l’arrivée des Européens. Le manuscrit, qui n’atteignit sans doute jamais le roi, dormit pendant trois siècles avant d’être découvert en 1908 à la Bibliothèque royale de Copenhague. Il est aujourd’hui une source majeure sur le monde andin et l’une des premières critiques de la colonisation écrites par un colonisé.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F61" s="0" t="inlineStr">
+      <c r="F62" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">__IaJh6gzA0</t>
         </is>
       </c>
-      <c r="G61" s="0" t="inlineStr">
+      <c r="G62" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">"📌Felipe Guamán Poma de Ayala: HISTORIA desde su mirada al mundo andino y la conquista española | EP1" par Gestión Mundo</t>
         </is>
       </c>
-      <c r="H61" s="0" t="inlineStr">
+      <c r="H62" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/guamanpoma-mini.webp</t>
         </is>
       </c>
-      <c r="I61" s="0"/>
-      <c r="J61" s="0" t="inlineStr">
+      <c r="I62" s="0"/>
+      <c r="J62" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">politique ; ethique</t>
         </is>
       </c>
-      <c r="K61" s="0" t="inlineStr">
+      <c r="K62" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Anticolonialisme</t>
         </is>
       </c>
-      <c r="L61" s="0" t="inlineStr">
+      <c r="L62" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">chroniqueur andin, auteur d’une immense lettre illustrée au roi d’Espagne dénonçant la colonisation du Pérou.</t>
         </is>
       </c>
-      <c r="M61" s="0"/>
-      <c r="N61" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sud</t>
-        </is>
-      </c>
-      <c r="O61" s="1">
-        <v>2</v>
-      </c>
-      <c r="P61" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Péruvienne</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="1">
-        <v>1853</v>
-      </c>
-      <c r="B62" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1895</t>
-        </is>
-      </c>
-      <c r="C62" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1853 – 1895</t>
-        </is>
-      </c>
-      <c r="D62" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">José MARTÍ</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jos%C3%A9_Mart%C3%AD" title=" Wikipedia"&gt;José MARTÍ&lt;/a&gt; est le grand penseur de l’indépendance cubaine et l’une des voix majeures de l’Amérique latine. Né à La Havane de parents espagnols, il est arrêté à seize ans pour ses idées indépendantistes et condamné aux travaux forcés dans une carrière, avant d’être déporté en Espagne, où il étudie le droit et la philosophie à Saragosse. Il vit ensuite au Mexique, au Guatemala et au Venezuela, puis s’installe en 1881 à New York, où il passe près de quinze ans comme journaliste, diplomate et organisateur de l’exil cubain. Il y écrit, pour de grands journaux d’Amérique latine, des chroniques sur la vie nord-américaine.&lt;/p&gt; &lt;p&gt;Dans son essai &lt;em&gt;Notre Amérique&lt;/em&gt; (1891), il appelle les nations latino-américaines à se penser à partir de leur propre réalité, métisse, indienne, noire et paysanne, plutôt qu’en copiant l’Europe ou les États-Unis : « Le gouvernement doit naître du pays. » Il y affirme aussi : « Il n’y a pas de haine des races, parce qu’il n’y a pas de races. » Observateur lucide de la puissance nord-américaine, il met en garde contre les ambitions des États-Unis sur Cuba et sur tout le continent.&lt;/p&gt; &lt;p&gt;Poète novateur, l’un des fondateurs du modernisme hispanique, il écrit les &lt;em&gt;Vers simples&lt;/em&gt; (1891), dont certains forment les paroles de la célèbre chanson &lt;em&gt;Guantanamera&lt;/em&gt;, et une revue pour les enfants, &lt;em&gt;L’Âge d’or&lt;/em&gt;. En 1892, il fonde le Parti révolutionnaire cubain et prépare la &lt;a href="https://fr.wikipedia.org/wiki/Guerre_d%27ind%C3%A9pendance_cubaine" title=" Wikipedia"&gt;guerre d’indépendance&lt;/a&gt;. Débarqué à Cuba avec les insurgés, il est tué au combat à Dos Ríos le 19 mai 1895. Il est considéré à Cuba comme le héros national et « l’Apôtre » de l’indépendance.&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">l5bN92K18g8</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"Filosofia Aquí y Ahora IV 5: El Pensamiento de José Martí" par Argen-Man</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/marti-mini.webp</t>
-        </is>
-      </c>
-      <c r="I62" s="1"/>
-      <c r="J62" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">politique ; esthetique</t>
-        </is>
-      </c>
-      <c r="K62" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Anticolonialisme ; Humanisme</t>
-        </is>
-      </c>
-      <c r="L62" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">poète et penseur de l’indépendance cubaine, auteur de « Notre Amérique », héros national de Cuba.</t>
-        </is>
-      </c>
+      <c r="M62" s="0"/>
       <c r="N62" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">sud</t>
@@ -5030,64 +5026,65 @@
       <c r="O62" s="1">
         <v>2</v>
       </c>
-      <c r="P62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cubaine</t>
+      <c r="P62" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Péruvienne</t>
         </is>
       </c>
     </row>
     <row r="63" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1">
-        <v>1921</v>
+        <v>1853</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1997</t>
+          <t xml:space="preserve">1895</t>
         </is>
       </c>
       <c r="C63" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1921 – 1997</t>
+          <t xml:space="preserve">1853 – 1895</t>
         </is>
       </c>
       <c r="D63" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paulo FREIRE</t>
+          <t xml:space="preserve">José MARTÍ</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Paulo_Freire" title=" Wikipedia"&gt;Paulo FREIRE&lt;/a&gt; est un pédagogue et philosophe brésilien, l’un des penseurs de l’éducation les plus lus au monde. Né à Recife, dans le Nordeste, il connaît la faim pendant la crise des années 1930, ce qui le marque pour toute sa vie. Formé au droit et à la philosophie, lecteur de Marx comme des penseurs chrétiens, il se consacre à l’&lt;a href="https://fr.wikipedia.org/wiki/Alphab%C3%A9tisation" title=" Wikipedia"&gt;alphabétisation&lt;/a&gt; des adultes pauvres. En 1963, à Angicos, sa méthode permet à 300 travailleurs agricoles d’apprendre à lire et à écrire en une quarantaine d’heures.&lt;/p&gt; &lt;p&gt;Sa méthode part des « mots générateurs » tirés de la vie des apprenants, comme la brique, la terre ou le salaire, et fait de la lecture une prise de conscience : apprendre à lire le mot, c’est apprendre à lire le monde. Après le coup d’État militaire de 1964, il est emprisonné puis contraint à un exil de seize ans. Au Chili, il écrit &lt;a href="https://fr.wikipedia.org/wiki/P%C3%A9dagogie_des_opprim%C3%A9s" title=" Wikipedia"&gt;&lt;em&gt;Pédagogie des opprimés&lt;/em&gt;&lt;/a&gt; (1968), où il critique l’éducation « bancaire », qui dépose des savoirs dans des élèves passifs comme on remplit un coffre, et lui oppose une éducation par le dialogue, où maître et élèves cherchent ensemble.&lt;/p&gt; &lt;p&gt;« Personne n’éduque autrui, personne ne s’éduque seul, les hommes s’éduquent ensemble par l’intermédiaire du monde. » L’éducation n’est jamais neutre : elle maintient l’oppression ou aide les opprimés à s’en libérer, sans devenir à leur tour oppresseurs. Rentré au Brésil en 1980, il dirige l’éducation de la ville de São Paulo. Son œuvre est à l’origine de la &lt;a href="https://fr.wikipedia.org/wiki/P%C3%A9dagogie_critique" title=" Wikipedia"&gt;pédagogie critique&lt;/a&gt;, et il a été proclamé en 2012 patron de l’éducation brésilienne.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jos%C3%A9_Mart%C3%AD" title=" Wikipedia"&gt;José MARTÍ&lt;/a&gt; est le grand penseur de l’indépendance cubaine et l’une des voix majeures de l’Amérique latine. Né à La Havane de parents espagnols, il est arrêté à seize ans pour ses idées indépendantistes et condamné aux travaux forcés dans une carrière, avant d’être déporté en Espagne, où il étudie le droit et la philosophie à Saragosse. Il vit ensuite au Mexique, au Guatemala et au Venezuela, puis s’installe en 1881 à New York, où il passe près de quinze ans comme journaliste, diplomate et organisateur de l’exil cubain. Il y écrit, pour de grands journaux d’Amérique latine, des chroniques sur la vie nord-américaine.&lt;/p&gt; &lt;p&gt;Dans son essai &lt;em&gt;Notre Amérique&lt;/em&gt; (1891), il appelle les nations latino-américaines à se penser à partir de leur propre réalité, métisse, indienne, noire et paysanne, plutôt qu’en copiant l’Europe ou les États-Unis : « Le gouvernement doit naître du pays. » Il y affirme aussi : « Il n’y a pas de haine des races, parce qu’il n’y a pas de races. » Observateur lucide de la puissance nord-américaine, il met en garde contre les ambitions des États-Unis sur Cuba et sur tout le continent.&lt;/p&gt; &lt;p&gt;Poète novateur, l’un des fondateurs du modernisme hispanique, il écrit les &lt;em&gt;Vers simples&lt;/em&gt; (1891), dont certains forment les paroles de la célèbre chanson &lt;em&gt;Guantanamera&lt;/em&gt;, et une revue pour les enfants, &lt;em&gt;L’Âge d’or&lt;/em&gt;. En 1892, il fonde le Parti révolutionnaire cubain et prépare la &lt;a href="https://fr.wikipedia.org/wiki/Guerre_d%27ind%C3%A9pendance_cubaine" title=" Wikipedia"&gt;guerre d’indépendance&lt;/a&gt;. Débarqué à Cuba avec les insurgés, il est tué au combat à Dos Ríos le 19 mai 1895. Il est considéré à Cuba comme le héros national et « l’Apôtre » de l’indépendance.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t xml:space="preserve">4FG6diR6fhU</t>
+          <t xml:space="preserve">l5bN92K18g8</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Une pédagogie pour éduquer au politique, contre l'oppression ? Paulo FREIRE - selon Philippe Meirieu" par Benoit Urgelli</t>
+          <t xml:space="preserve">"Filosofia Aquí y Ahora IV 5: El Pensamiento de José Martí" par Argen-Man</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/freire-mini.webp</t>
-        </is>
-      </c>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/marti-mini.webp</t>
+        </is>
+      </c>
+      <c r="I63" s="1"/>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ethique ; politique</t>
+          <t xml:space="preserve">politique ; esthetique</t>
         </is>
       </c>
       <c r="K63" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Humanisme ; Marxisme ; Théologie de la libération</t>
+          <t xml:space="preserve">Anticolonialisme ; Humanisme</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">pédagogue brésilien, auteur de Pédagogie des opprimés, penseur de l’éducation comme pratique de la liberté.</t>
+          <t xml:space="preserve">poète et penseur de l’indépendance cubaine, auteur de « Notre Amérique », héros national de Cuba.</t>
         </is>
       </c>
       <c r="N63" s="1" t="inlineStr">
@@ -5096,66 +5093,66 @@
         </is>
       </c>
       <c r="O63" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brésilienne</t>
+          <t xml:space="preserve">Cubaine</t>
         </is>
       </c>
     </row>
     <row r="64" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1">
-        <v>1882</v>
+        <v>1921</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1959</t>
+          <t xml:space="preserve">1997</t>
         </is>
       </c>
       <c r="C64" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1882 – 1959</t>
+          <t xml:space="preserve">1921 – 1997</t>
         </is>
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">José VASCONCELOS</t>
+          <t xml:space="preserve">Paulo FREIRE</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jos%C3%A9_Vasconcelos" title=" Wikipedia"&gt;José VASCONCELOS&lt;/a&gt; est un philosophe, écrivain et homme politique mexicain, l’un des grands éducateurs de l’Amérique latine. Né à Oaxaca, avocat, il fonde en 1909 avec Antonio Caso et Alfonso Reyes l’Ateneo de la Juventud, cercle de jeunes intellectuels qui rejette le positivisme officiel du régime de Porfirio Díaz. Il prend part à la &lt;a href="https://fr.wikipedia.org/wiki/R%C3%A9volution_mexicaine" title=" Wikipedia"&gt;révolution mexicaine&lt;/a&gt; aux côtés de Francisco Madero. Recteur de l’université nationale en 1920, il lui donne sa devise, toujours en usage : « Par ma race parlera l’esprit. »&lt;/p&gt; &lt;p&gt;Ministre de l’Éducation de 1921 à 1924, il mène une véritable croisade pour instruire le peuple : écoles rurales, missions culturelles dans les villages, bibliothèques, éditions populaires des grands classiques. Il commande aussi aux peintres &lt;a href="https://fr.wikipedia.org/wiki/Diego_Rivera" title=" Wikipedia"&gt;Diego Rivera&lt;/a&gt; et José Clemente Orozco les fresques murales qui racontent l’histoire du Mexique sur les murs des bâtiments publics. Il est surnommé le « maître de la jeunesse d’Amérique ».&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;La Race cosmique&lt;/em&gt; (1925), il prophétise que l’Amérique latine, terre de tous les mélanges, verra naître une « cinquième race », synthèse de toutes les autres, porteuse d’une civilisation de l’amour et de la beauté. Sa philosophie, un « monisme esthétique », voit dans l’émotion esthétique la forme la plus haute de connaissance. Battu en 1929 dans une élection présidentielle qu’il juge truquée, il s’exile, puis évolue vers un conservatisme catholique, au point de manifester en 1940 des sympathies pour l’Allemagne nazie. Il meurt à Mexico en 1959.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Paulo_Freire" title=" Wikipedia"&gt;Paulo FREIRE&lt;/a&gt; est un pédagogue et philosophe brésilien, l’un des penseurs de l’éducation les plus lus au monde. Né à Recife, dans le Nordeste, il connaît la faim pendant la crise des années 1930, ce qui le marque pour toute sa vie. Formé au droit et à la philosophie, lecteur de Marx comme des penseurs chrétiens, il se consacre à l’&lt;a href="https://fr.wikipedia.org/wiki/Alphab%C3%A9tisation" title=" Wikipedia"&gt;alphabétisation&lt;/a&gt; des adultes pauvres. En 1963, à Angicos, sa méthode permet à 300 travailleurs agricoles d’apprendre à lire et à écrire en une quarantaine d’heures.&lt;/p&gt; &lt;p&gt;Sa méthode part des « mots générateurs » tirés de la vie des apprenants, comme la brique, la terre ou le salaire, et fait de la lecture une prise de conscience : apprendre à lire le mot, c’est apprendre à lire le monde. Après le coup d’État militaire de 1964, il est emprisonné puis contraint à un exil de seize ans. Au Chili, il écrit &lt;a href="https://fr.wikipedia.org/wiki/P%C3%A9dagogie_des_opprim%C3%A9s" title=" Wikipedia"&gt;&lt;em&gt;Pédagogie des opprimés&lt;/em&gt;&lt;/a&gt; (1968), où il critique l’éducation « bancaire », qui dépose des savoirs dans des élèves passifs comme on remplit un coffre, et lui oppose une éducation par le dialogue, où maître et élèves cherchent ensemble.&lt;/p&gt; &lt;p&gt;« Personne n’éduque autrui, personne ne s’éduque seul, les hommes s’éduquent ensemble par l’intermédiaire du monde. » L’éducation n’est jamais neutre : elle maintient l’oppression ou aide les opprimés à s’en libérer, sans devenir à leur tour oppresseurs. Rentré au Brésil en 1980, il dirige l’éducation de la ville de São Paulo. Son œuvre est à l’origine de la &lt;a href="https://fr.wikipedia.org/wiki/P%C3%A9dagogie_critique" title=" Wikipedia"&gt;pédagogie critique&lt;/a&gt;, et il a été proclamé en 2012 patron de l’éducation brésilienne.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t xml:space="preserve">B3E3RuPB9qY</t>
+          <t xml:space="preserve">4FG6diR6fhU</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t xml:space="preserve">"José Vasconcelos filosofía de México" par Filosofia Corporativa</t>
+          <t xml:space="preserve">"Une pédagogie pour éduquer au politique, contre l'oppression ? Paulo FREIRE - selon Philippe Meirieu" par Benoit Urgelli</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/vasconcelos-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/freire-mini.webp</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">esthetique ; politique</t>
+          <t xml:space="preserve">ethique ; politique</t>
         </is>
       </c>
       <c r="K64" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monisme ; Spiritualisme</t>
+          <t xml:space="preserve">Humanisme ; Marxisme ; Théologie de la libération</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe et ministre mexicain de l’Éducation, auteur de La Race cosmique, penseur du métissage.</t>
+          <t xml:space="preserve">pédagogue brésilien, auteur de Pédagogie des opprimés, penseur de l’éducation comme pratique de la liberté.</t>
         </is>
       </c>
       <c r="N64" s="1" t="inlineStr">
@@ -5164,76 +5161,71 @@
         </is>
       </c>
       <c r="O64" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mexicaine</t>
+          <t xml:space="preserve">Brésilienne</t>
         </is>
       </c>
     </row>
     <row r="65" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1">
-        <v>1907</v>
+        <v>1882</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1972</t>
+          <t xml:space="preserve">1959</t>
         </is>
       </c>
       <c r="C65" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1907 – 1972</t>
+          <t xml:space="preserve">1882 – 1959</t>
         </is>
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abraham Joshua HESCHEL</t>
+          <t xml:space="preserve">José VASCONCELOS</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Abraham_Joshua_Heschel" title=" Wikipedia"&gt;Abraham Joshua HESCHEL&lt;/a&gt; est un rabbin, théologien et philosophe juif, l’une des grandes voix religieuses du XXe siècle. Né à Varsovie dans une illustre famille du &lt;a href="https://fr.wikipedia.org/wiki/Hassidisme" title=" Wikipedia"&gt;hassidisme&lt;/a&gt;, il étudie la philosophie à Berlin, où il soutient une thèse sur les prophètes d’Israël. Expulsé d’Allemagne vers la Pologne en 1938, il parvient à quitter Varsovie quelques semaines avant l’invasion allemande et gagne Londres, puis les États-Unis. Sa mère et ses sœurs sont assassinées pendant la Shoah. Il enseigne à partir de 1946 au Séminaire théologique juif de New York.&lt;/p&gt; &lt;p&gt;Pour Heschel, la religion commence par l’« étonnement radical » devant le monde, qui précède toute réflexion. Contre l’idée d’un Dieu impassible des philosophes, il parle du « pathos divin » : le Dieu des prophètes est concerné par le sort des hommes et souffre de l’injustice. La question n’est pas seulement de savoir si l’homme cherche Dieu, mais de comprendre que &lt;em&gt;Dieu est en quête de l’homme&lt;/em&gt;, titre de son livre de 1955. Dans &lt;em&gt;Les Bâtisseurs du temps&lt;/em&gt; (1951), il présente le &lt;a href="https://fr.wikipedia.org/wiki/Shabbat" title=" Wikipedia"&gt;shabbat&lt;/a&gt; comme « une cathédrale dans le temps » : le judaïsme sanctifie des moments plutôt que des lieux. Il consacre aussi un grand livre aux prophètes, témoins de la passion de Dieu pour la justice.&lt;/p&gt; &lt;p&gt;Sa foi le conduit à l’action. En 1965, il marche de Selma à Montgomery aux côtés de Martin Luther King et dira : « J’avais l’impression que mes jambes priaient. » Il s’oppose à la guerre du Vietnam et contribue au dialogue entre juifs et chrétiens lors du concile Vatican II. Il meurt à New York en 1972.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jos%C3%A9_Vasconcelos" title=" Wikipedia"&gt;José VASCONCELOS&lt;/a&gt; est un philosophe, écrivain et homme politique mexicain, l’un des grands éducateurs de l’Amérique latine. Né à Oaxaca, avocat, il fonde en 1909 avec Antonio Caso et Alfonso Reyes l’Ateneo de la Juventud, cercle de jeunes intellectuels qui rejette le positivisme officiel du régime de Porfirio Díaz. Il prend part à la &lt;a href="https://fr.wikipedia.org/wiki/R%C3%A9volution_mexicaine" title=" Wikipedia"&gt;révolution mexicaine&lt;/a&gt; aux côtés de Francisco Madero. Recteur de l’université nationale en 1920, il lui donne sa devise, toujours en usage : « Par ma race parlera l’esprit. »&lt;/p&gt; &lt;p&gt;Ministre de l’Éducation de 1921 à 1924, il mène une véritable croisade pour instruire le peuple : écoles rurales, missions culturelles dans les villages, bibliothèques, éditions populaires des grands classiques. Il commande aussi aux peintres &lt;a href="https://fr.wikipedia.org/wiki/Diego_Rivera" title=" Wikipedia"&gt;Diego Rivera&lt;/a&gt; et José Clemente Orozco les fresques murales qui racontent l’histoire du Mexique sur les murs des bâtiments publics. Il est surnommé le « maître de la jeunesse d’Amérique ».&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;La Race cosmique&lt;/em&gt; (1925), il prophétise que l’Amérique latine, terre de tous les mélanges, verra naître une « cinquième race », synthèse de toutes les autres, porteuse d’une civilisation de l’amour et de la beauté. Sa philosophie, un « monisme esthétique », voit dans l’émotion esthétique la forme la plus haute de connaissance. Battu en 1929 dans une élection présidentielle qu’il juge truquée, il s’exile, puis évolue vers un conservatisme catholique, au point de manifester en 1940 des sympathies pour l’Allemagne nazie. Il meurt à Mexico en 1959.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t xml:space="preserve">SLINbVsBz-Q</t>
+          <t xml:space="preserve">B3E3RuPB9qY</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t xml:space="preserve">"LA PENSEE D'AVRAHAM YOSHOUA HESCHEL" Rony Akrich"" par רוני אקריש</t>
+          <t xml:space="preserve">"José Vasconcelos filosofía de México" par Filosofia Corporativa</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/heschel-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/vasconcelos-mini.webp</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">spiritualite ; ethique</t>
+          <t xml:space="preserve">esthetique ; politique</t>
         </is>
       </c>
       <c r="K65" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existentialisme ; Mysticisme ; Hassidisme</t>
+          <t xml:space="preserve">Monisme ; Spiritualisme</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rabbin et philosophe juif, penseur du « pathos divin » et du shabbat, militant des droits civiques.</t>
-        </is>
-      </c>
-      <c r="M65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">juive</t>
+          <t xml:space="preserve">philosophe et ministre mexicain de l’Éducation, auteur de La Race cosmique, penseur du métissage.</t>
         </is>
       </c>
       <c r="N65" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">occident</t>
+          <t xml:space="preserve">sud</t>
         </is>
       </c>
       <c r="O65" s="1">
@@ -5241,67 +5233,72 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Américaine</t>
+          <t xml:space="preserve">Mexicaine</t>
         </is>
       </c>
     </row>
     <row r="66" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1">
-        <v>1914</v>
+        <v>1907</v>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1998</t>
+          <t xml:space="preserve">1972</t>
         </is>
       </c>
       <c r="C66" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1914 – 1998</t>
+          <t xml:space="preserve">1907 – 1972</t>
         </is>
       </c>
       <c r="D66" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Octavio PAZ</t>
+          <t xml:space="preserve">Abraham Joshua HESCHEL</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Octavio_Paz" title=" Wikipedia"&gt;Octavio PAZ&lt;/a&gt; est un poète, essayiste et diplomate mexicain, prix Nobel de littérature en 1990. Né à Mexico dans une famille marquée par la révolution, son père ayant été le représentant d’Emiliano Zapata aux États-Unis, il soutient les républicains pendant la guerre d’Espagne, puis rompt avec le communisme après l’assassinat de Trotski. Diplomate à Paris après la guerre, il y fréquente les surréalistes et André Breton.&lt;/p&gt; &lt;p&gt;Dans &lt;a href="https://fr.wikipedia.org/wiki/Le_Labyrinthe_de_la_solitude" title=" Wikipedia"&gt;&lt;em&gt;Le Labyrinthe de la solitude&lt;/em&gt;&lt;/a&gt; (1950), il interroge l’identité mexicaine : derrière les masques de la politesse et la violence des fêtes se cache une solitude née de l’histoire, celle d’un peuple issu de la conquête, qui a renié à la fois son passé indien et son passé espagnol. Il y évoque la figure de la &lt;a href="https://fr.wikipedia.org/wiki/La_Malinche" title=" Wikipedia"&gt;Malinche&lt;/a&gt;, compagne indienne de Cortés, symbole ambigu de l’origine métisse du pays. Mais cette solitude est aussi celle de l’homme moderne, et la poésie, l’amour et la fête sont des moyens de la dépasser. Dans &lt;em&gt;L’Arc et la Lyre&lt;/em&gt; (1956), il fait de la poésie une expérience de communion qui révèle l’homme à lui-même.&lt;/p&gt; &lt;p&gt;Ambassadeur du Mexique en Inde de 1962 à 1968, il découvre les philosophies et l’art de l’Orient, qui nourrissent sa poésie. Il démissionne après le &lt;a href="https://fr.wikipedia.org/wiki/Massacre_de_Tlatelolco" title=" Wikipedia"&gt;massacre de Tlatelolco&lt;/a&gt;, où des centaines d’étudiants sont tués par l’armée en 1968. Critique des totalitarismes de droite comme de gauche, il fonde la revue &lt;em&gt;Vuelta&lt;/em&gt; et consacre un grand livre à la poétesse et penseuse Juana Inés de la Cruz. Il meurt à Mexico en 1998, à quatre-vingt-quatre ans.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Abraham_Joshua_Heschel" title=" Wikipedia"&gt;Abraham Joshua HESCHEL&lt;/a&gt; est un rabbin, théologien et philosophe juif, l’une des grandes voix religieuses du XXe siècle. Né à Varsovie dans une illustre famille du &lt;a href="https://fr.wikipedia.org/wiki/Hassidisme" title=" Wikipedia"&gt;hassidisme&lt;/a&gt;, il étudie la philosophie à Berlin, où il soutient une thèse sur les prophètes d’Israël. Expulsé d’Allemagne vers la Pologne en 1938, il parvient à quitter Varsovie quelques semaines avant l’invasion allemande et gagne Londres, puis les États-Unis. Sa mère et ses sœurs sont assassinées pendant la Shoah. Il enseigne à partir de 1946 au Séminaire théologique juif de New York.&lt;/p&gt; &lt;p&gt;Pour Heschel, la religion commence par l’« étonnement radical » devant le monde, qui précède toute réflexion. Contre l’idée d’un Dieu impassible des philosophes, il parle du « pathos divin » : le Dieu des prophètes est concerné par le sort des hommes et souffre de l’injustice. La question n’est pas seulement de savoir si l’homme cherche Dieu, mais de comprendre que &lt;em&gt;Dieu est en quête de l’homme&lt;/em&gt;, titre de son livre de 1955. Dans &lt;em&gt;Les Bâtisseurs du temps&lt;/em&gt; (1951), il présente le &lt;a href="https://fr.wikipedia.org/wiki/Shabbat" title=" Wikipedia"&gt;shabbat&lt;/a&gt; comme « une cathédrale dans le temps » : le judaïsme sanctifie des moments plutôt que des lieux. Il consacre aussi un grand livre aux prophètes, témoins de la passion de Dieu pour la justice.&lt;/p&gt; &lt;p&gt;Sa foi le conduit à l’action. En 1965, il marche de Selma à Montgomery aux côtés de Martin Luther King et dira : « J’avais l’impression que mes jambes priaient. » Il s’oppose à la guerre du Vietnam et contribue au dialogue entre juifs et chrétiens lors du concile Vatican II. Il meurt à New York en 1972.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t xml:space="preserve">ZIxDHuVg9TQ</t>
+          <t xml:space="preserve">SLINbVsBz-Q</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Octavio PAZ – Un siècle d'écrivains : 1914-1990 (France 3, 2000)" par ÉCLAIR BRUT</t>
+          <t xml:space="preserve">"LA PENSEE D'AVRAHAM YOSHOUA HESCHEL" Rony Akrich"" par רוני אקריש</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/paz-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/heschel-mini.webp</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">esthetique ; politique</t>
+          <t xml:space="preserve">spiritualite ; ethique</t>
         </is>
       </c>
       <c r="K66" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Humanisme</t>
+          <t xml:space="preserve">Existentialisme ; Mysticisme ; Hassidisme</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">poète et essayiste mexicain, prix Nobel 1990, auteur du Labyrinthe de la solitude.</t>
+          <t xml:space="preserve">rabbin et philosophe juif, penseur du « pathos divin » et du shabbat, militant des droits civiques.</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
         </is>
       </c>
       <c r="N66" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">sud</t>
+          <t xml:space="preserve">occident</t>
         </is>
       </c>
       <c r="O66" s="1">
@@ -5309,62 +5306,62 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mexicaine</t>
+          <t xml:space="preserve">Américaine</t>
         </is>
       </c>
     </row>
     <row r="67" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1">
-        <v>1871</v>
+        <v>1914</v>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1917</t>
+          <t xml:space="preserve">1998</t>
         </is>
       </c>
       <c r="C67" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1871 – 1917</t>
+          <t xml:space="preserve">1914 – 1998</t>
         </is>
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">José Enrique RODÓ</t>
+          <t xml:space="preserve">Octavio PAZ</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jos%C3%A9_Enrique_Rod%C3%B3" title=" Wikipedia"&gt;José Enrique RODÓ&lt;/a&gt; est un écrivain et essayiste uruguayen, l’un des grands maîtres à penser de l’Amérique latine au début du XXe siècle. Né à Montevideo, il doit interrompre ses études après la ruine de sa famille, se forme largement seul et devient professeur de littérature à l’université de Montevideo, puis député. Correspondant de &lt;a href="https://fr.wikipedia.org/wiki/Rub%C3%A9n_Dar%C3%ADo" title=" Wikipedia"&gt;Rubén Darío&lt;/a&gt;, il est le principal théoricien du modernisme, le grand mouvement de renouvellement de la littérature hispano-américaine.&lt;/p&gt; &lt;p&gt;Son essai &lt;em&gt;Ariel&lt;/em&gt; (1900), écrit deux ans après la victoire des États-Unis sur l’Espagne à Cuba, prend la forme d’un dernier cours donné par un vieux maître, Prospero, à ses élèves. Empruntant les personnages de &lt;em&gt;La Tempête&lt;/em&gt; de Shakespeare, il oppose Ariel, l’esprit, la beauté, le désintéressement, à Caliban, la matière, l’utilité, les appétits. Il met en garde la jeunesse latino-américaine contre l’utilitarisme et la « nordomanie », la fascination pour le modèle des États-Unis, puissant mais tourné vers le seul profit.&lt;/p&gt; &lt;p&gt;Rodó invite les jeunes à cultiver toutes les facultés de l’esprit, à préserver un temps libre pour la pensée et la beauté, et à construire une démocratie qui élève chacun au lieu de niveler par le bas. Le livre connut un immense succès et inspira tout un courant, l’« arielisme ». Plus tard, des penseurs comme Roberto Fernández Retamar ont renversé le symbole en faisant de Caliban la figure du colonisé. Dans &lt;em&gt;Motifs de Protée&lt;/em&gt; (1909), il médite sur la transformation continuelle de soi. Rodó meurt à Palerme en 1917, au cours d’un voyage en Europe.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Octavio_Paz" title=" Wikipedia"&gt;Octavio PAZ&lt;/a&gt; est un poète, essayiste et diplomate mexicain, prix Nobel de littérature en 1990. Né à Mexico dans une famille marquée par la révolution, son père ayant été le représentant d’Emiliano Zapata aux États-Unis, il soutient les républicains pendant la guerre d’Espagne, puis rompt avec le communisme après l’assassinat de Trotski. Diplomate à Paris après la guerre, il y fréquente les surréalistes et André Breton.&lt;/p&gt; &lt;p&gt;Dans &lt;a href="https://fr.wikipedia.org/wiki/Le_Labyrinthe_de_la_solitude" title=" Wikipedia"&gt;&lt;em&gt;Le Labyrinthe de la solitude&lt;/em&gt;&lt;/a&gt; (1950), il interroge l’identité mexicaine : derrière les masques de la politesse et la violence des fêtes se cache une solitude née de l’histoire, celle d’un peuple issu de la conquête, qui a renié à la fois son passé indien et son passé espagnol. Il y évoque la figure de la &lt;a href="https://fr.wikipedia.org/wiki/La_Malinche" title=" Wikipedia"&gt;Malinche&lt;/a&gt;, compagne indienne de Cortés, symbole ambigu de l’origine métisse du pays. Mais cette solitude est aussi celle de l’homme moderne, et la poésie, l’amour et la fête sont des moyens de la dépasser. Dans &lt;em&gt;L’Arc et la Lyre&lt;/em&gt; (1956), il fait de la poésie une expérience de communion qui révèle l’homme à lui-même.&lt;/p&gt; &lt;p&gt;Ambassadeur du Mexique en Inde de 1962 à 1968, il découvre les philosophies et l’art de l’Orient, qui nourrissent sa poésie. Il démissionne après le &lt;a href="https://fr.wikipedia.org/wiki/Massacre_de_Tlatelolco" title=" Wikipedia"&gt;massacre de Tlatelolco&lt;/a&gt;, où des centaines d’étudiants sont tués par l’armée en 1968. Critique des totalitarismes de droite comme de gauche, il fonde la revue &lt;em&gt;Vuelta&lt;/em&gt; et consacre un grand livre à la poétesse et penseuse Juana Inés de la Cruz. Il meurt à Mexico en 1998, à quatre-vingt-quatre ans.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2csl4K2CTs</t>
+          <t xml:space="preserve">ZIxDHuVg9TQ</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t xml:space="preserve">"La Mesa de Filósofos: José Enrique Rodó, su legado a 150 años del nacimiento" par En Perspectiva + VIDEO </t>
+          <t xml:space="preserve">"Octavio PAZ – Un siècle d'écrivains : 1914-1990 (France 3, 2000)" par ÉCLAIR BRUT</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/rodo-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/paz-mini.webp</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">esthetique ; ethique</t>
+          <t xml:space="preserve">esthetique ; politique</t>
         </is>
       </c>
       <c r="K67" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Humanisme ; Spiritualisme</t>
+          <t xml:space="preserve">Humanisme</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">essayiste uruguayen, auteur d’Ariel, maître à penser de la jeunesse latino-américaine.</t>
+          <t xml:space="preserve">poète et essayiste mexicain, prix Nobel 1990, auteur du Labyrinthe de la solitude.</t>
         </is>
       </c>
       <c r="N67" s="1" t="inlineStr">
@@ -5377,62 +5374,62 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uruguayenne</t>
+          <t xml:space="preserve">Mexicaine</t>
         </is>
       </c>
     </row>
     <row r="68" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1">
-        <v>1922</v>
+        <v>1871</v>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1979</t>
+          <t xml:space="preserve">1917</t>
         </is>
       </c>
       <c r="C68" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1922 – 1979</t>
+          <t xml:space="preserve">1871 – 1917</t>
         </is>
       </c>
       <c r="D68" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rodolfo KUSCH</t>
+          <t xml:space="preserve">José Enrique RODÓ</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://es.wikipedia.org/wiki/Rodolfo_Kusch" title=" Wikipedia (es)"&gt;Rodolfo KUSCH&lt;/a&gt; est un philosophe et anthropologue argentin qui a cherché à fonder une philosophie à partir de la pensée indigène et populaire de l’Amérique. Né à Buenos Aires de parents allemands, il étudie la philosophie à l’université de Buenos Aires, enseigne l’esthétique et écrit aussi pour le théâtre, notamment sur le tango. Persécuté pour ses sympathies péronistes après 1955, il part pour la Bolivie et le Pérou, puis s’installe dans le nord-ouest de l’Argentine, à Maimará, dans la province de Jujuy.&lt;/p&gt; &lt;p&gt;Au contact des communautés &lt;a href="https://fr.wikipedia.org/wiki/Quechuas" title=" Wikipedia"&gt;quechuas&lt;/a&gt; et &lt;a href="https://fr.wikipedia.org/wiki/Aymaras" title=" Wikipedia"&gt;aymaras&lt;/a&gt; des Andes, il mène de longues enquêtes de terrain, dont il tire &lt;em&gt;L’Amérique profonde&lt;/em&gt; (1962) et &lt;em&gt;La Pensée indigène et populaire en Amérique&lt;/em&gt; (1970). Il y oppose deux attitudes. Celle de l’Occident, l’« être », qui veut dominer le monde, le transformer et accumuler. Et celle de l’Amérique indienne, l’« être là » ou le simple « se tenir » (en espagnol &lt;em&gt;estar&lt;/em&gt;), qui accepte l’incertitude du monde, ses forces et ses menaces, et cherche à vivre en équilibre avec lui.&lt;/p&gt; &lt;p&gt;Pour Kusch, les classes moyennes des villes, qui se veulent européennes, vivent dans la peur de cette « Amérique profonde » qu’elles refoulent. Penser en Amérique, c’est accepter cette part indienne et populaire au lieu de la mépriser. Son œuvre, longtemps marginale, a nourri la &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_la_lib%C3%A9ration" title=" Wikipedia"&gt;philosophie de la libération&lt;/a&gt; et les pensées décoloniales latino-américaines, et elle est aujourd’hui redécouverte. Il parle même de « phagocytose » : la culture populaire finirait par absorber ce que la modernité importée croit lui imposer. Il meurt en 1979 à Maimará, à cinquante-sept ans.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jos%C3%A9_Enrique_Rod%C3%B3" title=" Wikipedia"&gt;José Enrique RODÓ&lt;/a&gt; est un écrivain et essayiste uruguayen, l’un des grands maîtres à penser de l’Amérique latine au début du XXe siècle. Né à Montevideo, il doit interrompre ses études après la ruine de sa famille, se forme largement seul et devient professeur de littérature à l’université de Montevideo, puis député. Correspondant de &lt;a href="https://fr.wikipedia.org/wiki/Rub%C3%A9n_Dar%C3%ADo" title=" Wikipedia"&gt;Rubén Darío&lt;/a&gt;, il est le principal théoricien du modernisme, le grand mouvement de renouvellement de la littérature hispano-américaine.&lt;/p&gt; &lt;p&gt;Son essai &lt;em&gt;Ariel&lt;/em&gt; (1900), écrit deux ans après la victoire des États-Unis sur l’Espagne à Cuba, prend la forme d’un dernier cours donné par un vieux maître, Prospero, à ses élèves. Empruntant les personnages de &lt;em&gt;La Tempête&lt;/em&gt; de Shakespeare, il oppose Ariel, l’esprit, la beauté, le désintéressement, à Caliban, la matière, l’utilité, les appétits. Il met en garde la jeunesse latino-américaine contre l’utilitarisme et la « nordomanie », la fascination pour le modèle des États-Unis, puissant mais tourné vers le seul profit.&lt;/p&gt; &lt;p&gt;Rodó invite les jeunes à cultiver toutes les facultés de l’esprit, à préserver un temps libre pour la pensée et la beauté, et à construire une démocratie qui élève chacun au lieu de niveler par le bas. Le livre connut un immense succès et inspira tout un courant, l’« arielisme ». Plus tard, des penseurs comme Roberto Fernández Retamar ont renversé le symbole en faisant de Caliban la figure du colonisé. Dans &lt;em&gt;Motifs de Protée&lt;/em&gt; (1909), il médite sur la transformation continuelle de soi. Rodó meurt à Palerme en 1917, au cours d’un voyage en Europe.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t xml:space="preserve">xow95qdu2wE</t>
+          <t xml:space="preserve">C2csl4K2CTs</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Podcast filosófico -  Rodolfo Kusch" par Filo Errante</t>
+          <t xml:space="preserve">"La Mesa de Filósofos: José Enrique Rodó, su legado a 150 años del nacimiento" par En Perspectiva + VIDEO </t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/kusch-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/rodo-mini.webp</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">metaphysique ; epistemologie</t>
+          <t xml:space="preserve">esthetique ; ethique</t>
         </is>
       </c>
       <c r="K68" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buen Vivir (cosmovision andine) ; Philosophie de la libération</t>
+          <t xml:space="preserve">Humanisme ; Spiritualisme</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe et anthropologue argentin, penseur de l’« Amérique profonde » et de la pensée indigène et populaire.</t>
+          <t xml:space="preserve">essayiste uruguayen, auteur d’Ariel, maître à penser de la jeunesse latino-américaine.</t>
         </is>
       </c>
       <c r="N68" s="1" t="inlineStr">
@@ -5445,62 +5442,62 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Argentine</t>
+          <t xml:space="preserve">Uruguayenne</t>
         </is>
       </c>
     </row>
     <row r="69" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1">
-        <v>1925</v>
+        <v>1922</v>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1974</t>
+          <t xml:space="preserve">1979</t>
         </is>
       </c>
       <c r="C69" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1925 – 1974</t>
+          <t xml:space="preserve">1922 – 1979</t>
         </is>
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Augusto SALAZAR BONDY</t>
+          <t xml:space="preserve">Rodolfo KUSCH</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://es.wikipedia.org/wiki/Augusto_Salazar_Bondy" title=" Wikipedia (es)"&gt;Augusto SALAZAR BONDY&lt;/a&gt; est un philosophe et éducateur péruvien, l’une des figures fondatrices de la philosophie latino-américaine de la libération. Né à Lima, frère cadet de l’écrivain Sebastián Salazar Bondy, il étudie à l’université San Marcos, puis au Mexique auprès de José Gaos et de Leopoldo Zea, et à Paris, où il suit les cours de Jean Wahl, Jean Hyppolite et Gaston Bachelard. Professeur d’éthique à San Marcos, il écrit une grande histoire des idées au Pérou contemporain.&lt;/p&gt; &lt;p&gt;En 1968, il publie &lt;em&gt;Existe-t-il une philosophie de notre Amérique ?&lt;/em&gt;, qui provoque un vif débat avec Leopoldo Zea. Sa réponse est dure : jusqu’ici, il n’existe pas de philosophie latino-américaine authentique, mais seulement des imitations des courants européens, adoptés tour à tour sans être vraiment pensés. Ce n’est pas un manque de talent : c’est la conséquence de la domination et du sous-développement, qui produisent une culture dépendante et « aliénée », incapable de se penser elle-même.&lt;/p&gt; &lt;p&gt;Une philosophie authentique ne pourra naître qu’en prenant pour objet cette situation de domination, et en contribuant à la transformer. La philosophie devient ainsi une tâche de libération, comme le développera la &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_la_lib%C3%A9ration" title=" Wikipedia"&gt;philosophie de la libération&lt;/a&gt;. Engagé dans la réforme de l’éducation sous le gouvernement péruvien de la fin des années 1960, il défend une école qui forme des personnes libres et critiques. Il meurt prématurément à Lima en 1974, à quarante-huit ans. Ses idées ont notamment inspiré Enrique Dussel.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://es.wikipedia.org/wiki/Rodolfo_Kusch" title=" Wikipedia (es)"&gt;Rodolfo KUSCH&lt;/a&gt; est un philosophe et anthropologue argentin qui a cherché à fonder une philosophie à partir de la pensée indigène et populaire de l’Amérique. Né à Buenos Aires de parents allemands, il étudie la philosophie à l’université de Buenos Aires, enseigne l’esthétique et écrit aussi pour le théâtre, notamment sur le tango. Persécuté pour ses sympathies péronistes après 1955, il part pour la Bolivie et le Pérou, puis s’installe dans le nord-ouest de l’Argentine, à Maimará, dans la province de Jujuy.&lt;/p&gt; &lt;p&gt;Au contact des communautés &lt;a href="https://fr.wikipedia.org/wiki/Quechuas" title=" Wikipedia"&gt;quechuas&lt;/a&gt; et &lt;a href="https://fr.wikipedia.org/wiki/Aymaras" title=" Wikipedia"&gt;aymaras&lt;/a&gt; des Andes, il mène de longues enquêtes de terrain, dont il tire &lt;em&gt;L’Amérique profonde&lt;/em&gt; (1962) et &lt;em&gt;La Pensée indigène et populaire en Amérique&lt;/em&gt; (1970). Il y oppose deux attitudes. Celle de l’Occident, l’« être », qui veut dominer le monde, le transformer et accumuler. Et celle de l’Amérique indienne, l’« être là » ou le simple « se tenir » (en espagnol &lt;em&gt;estar&lt;/em&gt;), qui accepte l’incertitude du monde, ses forces et ses menaces, et cherche à vivre en équilibre avec lui.&lt;/p&gt; &lt;p&gt;Pour Kusch, les classes moyennes des villes, qui se veulent européennes, vivent dans la peur de cette « Amérique profonde » qu’elles refoulent. Penser en Amérique, c’est accepter cette part indienne et populaire au lieu de la mépriser. Son œuvre, longtemps marginale, a nourri la &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_la_lib%C3%A9ration" title=" Wikipedia"&gt;philosophie de la libération&lt;/a&gt; et les pensées décoloniales latino-américaines, et elle est aujourd’hui redécouverte. Il parle même de « phagocytose » : la culture populaire finirait par absorber ce que la modernité importée croit lui imposer. Il meurt en 1979 à Maimará, à cinquante-sept ans.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t xml:space="preserve">pKvpeeR1Q4Y</t>
+          <t xml:space="preserve">xow95qdu2wE</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t xml:space="preserve">"El concepto de alienación según Augusto Salazar Bondy" par Libros Peruanos</t>
+          <t xml:space="preserve">"Podcast filosófico -  Rodolfo Kusch" par Filo Errante</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/salazarbondy-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/kusch-mini.webp</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">politique ; ethique</t>
+          <t xml:space="preserve">metaphysique ; epistemologie</t>
         </is>
       </c>
       <c r="K69" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiers-mondisme ; Philosophie de la libération</t>
+          <t xml:space="preserve">Buen Vivir (cosmovision andine) ; Philosophie de la libération</t>
         </is>
       </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe péruvien, auteur d’Existe-t-il une philosophie de notre Amérique ?, penseur de la domination.</t>
+          <t xml:space="preserve">philosophe et anthropologue argentin, penseur de l’« Amérique profonde » et de la pensée indigène et populaire.</t>
         </is>
       </c>
       <c r="N69" s="1" t="inlineStr">
@@ -5513,62 +5510,62 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Péruvienne</t>
+          <t xml:space="preserve">Argentine</t>
         </is>
       </c>
     </row>
     <row r="70" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1">
-        <v>1839</v>
+        <v>1925</v>
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1903</t>
+          <t xml:space="preserve">1974</t>
         </is>
       </c>
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1839 – 1903</t>
+          <t xml:space="preserve">1925 – 1974</t>
         </is>
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eugenio María de HOSTOS</t>
+          <t xml:space="preserve">Augusto SALAZAR BONDY</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Eugenio_Mar%C3%ADa_de_Hostos" title=" Wikipedia (en)"&gt;Eugenio María de HOSTOS&lt;/a&gt; est un philosophe, éducateur, sociologue et écrivain de &lt;a href="https://fr.wikipedia.org/wiki/Porto_Rico" title=" Wikipedia"&gt;Porto Rico&lt;/a&gt;, surnommé « le Grand Citoyen des Amériques ». Né à Mayagüez dans une famille aisée, il fait ses études en Espagne, où il étudie le droit et la philosophie à Madrid et publie en 1863 un roman, &lt;em&gt;Le Pèlerinage de Bayoán&lt;/em&gt;, qui évoque déjà le destin des Antilles. Déçu que la République espagnole refuse l’autonomie de Porto Rico, il quitte l’Espagne en 1869 pour se consacrer à l’indépendance des colonies antillaises.&lt;/p&gt; &lt;p&gt;Il rêve d’une Confédération des Antilles, réunissant Porto Rico, Cuba et la République dominicaine, et parcourt pour la défendre les États-Unis, le Pérou, le Chili, l’Argentine, le Brésil et le Venezuela. Partout, il fonde ou réforme des écoles. En République dominicaine, il crée en 1880 la première école normale, qui forme des instituteurs à une pédagogie scientifique et laïque. Au Chili, il plaide pour que les femmes aient accès à l’enseignement supérieur et aux professions savantes.&lt;/p&gt; &lt;p&gt;Sa &lt;em&gt;Morale sociale&lt;/em&gt; (1888), inspirée du &lt;a href="https://fr.wikipedia.org/wiki/Positivisme" title=" Wikipedia"&gt;positivisme&lt;/a&gt;, fonde les devoirs de l’individu non sur la religion, mais sur la raison et sur les liens qui l’unissent à la famille, à la société et à l’humanité ; l’éducation doit former des consciences libres et responsables. Après la guerre de 1898, qui fait passer Porto Rico sous domination américaine, il milite pour que l’île puisse décider elle-même de son avenir. Il laisse aussi un traité de sociologie, l’un des premiers d’Amérique latine. Il meurt en exil à Saint-Domingue en 1903.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://es.wikipedia.org/wiki/Augusto_Salazar_Bondy" title=" Wikipedia (es)"&gt;Augusto SALAZAR BONDY&lt;/a&gt; est un philosophe et éducateur péruvien, l’une des figures fondatrices de la philosophie latino-américaine de la libération. Né à Lima, frère cadet de l’écrivain Sebastián Salazar Bondy, il étudie à l’université San Marcos, puis au Mexique auprès de José Gaos et de Leopoldo Zea, et à Paris, où il suit les cours de Jean Wahl, Jean Hyppolite et Gaston Bachelard. Professeur d’éthique à San Marcos, il écrit une grande histoire des idées au Pérou contemporain.&lt;/p&gt; &lt;p&gt;En 1968, il publie &lt;em&gt;Existe-t-il une philosophie de notre Amérique ?&lt;/em&gt;, qui provoque un vif débat avec Leopoldo Zea. Sa réponse est dure : jusqu’ici, il n’existe pas de philosophie latino-américaine authentique, mais seulement des imitations des courants européens, adoptés tour à tour sans être vraiment pensés. Ce n’est pas un manque de talent : c’est la conséquence de la domination et du sous-développement, qui produisent une culture dépendante et « aliénée », incapable de se penser elle-même.&lt;/p&gt; &lt;p&gt;Une philosophie authentique ne pourra naître qu’en prenant pour objet cette situation de domination, et en contribuant à la transformer. La philosophie devient ainsi une tâche de libération, comme le développera la &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_la_lib%C3%A9ration" title=" Wikipedia"&gt;philosophie de la libération&lt;/a&gt;. Engagé dans la réforme de l’éducation sous le gouvernement péruvien de la fin des années 1960, il défend une école qui forme des personnes libres et critiques. Il meurt prématurément à Lima en 1974, à quarante-huit ans. Ses idées ont notamment inspiré Enrique Dussel.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t xml:space="preserve">yxxhyhWr-N4</t>
+          <t xml:space="preserve">pKvpeeR1Q4Y</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Eugenio María de Hostos / intelectual educador, filósofo, sociólogo y escritor puertorriqueño" par Damián S. Vargas</t>
+          <t xml:space="preserve">"El concepto de alienación según Augusto Salazar Bondy" par Libros Peruanos</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/hostos-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/salazarbondy-mini.webp</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ethique ; politique</t>
+          <t xml:space="preserve">politique ; ethique</t>
         </is>
       </c>
       <c r="K70" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Positivisme</t>
+          <t xml:space="preserve">Tiers-mondisme ; Philosophie de la libération</t>
         </is>
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">éducateur et penseur portoricain, apôtre d’une confédération des Antilles et d’une morale sociale laïque.</t>
+          <t xml:space="preserve">philosophe péruvien, auteur d’Existe-t-il une philosophie de notre Amérique ?, penseur de la domination.</t>
         </is>
       </c>
       <c r="N70" s="1" t="inlineStr">
@@ -5581,62 +5578,62 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portoricaine</t>
+          <t xml:space="preserve">Péruvienne</t>
         </is>
       </c>
     </row>
     <row r="71" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1">
-        <v>1925</v>
+        <v>1839</v>
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2008</t>
+          <t xml:space="preserve">1903</t>
         </is>
       </c>
       <c r="C71" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1925 – 2008</t>
+          <t xml:space="preserve">1839 – 1903</t>
         </is>
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Orlando FALS BORDA</t>
+          <t xml:space="preserve">Eugenio María de HOSTOS</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Orlando_Fals_Borda" title=" Wikipedia (en)"&gt;Orlando FALS BORDA&lt;/a&gt; est un sociologue colombien, l’un des grands penseurs latino-américains des sciences sociales et le fondateur de la « recherche-action participative ». Né à Barranquilla, sur la côte caraïbe, formé aux États-Unis, il fonde en 1959 à l’Université nationale de Colombie, avec le prêtre Camilo Torres, l’une des premières facultés de sociologie d’Amérique latine. Son livre &lt;em&gt;La Violence en Colombie&lt;/em&gt; (1962), écrit avec Germán Guzmán et Eduardo Umaña, étudie pour la première fois la guerre civile qui ravage les campagnes.&lt;/p&gt; &lt;p&gt;Déçu par une sociologie qui observe les pauvres de l’extérieur sans rien changer à leur sort, il quitte l’université dans les années 1970 pour travailler avec les paysans et les communautés de la côte caraïbe. Il y développe la &lt;a href="https://fr.wikipedia.org/wiki/Recherche-action" title=" Wikipedia"&gt;recherche-action&lt;/a&gt; participative : le chercheur ne doit pas monopoliser le savoir ni imposer sa technique, mais travailler avec les communautés comme avec des partenaires et des co-chercheurs, recueillir leurs savoirs, leur mémoire et leurs récits, et partager les résultats sous une forme que tous peuvent comprendre.&lt;/p&gt; &lt;p&gt;La science n’est pas, selon lui, une affaire d’experts neutres : elle doit servir la transformation de la société et la libération des opprimés. Il parle d’une « subversion positive » qui conteste l’ordre injuste pour en construire un meilleur. Ses idées se sont répandues dans le monde entier, en éducation, en santé et en développement. Il participe aussi à l’Assemblée constituante qui rédige la Constitution colombienne de 1991. Il meurt à Bogotá en 2008.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Eugenio_Mar%C3%ADa_de_Hostos" title=" Wikipedia (en)"&gt;Eugenio María de HOSTOS&lt;/a&gt; est un philosophe, éducateur, sociologue et écrivain de &lt;a href="https://fr.wikipedia.org/wiki/Porto_Rico" title=" Wikipedia"&gt;Porto Rico&lt;/a&gt;, surnommé « le Grand Citoyen des Amériques ». Né à Mayagüez dans une famille aisée, il fait ses études en Espagne, où il étudie le droit et la philosophie à Madrid et publie en 1863 un roman, &lt;em&gt;Le Pèlerinage de Bayoán&lt;/em&gt;, qui évoque déjà le destin des Antilles. Déçu que la République espagnole refuse l’autonomie de Porto Rico, il quitte l’Espagne en 1869 pour se consacrer à l’indépendance des colonies antillaises.&lt;/p&gt; &lt;p&gt;Il rêve d’une Confédération des Antilles, réunissant Porto Rico, Cuba et la République dominicaine, et parcourt pour la défendre les États-Unis, le Pérou, le Chili, l’Argentine, le Brésil et le Venezuela. Partout, il fonde ou réforme des écoles. En République dominicaine, il crée en 1880 la première école normale, qui forme des instituteurs à une pédagogie scientifique et laïque. Au Chili, il plaide pour que les femmes aient accès à l’enseignement supérieur et aux professions savantes.&lt;/p&gt; &lt;p&gt;Sa &lt;em&gt;Morale sociale&lt;/em&gt; (1888), inspirée du &lt;a href="https://fr.wikipedia.org/wiki/Positivisme" title=" Wikipedia"&gt;positivisme&lt;/a&gt;, fonde les devoirs de l’individu non sur la religion, mais sur la raison et sur les liens qui l’unissent à la famille, à la société et à l’humanité ; l’éducation doit former des consciences libres et responsables. Après la guerre de 1898, qui fait passer Porto Rico sous domination américaine, il milite pour que l’île puisse décider elle-même de son avenir. Il laisse aussi un traité de sociologie, l’un des premiers d’Amérique latine. Il meurt en exil à Saint-Domingue en 1903.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t xml:space="preserve">CYIrjf9pID0</t>
+          <t xml:space="preserve">yxxhyhWr-N4</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t xml:space="preserve">"The work of Orlando Fals Borda" par stanbrad13</t>
+          <t xml:space="preserve">"Eugenio María de Hostos / intelectual educador, filósofo, sociólogo y escritor puertorriqueño" par Damián S. Vargas</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/falsborda-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/hostos-mini.webp</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">epistemologie ; politique</t>
+          <t xml:space="preserve">ethique ; politique</t>
         </is>
       </c>
       <c r="K71" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiers-mondisme</t>
+          <t xml:space="preserve">Positivisme</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sociologue colombien, fondateur de la recherche-action participative, penseur d’un savoir construit avec le peuple.</t>
+          <t xml:space="preserve">éducateur et penseur portoricain, apôtre d’une confédération des Antilles et d’une morale sociale laïque.</t>
         </is>
       </c>
       <c r="N71" s="1" t="inlineStr">
@@ -5649,72 +5646,67 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Colombienne</t>
+          <t xml:space="preserve">Portoricaine</t>
         </is>
       </c>
     </row>
     <row r="72" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1">
-        <v>1928</v>
+        <v>1925</v>
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2021</t>
+          <t xml:space="preserve">2008</t>
         </is>
       </c>
       <c r="C72" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1928 – 2021</t>
+          <t xml:space="preserve">1925 – 2008</t>
         </is>
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Humberto MATURANA</t>
+          <t xml:space="preserve">Orlando FALS BORDA</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Humberto_Maturana" title=" Wikipedia"&gt;Humberto MATURANA&lt;/a&gt; est un biologiste et philosophe chilien, l’un des penseurs les plus originaux de la biologie de la connaissance. Né à Santiago, il étudie la médecine et la biologie au Chili, puis en Angleterre et à Harvard. Au Massachusetts Institute of Technology, il participe en 1959 à une étude devenue célèbre sur ce que l’œil de la grenouille transmet à son cerveau, qui montre que la perception n’est pas une simple copie du monde extérieur. Il fonde ensuite à l’université du Chili un laboratoire d’« épistémologie expérimentale ».&lt;/p&gt; &lt;p&gt;Avec son élève Francisco Varela, il propose au début des années 1970 le concept d’&lt;a href="https://fr.wikipedia.org/wiki/Autopo%C3%AF%C3%A8se" title=" Wikipedia"&gt;autopoïèse&lt;/a&gt;, du grec « se produire soi-même » : un être vivant est un système qui produit et renouvelle sans cesse ses propres composants, et maintient ainsi sa propre organisation. La cellule en est le modèle. Le vivant n’est donc pas défini par ce qu’il contient, mais par cette manière de s’entretenir lui-même, en échange constant avec son milieu.&lt;/p&gt; &lt;p&gt;Il en tire une théorie de la connaissance : « Tout ce qui est dit est dit par un observateur. » Connaître n’est pas refléter un monde tout fait, mais une activité du vivant, qui fait émerger un monde à travers son action. Dans &lt;em&gt;L’Arbre de la connaissance&lt;/em&gt; (1984), écrit avec Varela, il montre aussi que le langage et la société naissent de la coordination entre les êtres, et que l’amour, l’acceptation de l’autre, est le fondement biologique de la vie sociale. Ses idées ont nourri le &lt;a href="https://fr.wikipedia.org/wiki/Constructivisme_%28%C3%A9pist%C3%A9mologie%29" title=" Wikipedia"&gt;constructivisme&lt;/a&gt;, la thérapie familiale et la théorie des systèmes sociaux de &lt;a href="https://fr.wikipedia.org/wiki/Niklas_Luhmann" title=" Wikipedia"&gt;Niklas Luhmann&lt;/a&gt;. Il meurt à Santiago en 2021.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Orlando_Fals_Borda" title=" Wikipedia (en)"&gt;Orlando FALS BORDA&lt;/a&gt; est un sociologue colombien, l’un des grands penseurs latino-américains des sciences sociales et le fondateur de la « recherche-action participative ». Né à Barranquilla, sur la côte caraïbe, formé aux États-Unis, il fonde en 1959 à l’Université nationale de Colombie, avec le prêtre Camilo Torres, l’une des premières facultés de sociologie d’Amérique latine. Son livre &lt;em&gt;La Violence en Colombie&lt;/em&gt; (1962), écrit avec Germán Guzmán et Eduardo Umaña, étudie pour la première fois la guerre civile qui ravage les campagnes.&lt;/p&gt; &lt;p&gt;Déçu par une sociologie qui observe les pauvres de l’extérieur sans rien changer à leur sort, il quitte l’université dans les années 1970 pour travailler avec les paysans et les communautés de la côte caraïbe. Il y développe la &lt;a href="https://fr.wikipedia.org/wiki/Recherche-action" title=" Wikipedia"&gt;recherche-action&lt;/a&gt; participative : le chercheur ne doit pas monopoliser le savoir ni imposer sa technique, mais travailler avec les communautés comme avec des partenaires et des co-chercheurs, recueillir leurs savoirs, leur mémoire et leurs récits, et partager les résultats sous une forme que tous peuvent comprendre.&lt;/p&gt; &lt;p&gt;La science n’est pas, selon lui, une affaire d’experts neutres : elle doit servir la transformation de la société et la libération des opprimés. Il parle d’une « subversion positive » qui conteste l’ordre injuste pour en construire un meilleur. Ses idées se sont répandues dans le monde entier, en éducation, en santé et en développement. Il participe aussi à l’Assemblée constituante qui rédige la Constitution colombienne de 1991. Il meurt à Bogotá en 2008.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t xml:space="preserve">19uV8wKpkZw</t>
+          <t xml:space="preserve">CYIrjf9pID0</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t xml:space="preserve">"La entrevista al académico Humberto Maturana que inspiró a Mon Laferte | La Belleza de Pensar" par Canal13C</t>
+          <t xml:space="preserve">"The work of Orlando Fals Borda" par stanbrad13</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/maturana-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/falsborda-mini.webp</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">epistemologie ; metaphysique</t>
+          <t xml:space="preserve">epistemologie ; politique</t>
         </is>
       </c>
       <c r="K72" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Constructivisme</t>
+          <t xml:space="preserve">Tiers-mondisme</t>
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">biologiste et philosophe chilien, inventeur avec Varela de l’autopoïèse, penseur de la connaissance comme fait biologique.</t>
-        </is>
-      </c>
-      <c r="M72" t="inlineStr">
+          <t xml:space="preserve">sociologue colombien, fondateur de la recherche-action participative, penseur d’un savoir construit avec le peuple.</t>
+        </is>
+      </c>
+      <c r="N72" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">sud</t>
-        </is>
-      </c>
-      <c r="N72" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
         </is>
       </c>
       <c r="O72" s="1">
@@ -5722,47 +5714,47 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chilienne</t>
+          <t xml:space="preserve">Colombienne</t>
         </is>
       </c>
     </row>
     <row r="73" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1">
-        <v>1946</v>
+        <v>1928</v>
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2001</t>
+          <t xml:space="preserve">2021</t>
         </is>
       </c>
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1946 – 2001</t>
+          <t xml:space="preserve">1928 – 2021</t>
         </is>
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Francisco VARELA</t>
+          <t xml:space="preserve">Humberto MATURANA</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Francisco_Varela" title=" Wikipedia"&gt;Francisco VARELA&lt;/a&gt; est un biologiste, neuroscientifique et philosophe chilien, l’un des fondateurs des sciences cognitives « incarnées ». Né à Talcahuano, élève d’Humberto Maturana, il soutient une thèse de biologie à Harvard, puis invente avec son maître le concept d’&lt;a href="https://fr.wikipedia.org/wiki/Autopo%C3%AF%C3%A8se" title=" Wikipedia"&gt;autopoïèse&lt;/a&gt;, qui définit le vivant par sa capacité à se produire lui-même. Après le coup d’État de Pinochet en 1973, il doit s’exiler aux États-Unis. Il s’installe en France en 1986 et dirige jusqu’à sa mort une équipe de recherche au CNRS, à Paris.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;L’Inscription corporelle de l’esprit&lt;/em&gt; (1991), écrit avec Evan Thompson et Eleanor Rosch, il critique l’idée que l’esprit serait un ordinateur qui traite des représentations d’un monde extérieur déjà donné. Il propose à la place l’« &lt;a href="https://fr.wikipedia.org/wiki/%C3%89naction" title=" Wikipedia"&gt;énaction&lt;/a&gt; » : la cognition est une action incarnée, par laquelle un être vivant fait émerger son monde à travers son corps, ses sens et ses gestes. Il fonde aussi la « neurophénoménologie », qui veut unir les mesures du cerveau et la description rigoureuse de l’expérience vécue, à la manière de Husserl et de Merleau-Ponty.&lt;/p&gt; &lt;p&gt;Pratiquant du bouddhisme tibétain depuis les années 1970, il voit dans la méditation une méthode précise pour explorer l’expérience. En 1987, il cofonde le &lt;a href="https://fr.wikipedia.org/wiki/Mind_and_Life_Institute" title=" Wikipedia"&gt;Mind and Life Institute&lt;/a&gt;, qui organise des rencontres entre scientifiques et le dalaï-lama. Il est l’un des inspirateurs de l’idée d’un esprit « incarné », aujourd’hui centrale en &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_l%27esprit" title=" Wikipedia"&gt;philosophie de l’esprit&lt;/a&gt;. Il meurt à Paris en 2001, à cinquante-quatre ans, d’une maladie du foie.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Humberto_Maturana" title=" Wikipedia"&gt;Humberto MATURANA&lt;/a&gt; est un biologiste et philosophe chilien, l’un des penseurs les plus originaux de la biologie de la connaissance. Né à Santiago, il étudie la médecine et la biologie au Chili, puis en Angleterre et à Harvard. Au Massachusetts Institute of Technology, il participe en 1959 à une étude devenue célèbre sur ce que l’œil de la grenouille transmet à son cerveau, qui montre que la perception n’est pas une simple copie du monde extérieur. Il fonde ensuite à l’université du Chili un laboratoire d’« épistémologie expérimentale ».&lt;/p&gt; &lt;p&gt;Avec son élève Francisco Varela, il propose au début des années 1970 le concept d’&lt;a href="https://fr.wikipedia.org/wiki/Autopo%C3%AF%C3%A8se" title=" Wikipedia"&gt;autopoïèse&lt;/a&gt;, du grec « se produire soi-même » : un être vivant est un système qui produit et renouvelle sans cesse ses propres composants, et maintient ainsi sa propre organisation. La cellule en est le modèle. Le vivant n’est donc pas défini par ce qu’il contient, mais par cette manière de s’entretenir lui-même, en échange constant avec son milieu.&lt;/p&gt; &lt;p&gt;Il en tire une théorie de la connaissance : « Tout ce qui est dit est dit par un observateur. » Connaître n’est pas refléter un monde tout fait, mais une activité du vivant, qui fait émerger un monde à travers son action. Dans &lt;em&gt;L’Arbre de la connaissance&lt;/em&gt; (1984), écrit avec Varela, il montre aussi que le langage et la société naissent de la coordination entre les êtres, et que l’amour, l’acceptation de l’autre, est le fondement biologique de la vie sociale. Ses idées ont nourri le &lt;a href="https://fr.wikipedia.org/wiki/Constructivisme_%28%C3%A9pist%C3%A9mologie%29" title=" Wikipedia"&gt;constructivisme&lt;/a&gt;, la thérapie familiale et la théorie des systèmes sociaux de &lt;a href="https://fr.wikipedia.org/wiki/Niklas_Luhmann" title=" Wikipedia"&gt;Niklas Luhmann&lt;/a&gt;. Il meurt à Santiago en 2021.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t xml:space="preserve">HPh_uAetJ8U</t>
+          <t xml:space="preserve">19uV8wKpkZw</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Francisco VARELA 2. COPYRIGHT INA ET FRANCETV" par Catherine BARRY - Au coeur du Bouddhisme</t>
+          <t xml:space="preserve">"La entrevista al académico Humberto Maturana que inspiró a Mon Laferte | La Belleza de Pensar" par Canal13C</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/varela-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/maturana-mini.webp</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -5772,12 +5764,12 @@
       </c>
       <c r="K73" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Constructivisme ; Phénoménologie</t>
+          <t xml:space="preserve">Constructivisme</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">neurobiologiste et philosophe chilien, penseur de l’énaction et du dialogue entre sciences cognitives et bouddhisme.</t>
+          <t xml:space="preserve">biologiste et philosophe chilien, inventeur avec Varela de l’autopoïèse, penseur de la connaissance comme fait biologique.</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -5801,56 +5793,56 @@
     </row>
     <row r="74" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="1">
-        <v>1868</v>
+        <v>1946</v>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1963</t>
+          <t xml:space="preserve">2001</t>
         </is>
       </c>
       <c r="C74" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1868 – 1963</t>
+          <t xml:space="preserve">1946 – 2001</t>
         </is>
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">W. E. B. DU BOIS</t>
+          <t xml:space="preserve">Francisco VARELA</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/W._E._B._Du_Bois" title=" Wikipedia"&gt;W. E. B. DU BOIS&lt;/a&gt; (William Edward Burghardt Du Bois) est un sociologue, historien et militant africain-américain, l’un des plus grands penseurs américains du XXe siècle. Né en 1868 dans le Massachusetts, il étudie à Fisk, à Berlin, puis à Harvard, où il devient en 1895 le premier Africain-Américain à obtenir un doctorat. Son étude &lt;em&gt;The Philadelphia Negro&lt;/em&gt; (1899) est l’une des premières grandes enquêtes de sociologie empirique aux États-Unis.&lt;/p&gt; &lt;p&gt;Dans &lt;a href="https://fr.wikipedia.org/wiki/Les_%C3%82mes_du_peuple_noir" title=" Wikipedia"&gt;&lt;em&gt;Les Âmes du peuple noir&lt;/em&gt;&lt;/a&gt; (1903), il affirme que « le problème du XXe siècle est le problème de la ligne de couleur ». Il y décrit la « double conscience » des Noirs américains : le sentiment de se voir toujours à travers les yeux d’un monde qui les méprise, d’être à la fois américain et noir, « deux âmes, deux pensées, deux combats inconciliables dans un seul corps sombre ». Dans &lt;em&gt;Black Reconstruction&lt;/em&gt; (1935), il réhabilitera le rôle des anciens esclaves dans l’histoire américaine d’après la guerre de Sécession. Il y critique aussi Booker T. Washington, qui conseillait aux Noirs d’accepter la ségrégation en échange du progrès économique.&lt;/p&gt; &lt;p&gt;En 1909, il est l’un des fondateurs de la &lt;a href="https://fr.wikipedia.org/wiki/National_Association_for_the_Advancement_of_Colored_People" title=" Wikipedia"&gt;NAACP&lt;/a&gt;, la grande organisation de défense des droits civiques, dont il dirige la revue &lt;em&gt;The Crisis&lt;/em&gt;. Il organise plusieurs congrès panafricains et devient le « père du &lt;a href="https://fr.wikipedia.org/wiki/Panafricanisme" title=" Wikipedia"&gt;panafricanisme&lt;/a&gt; ». Proche du socialisme, persécuté pendant le maccarthysme, il s’installe à la fin de sa vie au &lt;a href="https://fr.wikipedia.org/wiki/Ghana" title=" Wikipedia"&gt;Ghana&lt;/a&gt;, à l’invitation de Kwame Nkrumah, et y meurt en 1963, à la veille de la marche sur Washington de Martin Luther King.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Francisco_Varela" title=" Wikipedia"&gt;Francisco VARELA&lt;/a&gt; est un biologiste, neuroscientifique et philosophe chilien, l’un des fondateurs des sciences cognitives « incarnées ». Né à Talcahuano, élève d’Humberto Maturana, il soutient une thèse de biologie à Harvard, puis invente avec son maître le concept d’&lt;a href="https://fr.wikipedia.org/wiki/Autopo%C3%AF%C3%A8se" title=" Wikipedia"&gt;autopoïèse&lt;/a&gt;, qui définit le vivant par sa capacité à se produire lui-même. Après le coup d’État de Pinochet en 1973, il doit s’exiler aux États-Unis. Il s’installe en France en 1986 et dirige jusqu’à sa mort une équipe de recherche au CNRS, à Paris.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;L’Inscription corporelle de l’esprit&lt;/em&gt; (1991), écrit avec Evan Thompson et Eleanor Rosch, il critique l’idée que l’esprit serait un ordinateur qui traite des représentations d’un monde extérieur déjà donné. Il propose à la place l’« &lt;a href="https://fr.wikipedia.org/wiki/%C3%89naction" title=" Wikipedia"&gt;énaction&lt;/a&gt; » : la cognition est une action incarnée, par laquelle un être vivant fait émerger son monde à travers son corps, ses sens et ses gestes. Il fonde aussi la « neurophénoménologie », qui veut unir les mesures du cerveau et la description rigoureuse de l’expérience vécue, à la manière de Husserl et de Merleau-Ponty.&lt;/p&gt; &lt;p&gt;Pratiquant du bouddhisme tibétain depuis les années 1970, il voit dans la méditation une méthode précise pour explorer l’expérience. En 1987, il cofonde le &lt;a href="https://fr.wikipedia.org/wiki/Mind_and_Life_Institute" title=" Wikipedia"&gt;Mind and Life Institute&lt;/a&gt;, qui organise des rencontres entre scientifiques et le dalaï-lama. Il est l’un des inspirateurs de l’idée d’un esprit « incarné », aujourd’hui centrale en &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_l%27esprit" title=" Wikipedia"&gt;philosophie de l’esprit&lt;/a&gt;. Il meurt à Paris en 2001, à cinquante-quatre ans, d’une maladie du foie.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Li9wCyjag3Q</t>
+          <t xml:space="preserve">HPh_uAetJ8U</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t xml:space="preserve">"W.E.B. Du Bois : Pionnier des Droits Civiques - Une Conférence par Christian Monjou" par Art et Leadership</t>
+          <t xml:space="preserve">"Francisco VARELA 2. COPYRIGHT INA ET FRANCETV" par Catherine BARRY - Au coeur du Bouddhisme</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/dubois-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/varela-mini.webp</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">politique ; ethique</t>
+          <t xml:space="preserve">epistemologie ; metaphysique</t>
         </is>
       </c>
       <c r="K74" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pan-africanisme</t>
+          <t xml:space="preserve">Constructivisme ; Phénoménologie</t>
         </is>
       </c>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sociologue et militant africain-américain, penseur de la « double conscience » et père du panafricanisme.</t>
+          <t xml:space="preserve">neurobiologiste et philosophe chilien, penseur de l’énaction et du dialogue entre sciences cognitives et bouddhisme.</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -5864,200 +5856,207 @@
         </is>
       </c>
       <c r="O74" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Américaine</t>
+          <t xml:space="preserve">Chilienne</t>
         </is>
       </c>
     </row>
     <row r="75" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="1">
-        <v>1928</v>
+        <v>1868</v>
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024</t>
+          <t xml:space="preserve">1963</t>
         </is>
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1928 – 2024</t>
+          <t xml:space="preserve">1868 – 1963</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gustavo GUTIÉRREZ</t>
+          <t xml:space="preserve">W. E. B. DU BOIS</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Gustavo_Guti%C3%A9rrez_Merino" title=" Wikipedia"&gt;Gustavo GUTIÉRREZ&lt;/a&gt; est un prêtre et théologien péruvien, considéré comme le père de la &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9ologie_de_la_lib%C3%A9ration" title=" Wikipedia"&gt;théologie de la libération&lt;/a&gt;. Né à Lima en 1928 dans un milieu modeste, il souffre adolescent d’une ostéomyélite qui le cloue longtemps au lit ; il lit alors beaucoup et commence des études de médecine pour devenir psychiatre. À vingt-quatre ans, il choisit la prêtrise et part étudier la philosophie et la psychologie à Louvain, puis la théologie à Lyon.&lt;/p&gt; &lt;p&gt;Ordonné prêtre en 1959, il devient vicaire dans un quartier pauvre de Lima, tout en enseignant à l’université catholique, et repense toute sa théologie au contact de ce peuple. En 1971, il publie &lt;em&gt;Théologie de la libération&lt;/em&gt;, traduit dans une vingtaine de langues. La pauvreté, écrit-il, n’est pas une fatalité mais le fruit d’injustices, et elle est contraire à la volonté de Dieu. La théologie est une « réflexion critique sur la pratique à la lumière de la Parole » : elle vient en second, après l’engagement aux côtés des pauvres. Le salut ne se joue pas seulement dans l’au-delà ; il touche toute l’existence, et la libération sociale et politique en fait partie, sans s’y réduire. Dans &lt;em&gt;Boire à son propre puits&lt;/em&gt; (1983), il montre que cet engagement est aussi une spiritualité, une manière de suivre le Christ.&lt;/p&gt; &lt;p&gt;Ses positions lui valent la méfiance de Rome dans les années 1980, sans condamnation. Entré chez les Dominicains en 1998, il enseigne dans de nombreuses universités d’Europe et des États-Unis. Le pape François le reçoit en 2013, signe de la réhabilitation de son œuvre, et l’« option préférentielle pour les pauvres » est devenue un principe de l’enseignement de l’Église. Il meurt à Lima en 2024, à quatre-vingt-seize ans.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/W._E._B._Du_Bois" title=" Wikipedia"&gt;W. E. B. DU BOIS&lt;/a&gt; (William Edward Burghardt Du Bois) est un sociologue, historien et militant africain-américain, l’un des plus grands penseurs américains du XXe siècle. Né en 1868 dans le Massachusetts, il étudie à Fisk, à Berlin, puis à Harvard, où il devient en 1895 le premier Africain-Américain à obtenir un doctorat. Son étude &lt;em&gt;The Philadelphia Negro&lt;/em&gt; (1899) est l’une des premières grandes enquêtes de sociologie empirique aux États-Unis.&lt;/p&gt; &lt;p&gt;Dans &lt;a href="https://fr.wikipedia.org/wiki/Les_%C3%82mes_du_peuple_noir" title=" Wikipedia"&gt;&lt;em&gt;Les Âmes du peuple noir&lt;/em&gt;&lt;/a&gt; (1903), il affirme que « le problème du XXe siècle est le problème de la ligne de couleur ». Il y décrit la « double conscience » des Noirs américains : le sentiment de se voir toujours à travers les yeux d’un monde qui les méprise, d’être à la fois américain et noir, « deux âmes, deux pensées, deux combats inconciliables dans un seul corps sombre ». Dans &lt;em&gt;Black Reconstruction&lt;/em&gt; (1935), il réhabilitera le rôle des anciens esclaves dans l’histoire américaine d’après la guerre de Sécession. Il y critique aussi Booker T. Washington, qui conseillait aux Noirs d’accepter la ségrégation en échange du progrès économique.&lt;/p&gt; &lt;p&gt;En 1909, il est l’un des fondateurs de la &lt;a href="https://fr.wikipedia.org/wiki/National_Association_for_the_Advancement_of_Colored_People" title=" Wikipedia"&gt;NAACP&lt;/a&gt;, la grande organisation de défense des droits civiques, dont il dirige la revue &lt;em&gt;The Crisis&lt;/em&gt;. Il organise plusieurs congrès panafricains et devient le « père du &lt;a href="https://fr.wikipedia.org/wiki/Panafricanisme" title=" Wikipedia"&gt;panafricanisme&lt;/a&gt; ». Proche du socialisme, persécuté pendant le maccarthysme, il s’installe à la fin de sa vie au &lt;a href="https://fr.wikipedia.org/wiki/Ghana" title=" Wikipedia"&gt;Ghana&lt;/a&gt;, à l’invitation de Kwame Nkrumah, et y meurt en 1963, à la veille de la marche sur Washington de Martin Luther King.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t xml:space="preserve">mdBvcdTUDRg</t>
+          <t xml:space="preserve">Li9wCyjag3Q</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t xml:space="preserve">"La libération comme espérance chez Gustavo Gutierrez" par Didascale</t>
+          <t xml:space="preserve">"W.E.B. Du Bois : Pionnier des Droits Civiques - Une Conférence par Christian Monjou" par Art et Leadership</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/ggutierrez-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/dubois-mini.webp</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">spiritualite ; politique</t>
+          <t xml:space="preserve">politique ; ethique</t>
         </is>
       </c>
       <c r="K75" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Théologie de la libération</t>
+          <t xml:space="preserve">Pan-africanisme</t>
         </is>
       </c>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">prêtre et théologien péruvien, père de la théologie de la libération et de l’« option préférentielle pour les pauvres ».</t>
+          <t xml:space="preserve">sociologue et militant africain-américain, penseur de la « double conscience » et père du panafricanisme.</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
         </is>
       </c>
       <c r="N75" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">sud</t>
+          <t xml:space="preserve">occident</t>
         </is>
       </c>
       <c r="O75" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Péruvienne</t>
+          <t xml:space="preserve">Américaine</t>
         </is>
       </c>
     </row>
     <row r="76" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="1">
-        <v>1840</v>
+        <v>1928</v>
       </c>
       <c r="B76" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1910</t>
+          <t xml:space="preserve">2024</t>
         </is>
       </c>
       <c r="C76" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1840 – 1910</t>
+          <t xml:space="preserve">1928 – 2024</t>
         </is>
       </c>
       <c r="D76" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">William Graham SUMNER</t>
+          <t xml:space="preserve">Gustavo GUTIÉRREZ</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/William_Graham_Sumner" title=" Wikipedia"&gt;William Graham SUMNER&lt;/a&gt; est un sociologue et économiste américain, l’un des fondateurs de la sociologie aux États-Unis et la figure majeure de ce qu’on appellera le &lt;a href="https://fr.wikipedia.org/wiki/Darwinisme_social" title=" Wikipedia"&gt;darwinisme social&lt;/a&gt; américain. Né en 1840 à Paterson, dans le New Jersey, fils d’un ouvrier anglais immigré, il étudie à Yale, puis en Europe, et devient d’abord pasteur épiscopalien. En 1872, il est nommé professeur à Yale, où il donne l’un des premiers cours intitulés « sociologie ».&lt;/p&gt; &lt;p&gt;Lecteur de Herbert Spencer, il applique à la société l’idée de lutte pour l’existence. Dans &lt;em&gt;Ce que les classes sociales se doivent les unes aux autres&lt;/em&gt; (1883), il répond : rien, sinon le respect de la liberté et des contrats. L’aide de l’État aux pauvres se fait toujours aux dépens de l’« homme oublié », le travailleur modeste qui paie ses impôts sans rien demander. La richesse récompense le travail, l’épargne et la tempérance, et la réussite des plus capables profite à toute la société. Ces positions ont fait de lui, aux yeux de ses critiques, le défenseur d’un capitalisme sans pitié pour les faibles.&lt;/p&gt; &lt;p&gt;Mais il défend aussi le libre-échange contre les monopoles protégés et s’oppose fermement à l’impérialisme : en 1898, il dénonce la guerre contre l’Espagne et la conquête des Philippines dans &lt;em&gt;La Conquête des États-Unis par l’Espagne&lt;/em&gt;. Dans &lt;em&gt;Folkways&lt;/em&gt; (1906), il étudie les coutumes et les mœurs des sociétés, et forge le mot « ethnocentrisme » pour désigner la tendance de chaque groupe à juger les autres d’après ses propres valeurs. Il meurt en 1910.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Gustavo_Guti%C3%A9rrez_Merino" title=" Wikipedia"&gt;Gustavo GUTIÉRREZ&lt;/a&gt; est un prêtre et théologien péruvien, considéré comme le père de la &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9ologie_de_la_lib%C3%A9ration" title=" Wikipedia"&gt;théologie de la libération&lt;/a&gt;. Né à Lima en 1928 dans un milieu modeste, il souffre adolescent d’une ostéomyélite qui le cloue longtemps au lit ; il lit alors beaucoup et commence des études de médecine pour devenir psychiatre. À vingt-quatre ans, il choisit la prêtrise et part étudier la philosophie et la psychologie à Louvain, puis la théologie à Lyon.&lt;/p&gt; &lt;p&gt;Ordonné prêtre en 1959, il devient vicaire dans un quartier pauvre de Lima, tout en enseignant à l’université catholique, et repense toute sa théologie au contact de ce peuple. En 1971, il publie &lt;em&gt;Théologie de la libération&lt;/em&gt;, traduit dans une vingtaine de langues. La pauvreté, écrit-il, n’est pas une fatalité mais le fruit d’injustices, et elle est contraire à la volonté de Dieu. La théologie est une « réflexion critique sur la pratique à la lumière de la Parole » : elle vient en second, après l’engagement aux côtés des pauvres. Le salut ne se joue pas seulement dans l’au-delà ; il touche toute l’existence, et la libération sociale et politique en fait partie, sans s’y réduire. Dans &lt;em&gt;Boire à son propre puits&lt;/em&gt; (1983), il montre que cet engagement est aussi une spiritualité, une manière de suivre le Christ.&lt;/p&gt; &lt;p&gt;Ses positions lui valent la méfiance de Rome dans les années 1980, sans condamnation. Entré chez les Dominicains en 1998, il enseigne dans de nombreuses universités d’Europe et des États-Unis. Le pape François le reçoit en 2013, signe de la réhabilitation de son œuvre, et l’« option préférentielle pour les pauvres » est devenue un principe de l’enseignement de l’Église. Il meurt à Lima en 2024, à quatre-vingt-seize ans.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t xml:space="preserve">r-myUjOJ0qY</t>
+          <t xml:space="preserve">mdBvcdTUDRg</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Folkways by William Graham Sumner" par Sociologylearners</t>
+          <t xml:space="preserve">"La libération comme espérance chez Gustavo Gutierrez" par Didascale</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/sumner-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/ggutierrez-mini.webp</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">politique ; ethique</t>
+          <t xml:space="preserve">spiritualite ; politique</t>
         </is>
       </c>
       <c r="K76" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Darwinisme social ; Libéralisme</t>
+          <t xml:space="preserve">Théologie de la libération</t>
         </is>
       </c>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sociologue américain de Yale, défenseur d’un libéralisme sans État-providence, inventeur du mot « ethnocentrisme ».</t>
+          <t xml:space="preserve">prêtre et théologien péruvien, père de la théologie de la libération et de l’« option préférentielle pour les pauvres ».</t>
         </is>
       </c>
       <c r="N76" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O76" s="1"/>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="O76" s="1">
+        <v>2</v>
+      </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Américaine</t>
+          <t xml:space="preserve">Péruvienne</t>
         </is>
       </c>
     </row>
     <row r="77" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="1">
-        <v>1917</v>
+        <v>1840</v>
       </c>
       <c r="B77" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2003</t>
+          <t xml:space="preserve">1910</t>
         </is>
       </c>
       <c r="C77" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1917 – 2003</t>
+          <t xml:space="preserve">1840 – 1910</t>
         </is>
       </c>
       <c r="D77" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Donald DAVIDSON</t>
+          <t xml:space="preserve">William Graham SUMNER</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Donald_Davidson" title=" Wikipedia"&gt;Donald DAVIDSON&lt;/a&gt; est un philosophe américain, l’un des plus influents de la &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_analytique" title=" Wikipedia"&gt;philosophie analytique&lt;/a&gt; de la seconde moitié du XXe siècle. Né en 1917 à Springfield, dans le Massachusetts, il étudie à Harvard la littérature et les lettres classiques avant de se tourner vers la philosophie sous l’influence de Quine. Après avoir servi dans la marine pendant la guerre, il enseigne notamment à Stanford, à Princeton et à Berkeley.&lt;/p&gt; &lt;p&gt;Dans « Actions, raisons et causes » (1963), il soutient que nos raisons d’agir, nos désirs et nos croyances, sont aussi les causes de nos actions. Dans « Les événements mentaux » (1970), il défend le « monisme anomal » : chaque événement mental est un événement physique, mais il n’existe pas de lois strictes qui relient le mental au physique, car le mental obéit à d’autres principes, ceux de la rationalité. Il réconcilie ainsi le matérialisme avec l’autonomie de la pensée.&lt;/p&gt; &lt;p&gt;Sa théorie de l’« interprétation radicale » prolonge le &lt;a href="https://fr.wikipedia.org/wiki/Holisme" title=" Wikipedia"&gt;holisme&lt;/a&gt; de Quine : pour comprendre un locuteur dont on ignore tout de la langue, il faut lui attribuer en même temps des croyances et des significations, en supposant qu’il pense en grande partie comme nous. C’est le « principe de charité ». Le sens d’un mot dépend du sens de toute la langue, et nos croyances forment un réseau. Il en conclut, dans un article célèbre de 1974, que l’idée de « schèmes conceptuels » radicalement incommensurables n’a pas de sens. Il meurt à Berkeley en 2003.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/William_Graham_Sumner" title=" Wikipedia"&gt;William Graham SUMNER&lt;/a&gt; est un sociologue et économiste américain, l’un des fondateurs de la sociologie aux États-Unis et la figure majeure de ce qu’on appellera le &lt;a href="https://fr.wikipedia.org/wiki/Darwinisme_social" title=" Wikipedia"&gt;darwinisme social&lt;/a&gt; américain. Né en 1840 à Paterson, dans le New Jersey, fils d’un ouvrier anglais immigré, il étudie à Yale, puis en Europe, et devient d’abord pasteur épiscopalien. En 1872, il est nommé professeur à Yale, où il donne l’un des premiers cours intitulés « sociologie ».&lt;/p&gt; &lt;p&gt;Lecteur de Herbert Spencer, il applique à la société l’idée de lutte pour l’existence. Dans &lt;em&gt;Ce que les classes sociales se doivent les unes aux autres&lt;/em&gt; (1883), il répond : rien, sinon le respect de la liberté et des contrats. L’aide de l’État aux pauvres se fait toujours aux dépens de l’« homme oublié », le travailleur modeste qui paie ses impôts sans rien demander. La richesse récompense le travail, l’épargne et la tempérance, et la réussite des plus capables profite à toute la société. Ces positions ont fait de lui, aux yeux de ses critiques, le défenseur d’un capitalisme sans pitié pour les faibles.&lt;/p&gt; &lt;p&gt;Mais il défend aussi le libre-échange contre les monopoles protégés et s’oppose fermement à l’impérialisme : en 1898, il dénonce la guerre contre l’Espagne et la conquête des Philippines dans &lt;em&gt;La Conquête des États-Unis par l’Espagne&lt;/em&gt;. Dans &lt;em&gt;Folkways&lt;/em&gt; (1906), il étudie les coutumes et les mœurs des sociétés, et forge le mot « ethnocentrisme » pour désigner la tendance de chaque groupe à juger les autres d’après ses propres valeurs. Il meurt en 1910.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t xml:space="preserve">ecqO4LMbYvk</t>
+          <t xml:space="preserve">r-myUjOJ0qY</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Donald Davidson Interview: Language, Interpretation, &amp; Philosophy (1993)" par Philosophy Overdose</t>
+          <t xml:space="preserve">"Folkways by William Graham Sumner" par Sociologylearners</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/donalddavidson-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/sumner-mini.webp</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">langage ; epistemologie ; metaphysique</t>
+          <t xml:space="preserve">politique ; ethique</t>
         </is>
       </c>
       <c r="K77" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Holisme ; Analytique</t>
+          <t xml:space="preserve">Darwinisme social ; Libéralisme</t>
         </is>
       </c>
       <c r="L77" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe américain de l’action et du langage, auteur du « monisme anomal ».</t>
+          <t xml:space="preserve">sociologue américain de Yale, défenseur d’un libéralisme sans État-providence, inventeur du mot « ethnocentrisme ».</t>
         </is>
       </c>
       <c r="N77" s="1" t="inlineStr">
@@ -6074,56 +6073,56 @@
     </row>
     <row r="78" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="1">
-        <v>1912</v>
+        <v>1917</v>
       </c>
       <c r="B78" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1989</t>
+          <t xml:space="preserve">2003</t>
         </is>
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1912 – 1989</t>
+          <t xml:space="preserve">1917 – 2003</t>
         </is>
       </c>
       <c r="D78" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wilfrid SELLARS</t>
+          <t xml:space="preserve">Donald DAVIDSON</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Wilfrid_Sellars" title=" Wikipedia"&gt;Wilfrid SELLARS&lt;/a&gt; est un philosophe américain, l’un des plus profonds de la &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_analytique" title=" Wikipedia"&gt;philosophie analytique&lt;/a&gt; du XXe siècle. Né en 1912 à Ann Arbor, fils du philosophe Roy Wood Sellars, il étudie au Michigan, à Buffalo puis à Oxford. Il enseigne au Minnesota, à Yale, et à partir de 1963 à l’université de Pittsburgh, où il fait école. Avec Herbert Feigl, il fonde en 1950 la revue &lt;em&gt;Philosophical Studies&lt;/em&gt;.&lt;/p&gt; &lt;p&gt;Dans « Empirisme et philosophie de l’esprit » (1956), il s’attaque au « mythe du donné » : l’idée, commune aux empiristes, que notre connaissance repose sur des données des sens que nous saisirions immédiatement, sans concepts. Pour Sellars, voir que quelque chose est rouge, c’est déjà savoir ce qu’est le rouge et être capable de le justifier. La connaissance appartient à l’« espace logique des raisons », où l’on donne et demande des justifications, et non à un simple contact causal avec le monde. Même l’observation la plus simple suppose tout un langage et tout un savoir, appris avec lui.&lt;/p&gt; &lt;p&gt;Dans « La philosophie et l’image scientifique de l’homme » (1962), il oppose l’« image manifeste », celle du monde de la vie quotidienne, peuplé de personnes, de couleurs et d’intentions, et l’« image scientifique », faite de particules et de processus. La tâche de la philosophie est de les unir en une seule vision. Pour lui, la science est « la mesure de toutes choses ». Il meurt à Pittsburgh en 1989. Longtemps jugé difficile, il est aujourd’hui l’un des philosophes américains les plus étudiés. Ses idées inspirent Richard Rorty, Robert Brandom et John McDowell.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Donald_Davidson" title=" Wikipedia"&gt;Donald DAVIDSON&lt;/a&gt; est un philosophe américain, l’un des plus influents de la &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_analytique" title=" Wikipedia"&gt;philosophie analytique&lt;/a&gt; de la seconde moitié du XXe siècle. Né en 1917 à Springfield, dans le Massachusetts, il étudie à Harvard la littérature et les lettres classiques avant de se tourner vers la philosophie sous l’influence de Quine. Après avoir servi dans la marine pendant la guerre, il enseigne notamment à Stanford, à Princeton et à Berkeley.&lt;/p&gt; &lt;p&gt;Dans « Actions, raisons et causes » (1963), il soutient que nos raisons d’agir, nos désirs et nos croyances, sont aussi les causes de nos actions. Dans « Les événements mentaux » (1970), il défend le « monisme anomal » : chaque événement mental est un événement physique, mais il n’existe pas de lois strictes qui relient le mental au physique, car le mental obéit à d’autres principes, ceux de la rationalité. Il réconcilie ainsi le matérialisme avec l’autonomie de la pensée.&lt;/p&gt; &lt;p&gt;Sa théorie de l’« interprétation radicale » prolonge le &lt;a href="https://fr.wikipedia.org/wiki/Holisme" title=" Wikipedia"&gt;holisme&lt;/a&gt; de Quine : pour comprendre un locuteur dont on ignore tout de la langue, il faut lui attribuer en même temps des croyances et des significations, en supposant qu’il pense en grande partie comme nous. C’est le « principe de charité ». Le sens d’un mot dépend du sens de toute la langue, et nos croyances forment un réseau. Il en conclut, dans un article célèbre de 1974, que l’idée de « schèmes conceptuels » radicalement incommensurables n’a pas de sens. Il meurt à Berkeley en 2003.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t xml:space="preserve">eJ_0-_NGXQE</t>
+          <t xml:space="preserve">ecqO4LMbYvk</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Wilfrid Sellars : Science et métaphysique (1) - Jacques Bouveresse (2008-2009)" par Lettres, langage, philosophie - Collège de France</t>
+          <t xml:space="preserve">"Donald Davidson Interview: Language, Interpretation, &amp; Philosophy (1993)" par Philosophy Overdose</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/wsellars-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/donalddavidson-mini.webp</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">epistemologie ; metaphysique ; langage</t>
+          <t xml:space="preserve">langage ; epistemologie ; metaphysique</t>
         </is>
       </c>
       <c r="K78" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Analytique ; Réalisme scientifique</t>
+          <t xml:space="preserve">Holisme ; Analytique</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe américain, critique du « mythe du donné » et penseur de l’« image scientifique » de l’homme.</t>
+          <t xml:space="preserve">philosophe américain de l’action et du langage, auteur du « monisme anomal ».</t>
         </is>
       </c>
       <c r="N78" s="1" t="inlineStr">
@@ -6131,9 +6130,7 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
-      <c r="O78" s="1">
-        <v>2</v>
-      </c>
+      <c r="O78" s="1"/>
       <c r="P78" t="inlineStr">
         <is>
           <t xml:space="preserve">Américaine</t>
@@ -6142,56 +6139,56 @@
     </row>
     <row r="79" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="1">
-        <v>1924</v>
+        <v>1912</v>
       </c>
       <c r="B79" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2013</t>
+          <t xml:space="preserve">1989</t>
         </is>
       </c>
       <c r="C79" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1924 – 2013</t>
+          <t xml:space="preserve">1912 – 1989</t>
         </is>
       </c>
       <c r="D79" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arthur DANTO</t>
+          <t xml:space="preserve">Wilfrid SELLARS</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Arthur_Danto" title=" Wikipedia"&gt;Arthur DANTO&lt;/a&gt; est un philosophe et critique d’art américain. Né en 1924 à Ann Arbor, il grandit à Detroit, sert pendant la Seconde Guerre mondiale en Afrique du Nord et en Italie, puis étudie l’art et la philosophie. D’abord graveur, il enseigne à l’université Columbia, à New York, de 1951 à 1992. Ses premiers livres portent sur la philosophie de l’histoire, où il étudie les « phrases narratives », qui décrivent un événement à la lumière de ce qui l’a suivi, et sur Nietzsche, qu’il fait connaître aux philosophes analytiques.&lt;/p&gt; &lt;p&gt;En 1964, il voit exposées les &lt;em&gt;Brillo Boxes&lt;/em&gt; d’Andy Warhol, des boîtes identiques à celles des supermarchés. Pourquoi l’une est-elle une œuvre d’art, et l’autre non, alors qu’on ne peut pas les distinguer à l’œil ? Dans l’article « Le monde de l’art », il répond que ce qui fait l’œuvre n’est pas une propriété visible, mais une théorie et une histoire de l’art, une atmosphère que seul connaît ce « monde de l’art ». Dans &lt;em&gt;La Transfiguration du banal&lt;/em&gt; (1981), il précise : une œuvre d’art est toujours à propos de quelque chose, et elle incarne ce sens, ce qui la distingue d’une simple chose.&lt;/p&gt; &lt;p&gt;Il en tire en 1984 la thèse de la « fin de l’art » : non que l’on cesse de créer, mais l’art, depuis Warhol, n’a plus d’histoire orientée, et tout est désormais possible. C’est à la &lt;a href="https://fr.wikipedia.org/wiki/Esth%C3%A9tique" title=" Wikipedia"&gt;philosophie&lt;/a&gt;, et non plus à l’art, de dire ce qu’est l’art. Critique d’art à l’hebdomadaire &lt;em&gt;The Nation&lt;/em&gt; de 1984 à 2009, il est l’un des esthéticiens les plus lus de son temps. Il meurt à New York en 2013.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Wilfrid_Sellars" title=" Wikipedia"&gt;Wilfrid SELLARS&lt;/a&gt; est un philosophe américain, l’un des plus profonds de la &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_analytique" title=" Wikipedia"&gt;philosophie analytique&lt;/a&gt; du XXe siècle. Né en 1912 à Ann Arbor, fils du philosophe Roy Wood Sellars, il étudie au Michigan, à Buffalo puis à Oxford. Il enseigne au Minnesota, à Yale, et à partir de 1963 à l’université de Pittsburgh, où il fait école. Avec Herbert Feigl, il fonde en 1950 la revue &lt;em&gt;Philosophical Studies&lt;/em&gt;.&lt;/p&gt; &lt;p&gt;Dans « Empirisme et philosophie de l’esprit » (1956), il s’attaque au « mythe du donné » : l’idée, commune aux empiristes, que notre connaissance repose sur des données des sens que nous saisirions immédiatement, sans concepts. Pour Sellars, voir que quelque chose est rouge, c’est déjà savoir ce qu’est le rouge et être capable de le justifier. La connaissance appartient à l’« espace logique des raisons », où l’on donne et demande des justifications, et non à un simple contact causal avec le monde. Même l’observation la plus simple suppose tout un langage et tout un savoir, appris avec lui.&lt;/p&gt; &lt;p&gt;Dans « La philosophie et l’image scientifique de l’homme » (1962), il oppose l’« image manifeste », celle du monde de la vie quotidienne, peuplé de personnes, de couleurs et d’intentions, et l’« image scientifique », faite de particules et de processus. La tâche de la philosophie est de les unir en une seule vision. Pour lui, la science est « la mesure de toutes choses ». Il meurt à Pittsburgh en 1989. Longtemps jugé difficile, il est aujourd’hui l’un des philosophes américains les plus étudiés. Ses idées inspirent Richard Rorty, Robert Brandom et John McDowell.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t xml:space="preserve">3xVufNOZPqE</t>
+          <t xml:space="preserve">eJ_0-_NGXQE</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Arthur Danto: La transfiguration du banal. Une philosophie de l'art." par Jtgrandtour</t>
+          <t xml:space="preserve">"Wilfrid Sellars : Science et métaphysique (1) - Jacques Bouveresse (2008-2009)" par Lettres, langage, philosophie - Collège de France</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/danto-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/wsellars-mini.webp</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">esthetique ; epistemologie</t>
+          <t xml:space="preserve">epistemologie ; metaphysique ; langage</t>
         </is>
       </c>
       <c r="K79" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Analytique</t>
+          <t xml:space="preserve">Analytique ; Réalisme scientifique</t>
         </is>
       </c>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe et critique d’art américain, théoricien du « monde de l’art » et de la fin de l’art.</t>
+          <t xml:space="preserve">philosophe américain, critique du « mythe du donné » et penseur de l’« image scientifique » de l’homme.</t>
         </is>
       </c>
       <c r="N79" s="1" t="inlineStr">
@@ -6210,56 +6207,56 @@
     </row>
     <row r="80" customFormat="false" ht="242.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="1">
-        <v>1929</v>
+        <v>1924</v>
       </c>
       <c r="B80" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2023</t>
+          <t xml:space="preserve">2013</t>
         </is>
       </c>
       <c r="C80" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1929 – 2023</t>
+          <t xml:space="preserve">1924 – 2013</t>
         </is>
       </c>
       <c r="D80" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Harry FRANKFURT</t>
+          <t xml:space="preserve">Arthur DANTO</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Harry_Frankfurt" title=" Wikipedia"&gt;Harry FRANKFURT&lt;/a&gt; est un philosophe américain. Né en 1929 à Langhorne, en Pennsylvanie, il étudie à l’université Johns-Hopkins et enseigne à l’université Rockefeller, à Yale, puis à Princeton jusqu’en 2002. Spécialiste de Descartes, il devient surtout l’un des penseurs majeurs de la liberté, de la responsabilité et de la personne, dans un style d’une grande clarté.&lt;/p&gt; &lt;p&gt;En 1969, il imagine des cas, appelés depuis « cas de Frankfurt », pour contester l’idée qu’on n’est responsable d’un acte que si l’on aurait pu agir autrement. Un neurologue malveillant est prêt à intervenir dans le cerveau de Jones pour le forcer à agir, mais Jones fait de lui-même ce qu’on attendait, sans intervention : il est responsable, bien qu’il n’ait pas eu d’autre possibilité. En 1971, il définit la personne par les « désirs de second ordre » : nous ne voulons pas seulement des choses, nous voulons aussi avoir ou ne pas avoir certains désirs. Être libre, c’est agir selon les désirs que l’on approuve. Ces idées font de lui l’un des grands défenseurs du &lt;a href="https://fr.wikipedia.org/wiki/Compatibilisme" title=" Wikipedia"&gt;compatibilisme&lt;/a&gt;.&lt;/p&gt; &lt;p&gt;Son petit essai &lt;em&gt;De l’art de dire des conneries&lt;/em&gt;, écrit en 1986 et publié en livre en 2005, devient un best-seller : le baratineur est plus dangereux que le menteur, car le menteur se soucie encore de la vérité pour la cacher, alors que le baratineur y est indifférent. Dans &lt;em&gt;Les Raisons de l’amour&lt;/em&gt; (2004), il montre que c’est ce que nous aimons qui donne sens à notre vie. Dans &lt;em&gt;On Inequality&lt;/em&gt; (2015), il soutient que l’important n’est pas que chacun ait autant, mais que chacun ait assez. Il meurt à Santa Monica en 2023.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Arthur_Danto" title=" Wikipedia"&gt;Arthur DANTO&lt;/a&gt; est un philosophe et critique d’art américain. Né en 1924 à Ann Arbor, il grandit à Detroit, sert pendant la Seconde Guerre mondiale en Afrique du Nord et en Italie, puis étudie l’art et la philosophie. D’abord graveur, il enseigne à l’université Columbia, à New York, de 1951 à 1992. Ses premiers livres portent sur la philosophie de l’histoire, où il étudie les « phrases narratives », qui décrivent un événement à la lumière de ce qui l’a suivi, et sur Nietzsche, qu’il fait connaître aux philosophes analytiques.&lt;/p&gt; &lt;p&gt;En 1964, il voit exposées les &lt;em&gt;Brillo Boxes&lt;/em&gt; d’Andy Warhol, des boîtes identiques à celles des supermarchés. Pourquoi l’une est-elle une œuvre d’art, et l’autre non, alors qu’on ne peut pas les distinguer à l’œil ? Dans l’article « Le monde de l’art », il répond que ce qui fait l’œuvre n’est pas une propriété visible, mais une théorie et une histoire de l’art, une atmosphère que seul connaît ce « monde de l’art ». Dans &lt;em&gt;La Transfiguration du banal&lt;/em&gt; (1981), il précise : une œuvre d’art est toujours à propos de quelque chose, et elle incarne ce sens, ce qui la distingue d’une simple chose.&lt;/p&gt; &lt;p&gt;Il en tire en 1984 la thèse de la « fin de l’art » : non que l’on cesse de créer, mais l’art, depuis Warhol, n’a plus d’histoire orientée, et tout est désormais possible. C’est à la &lt;a href="https://fr.wikipedia.org/wiki/Esth%C3%A9tique" title=" Wikipedia"&gt;philosophie&lt;/a&gt;, et non plus à l’art, de dire ce qu’est l’art. Critique d’art à l’hebdomadaire &lt;em&gt;The Nation&lt;/em&gt; de 1984 à 2009, il est l’un des esthéticiens les plus lus de son temps. Il meurt à New York en 2013.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t xml:space="preserve">FXewQRCpKAs</t>
+          <t xml:space="preserve">3xVufNOZPqE</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t xml:space="preserve">"La Rhétorique Toxique et le Bullshit - Harry.G.Frankfurt" par MLHORION</t>
+          <t xml:space="preserve">"Arthur Danto: La transfiguration du banal. Une philosophie de l'art." par Jtgrandtour</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/frankfurt-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/danto-mini.webp</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ethique ; metaphysique</t>
+          <t xml:space="preserve">esthetique ; epistemologie</t>
         </is>
       </c>
       <c r="K80" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compatibilisme</t>
+          <t xml:space="preserve">Analytique</t>
         </is>
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe américain de la liberté et de la personne, auteur de « De l’art de dire des conneries ».</t>
+          <t xml:space="preserve">philosophe et critique d’art américain, théoricien du « monde de l’art » et de la fin de l’art.</t>
         </is>
       </c>
       <c r="N80" s="1" t="inlineStr">
@@ -6282,52 +6279,65 @@
       </c>
       <c r="B81" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024</t>
+          <t xml:space="preserve">2023</t>
         </is>
       </c>
       <c r="C81" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1929 – 2024</t>
+          <t xml:space="preserve">1929 – 2023</t>
         </is>
       </c>
       <c r="D81" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Newton DA COSTA</t>
+          <t xml:space="preserve">Harry FRANKFURT</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Newton_da_Costa" title=" Wikipedia (en)"&gt;Newton DA COSTA&lt;/a&gt; est un logicien et philosophe brésilien, l’un des fondateurs de la &lt;a href="https://fr.wikipedia.org/wiki/Logique_paraconsistante" title=" Wikipedia"&gt;logique paraconsistante&lt;/a&gt;. Né en 1929 à Curitiba, il étudie d’abord le génie civil puis les mathématiques, et enseigne à l’université fédérale du Paraná, puis à l’université de São Paulo et à l’université fédérale de Santa Catarina.&lt;/p&gt; &lt;p&gt;Dans la logique classique, une seule contradiction suffit à tout prouver : si l’on admet à la fois une proposition et sa négation, on peut en déduire n’importe quoi. C’est le principe d’« explosion ». Dès sa thèse de 1963, da Costa construit des systèmes logiques, appelés « calculs C », où l’on peut admettre certaines contradictions sans que toute la théorie s’effondre. Le nom de « paraconsistance » leur est donné en 1976 par le philosophe péruvien Francisco Miró Quesada. Ces logiques permettent de raisonner rigoureusement sur des informations contradictoires, comme celles d’une base de données, d’un témoignage ou d’une théorie scientifique en crise.&lt;/p&gt; &lt;p&gt;Da Costa étend ces travaux à la théorie des ensembles et à la philosophie des sciences. Avec Steven French, il développe la notion de « quasi-vérité » : une théorie scientifique peut être partiellement vraie et utile sans être entièrement exacte. Avec Francisco Antônio Dória, il montre en 1991 que certaines questions de la théorie du chaos sont indécidables : aucun calcul ne peut y répondre. Membre de nombreuses académies, il a formé une importante école de logique au Brésil et en Amérique latine. Il meurt en 2024 à Florianópolis.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Harry_Frankfurt" title=" Wikipedia"&gt;Harry FRANKFURT&lt;/a&gt; est un philosophe américain. Né en 1929 à Langhorne, en Pennsylvanie, il étudie à l’université Johns-Hopkins et enseigne à l’université Rockefeller, à Yale, puis à Princeton jusqu’en 2002. Spécialiste de Descartes, il devient surtout l’un des penseurs majeurs de la liberté, de la responsabilité et de la personne, dans un style d’une grande clarté.&lt;/p&gt; &lt;p&gt;En 1969, il imagine des cas, appelés depuis « cas de Frankfurt », pour contester l’idée qu’on n’est responsable d’un acte que si l’on aurait pu agir autrement. Un neurologue malveillant est prêt à intervenir dans le cerveau de Jones pour le forcer à agir, mais Jones fait de lui-même ce qu’on attendait, sans intervention : il est responsable, bien qu’il n’ait pas eu d’autre possibilité. En 1971, il définit la personne par les « désirs de second ordre » : nous ne voulons pas seulement des choses, nous voulons aussi avoir ou ne pas avoir certains désirs. Être libre, c’est agir selon les désirs que l’on approuve. Ces idées font de lui l’un des grands défenseurs du &lt;a href="https://fr.wikipedia.org/wiki/Compatibilisme" title=" Wikipedia"&gt;compatibilisme&lt;/a&gt;.&lt;/p&gt; &lt;p&gt;Son petit essai &lt;em&gt;De l’art de dire des conneries&lt;/em&gt;, écrit en 1986 et publié en livre en 2005, devient un best-seller : le baratineur est plus dangereux que le menteur, car le menteur se soucie encore de la vérité pour la cacher, alors que le baratineur y est indifférent. Dans &lt;em&gt;Les Raisons de l’amour&lt;/em&gt; (2004), il montre que c’est ce que nous aimons qui donne sens à notre vie. Dans &lt;em&gt;On Inequality&lt;/em&gt; (2015), il soutient que l’important n’est pas que chacun ait autant, mais que chacun ait assez. Il meurt à Santa Monica en 2023.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FXewQRCpKAs</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"La Rhétorique Toxique et le Bullshit - Harry.G.Frankfurt" par MLHORION</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/dacosta-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/frankfurt-mini.webp</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">logique ; epistemologie</t>
+          <t xml:space="preserve">ethique ; metaphysique</t>
         </is>
       </c>
       <c r="K81" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Logique paraconsistante</t>
+          <t xml:space="preserve">Compatibilisme</t>
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">logicien brésilien, l’un des fondateurs des logiques paraconsistantes.</t>
+          <t xml:space="preserve">philosophe américain de la liberté et de la personne, auteur de « De l’art de dire des conneries ».</t>
         </is>
       </c>
       <c r="N81" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">sud</t>
-        </is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O81" s="1">
+        <v>2</v>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brésilienne</t>
+          <t xml:space="preserve">Américaine</t>
         </is>
       </c>
     </row>
@@ -6970,17 +6980,17 @@
     <hyperlink ref="H40" r:id="rId25" display="https://www.laphilo.fr/pho/scavell-mini.webp"/>
     <hyperlink ref="H41" r:id="rId26" display="https://www.laphilo.fr/pho/mrothbard-mini.webp"/>
     <hyperlink ref="H42" r:id="rId27" display="https://www.laphilo.fr/pho/ewiesel-mini.webp"/>
-    <hyperlink ref="H43" r:id="rId28" display="https://www.laphilo.fr/pho/abracken-mini.webp"/>
-    <hyperlink ref="E45" r:id="rId29" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Richard_Rorty&quot; title=&quot; Wikipedia&quot;&gt;Richard RORTY&lt;/a&gt; était un  philosophe américain, figure majeure du  &lt;a href=&quot;https://www.youtube.com/watch?v=lfx4Jag1ic4&quot;  title=&quot;Le pragmatisme : définition, exemples par le savoir partagé&quot;&gt;pragmatisme&lt;/a&gt; et du postmodernisme, il a remis en cause les fondements de la philosophie occidentale et proposé une &lt;a href=&quot;https://laviedesidees.fr/Rorty-Pragmatism-Anti-Authoritarianism&quot; title=&quot; a bas l'autorité par laviedesidees&quot;&gt;vision radicale&lt;/a&gt;  de la vérité, de la culture et de la société. Il rejette l'idée que la vérité soit une correspondance entre le langage et la réalité. Pour lui, la vérité est simplement ce qui est utile ou avantageux à croire dans une communauté donnée et il propose d'abandonner la quête de fondements absolus de la connaissance, jugée vaine. &lt;/p&gt; &lt;p&gt; Inspiré par Wittgenstein et Davidson, il considère le langage non pas comme un miroir de la réalité, mais comme un ensemble d'outils pour résoudre des problèmes pratiques.  Les vocabularies que nous utilisons sont historiquement et culturellement contingents, non pas &quot;vrais&quot; ou &quot;faux&quot;. &lt;/p&gt; &lt;p&gt; Dans ces oeuvres principales , on trouve  &lt;a href=&quot;https://www.youtube.com/watch?v=MgU0dXZ3umM&quot; title=&quot;L’ironiste libéral chez Rorty : Contingence, ironie et solidarité par Darina Metreveli&quot;&gt;&quot; Contingence, ironie et solidarité &quot;&lt;/a&gt; (1989) ou il décrit l'ironiste comme quelqu'un qui doute de ses propres croyances tout en œuvrant pour une société plus juste. Dans &quot; Achieving Our Country&quot; (1998),  il y appelle la gauche américaine à abandonner le &quot;culturalisme&quot; pour se recentrer sur les inégalités économiques et sociales. Cet ouvrage est souvent cité pour avoir anticipé les crises politiques du XXIe siècle. &lt;/p&gt; &lt;p&gt;  Ses thèses sur la contingence de la vérité sont souvent invoquées pour analyser l'ère de la &quot;post-vérité&quot;. Son insistance sur la conversation comme fondement du lien social influence la philosophie politique contemporaine. Il  a bouleversé la philosophie en démystifiant ses prétentions à la vérité absolue. Son œuvre, à la fois provocante et humaniste, invite à remplacer la quête métaphysique par un engagement en faveur d'une société plus juste et plus inclusive. &lt;/p&gt; "/>
-    <hyperlink ref="E47" r:id="rId30" display="&lt;p&gt;&lt;a href=&quot;https://en.wikipedia.org/wiki/Charles_Parsons_(philosopher)&quot;  title=&quot; Wikipedia&quot;&gt;Charles Dacre PARSONS&lt;/a&gt; était un philosophe américain connu pour ses travaux en philosophie des mathématiques et en philosophie de Kant. Il a enseigné à Columbia puis à Harvard, où il est devenu professeur émérite. Il s’est formé à Harvard, avec une thèse dirigée par Willard Van Orman Quine, ce qui le place au croisement de la logique, de la philosophie analytique et des fondements des mathématiques. Son parcours intellectuel a été marqué très tôt par la rigueur mathématique, puisqu’il avait d’abord étudié les mathématiques avant de se tourner vers la philosophie. &lt;/p&gt; &lt;p&gt; Son apport principal concerne la philosophie des mathématiques, domaine dans lequel il a travaillé sur la nature des objets mathématiques, la logique, la preuve et l’interprétation constructive des mathématiques prédicatives. Il a aussi beaucoup écrit sur Frege, Gödel, Hilbert et Quine, en lisant ces auteurs à la fois comme philosophes et comme figures majeures des fondements. &lt;/p&gt; &lt;p&gt; Il n’était pas seulement un spécialiste de logique ; il a aussi produit des travaux importants sur Kant, montrant comment les questions de connaissance, d’expérience et de structure de l’esprit se relient aux mathématiques. Cette double compétence, en philosophie des mathématiques et en histoire de la philosophie, explique pourquoi il est souvent vu comme un auteur à la fois technique et très large dans ses intérêts.&lt;/p&gt; &lt;p&gt; Son influence est restée forte dans le monde anglophone, au point d’être décrit comme l’un des philosophes des mathématiques les plus importants de sa génération. En plus de ses livres et articles, il a aussi contribué à l’édition de textes posthumes de Gödel, ce qui a renforcé son rôle dans l’étude contemporaine des fondements des mathématiques. &lt;/p&gt; &#10;&#10;&#10;"/>
-    <hyperlink ref="I47" r:id="rId31" display="https://www.laphilo.fr/photo/cparsons.webp"/>
-    <hyperlink ref="H49" r:id="rId32" display="https://www.laphilo.fr/pho/dihde-mini.webp"/>
-    <hyperlink ref="E51" r:id="rId33" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Edward_Sa%C3%AFd&quot;  title=&quot; Wikipedia&quot;&gt;Edward SAÏD&lt;/a&gt; était un intellectuel palestinien-américain, critique littéraire et professeur de littérature anglaise et comparée à l’université Columbia de New York. D’origine palestinienne et né à Jérusalem, il a grandi entre l’Égypte, les États-Unis et l’Europe, une expérience de déplacement qui a profondément marqué sa pensée sur l’identité, la colonisation et l’altérité.  &lt;/p&gt; &lt;p&gt; Sa contribution la plus célèbre est l’essai &lt;a href=&quot;https://www.youtube.com/watch?v=Ne4WRykmjhA&quot; title=&quot;Edward Said  Orientalisme par HD Doc&quot;&gt;L’Orientalisme : &lt;/a&gt;  L’Orient créé par l’Occident* (1978), considéré comme le texte fondateur des postcolonial studies. Dans cet ouvrage, Saïd montre que l’« Orient » n’est pas une réalité objective mais une invention de l’Occident : un discours façonné par des siècles de domination coloniale pour mieux contrôler et représenter l’Autre. &lt;/p&gt; &lt;p&gt; Pour lui, l’orientalisme est à la fois un savoir et un outil de pouvoir : il ne s’agit pas seulement de décrire l’Orient, mais de le hiérarchiser, de l’essentialiser et de le rendre  &lt;a href=&quot;https://www.youtube.com/watch?v=QBj-yWLnayM&quot; title=&quot;Edward Said writings on Orientalism par Middle East Eye&quot;&gt; inférieur à l’Occident. &lt;/a&gt; Il analyse quatre thèses principales : la domination politique et culturelle de l’Orient par l’Occident, la dépréciation de la langue arabe, la diabolisation de l’arabe et de l’islam, et la défense de la cause palestinienne. &lt;/p&gt; &lt;p&gt; Sa pensée articule critique littéraire, histoire, philosophie et sciences politiques, en s’inspirant notamment de Michel Foucault (discours–pouvoir) et de Jacques Derrida (déconstruction). Il montre que la violence du colonialisme n’est pas seulement matérielle (conquête, pillage), mais aussi épistémique : une violence de la raison qui classe, essentialise et dévalue les « Autres » de l’Occident. &lt;/p&gt; &lt;p&gt;  Intéressé par &lt;a href=&quot;https://www.lesclesdumoyenorient.com/Edward-W-Said-1935-2003.html&quot; title=&quot;Edward Said par lesclesdumoyenorient&quot;&gt; l’engagement politique, &lt;/a&gt; il a aussi défendu la cause palestinienne et la légitimité des revendications d’autodétermination du peuple palestinien, tout en reconnaissance du droit à une patrie juive. Il rejetait le repli identitaire et prônait une vision universelle qui défend les différences et les droits, tissant des liens entre classicisme et excentricité, histoire et actualité. &lt;/p&gt;  &lt;audio controls title=&quot;Edward Said, une conscience morale par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/12360-08.12.2017-ITEMA_21518070-2017C19327S0342-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;  &#10;&#10;&#10;"/>
-    <hyperlink ref="H51" r:id="rId34" display="https://laphilo.fr/pho/esaid-mini.webp"/>
-    <hyperlink ref="H52" r:id="rId35" display="https://www.laphilo.fr/pho/rmadams-mini.webp"/>
-    <hyperlink ref="E53" r:id="rId36" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Robert_Nozick&quot;  title=&quot; Wikipedia&quot;&gt;Robert NOZICK&lt;/a&gt; était un philosophe américain connu pour &lt;a href=&quot;https://www.youtube.com/watch?v=Q-t3cpFAk4o&quot;  title=&quot; Libertarianisme par Vadim Media&quot;&gt; son libertarianisme &lt;/a&gt; et sa critique des théories égalitaristes comme celle de John Rawls. Professeur à Harvard, il a marqué la philosophie politique, morale et épistémologique par son œuvre principale, Anarchie, État et utopie (1974), qui défend un  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Minarchisme&quot;  title=&quot; Minarchisme par Wikipédia&quot;&gt; Etat Minimal. &lt;/a&gt; &lt;/p&gt; &lt;p&gt; Il argue que seul l'État minimal, ou &quot;État gardien de nuit&quot;, est légitime, car il se limite à protéger les individus contre la force, la fraude et le vol, sans redistribuer les richesses. Il rejette l'anarcho-capitalisme en montrant, via des agences de protection privée, comment un État dominant émerge naturellement pour monopoliser la coercition légitime, justifié par le droit naturel à la personne. &lt;/p&gt; &lt;p&gt; Contrairement à la justice distributive de Rawls, il propose une théorie de l'entitlement : une acquisition initiale juste et des transferts volontaires rendent la distribution légitime, sans besoin d'égalisation par l'État. Toute intervention redistributive viole les droits individuels, traitant les personnes comme des moyens plutôt que des fins, en écho à Kant. &lt;/p&gt; &lt;p&gt; Dans Anarchie, État et utopie, Il réfute l'utilitarisme via l'expérience de pensée de la &lt;a href=&quot;https://www.youtube.com/watch?v=2FVwXaNWPQ0&quot;  title=&quot; La machine à expérience par Monsieur Phi&quot;&gt;&quot;machine à expérience&quot; :&lt;/a&gt;  même si elle offre un bonheur parfait et indistinguable de la réalité, les gens préfèrent vivre des actions réelles et façonner leur identité plutôt que des simulations. Cela prouve que le bonheur n'est pas le seul bien suprême. &lt;/p&gt; &lt;p&gt; Plus tard, dans Explications philosophiques (1981), il développe une théorie du suivi (tracking theory) en épistémologie, où la connaissance repose sur des conditionnels contrefactuels fiables, contournant le scepticisme sans justification traditionnelle. Son anti-coercitivisme intellectuel invite à une philosophie ouverte, non imposée. &lt;/p&gt; &#10;&lt;audio controls title=&quot;Qui a peur des Libertariens par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10467-14.06.2022-ITEMA_23058436-2022C12410S0165-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt;&lt;/audio&gt;&#10;"/>
-    <hyperlink ref="H59" r:id="rId37" display="https://www.laphilo.fr/pho/imyoung-mini.webp"/>
-    <hyperlink ref="H60" r:id="rId38" display="https://www.laphilo.fr/pho/bhooks-mini.webp"/>
+    <hyperlink ref="H44" r:id="rId28" display="https://www.laphilo.fr/pho/abracken-mini.webp"/>
+    <hyperlink ref="E46" r:id="rId29" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Richard_Rorty&quot; title=&quot; Wikipedia&quot;&gt;Richard RORTY&lt;/a&gt; était un  philosophe américain, figure majeure du  &lt;a href=&quot;https://www.youtube.com/watch?v=lfx4Jag1ic4&quot;  title=&quot;Le pragmatisme : définition, exemples par le savoir partagé&quot;&gt;pragmatisme&lt;/a&gt; et du postmodernisme, il a remis en cause les fondements de la philosophie occidentale et proposé une &lt;a href=&quot;https://laviedesidees.fr/Rorty-Pragmatism-Anti-Authoritarianism&quot; title=&quot; a bas l'autorité par laviedesidees&quot;&gt;vision radicale&lt;/a&gt;  de la vérité, de la culture et de la société. Il rejette l'idée que la vérité soit une correspondance entre le langage et la réalité. Pour lui, la vérité est simplement ce qui est utile ou avantageux à croire dans une communauté donnée et il propose d'abandonner la quête de fondements absolus de la connaissance, jugée vaine. &lt;/p&gt; &lt;p&gt; Inspiré par Wittgenstein et Davidson, il considère le langage non pas comme un miroir de la réalité, mais comme un ensemble d'outils pour résoudre des problèmes pratiques.  Les vocabularies que nous utilisons sont historiquement et culturellement contingents, non pas &quot;vrais&quot; ou &quot;faux&quot;. &lt;/p&gt; &lt;p&gt; Dans ces oeuvres principales , on trouve  &lt;a href=&quot;https://www.youtube.com/watch?v=MgU0dXZ3umM&quot; title=&quot;L’ironiste libéral chez Rorty : Contingence, ironie et solidarité par Darina Metreveli&quot;&gt;&quot; Contingence, ironie et solidarité &quot;&lt;/a&gt; (1989) ou il décrit l'ironiste comme quelqu'un qui doute de ses propres croyances tout en œuvrant pour une société plus juste. Dans &quot; Achieving Our Country&quot; (1998),  il y appelle la gauche américaine à abandonner le &quot;culturalisme&quot; pour se recentrer sur les inégalités économiques et sociales. Cet ouvrage est souvent cité pour avoir anticipé les crises politiques du XXIe siècle. &lt;/p&gt; &lt;p&gt;  Ses thèses sur la contingence de la vérité sont souvent invoquées pour analyser l'ère de la &quot;post-vérité&quot;. Son insistance sur la conversation comme fondement du lien social influence la philosophie politique contemporaine. Il  a bouleversé la philosophie en démystifiant ses prétentions à la vérité absolue. Son œuvre, à la fois provocante et humaniste, invite à remplacer la quête métaphysique par un engagement en faveur d'une société plus juste et plus inclusive. &lt;/p&gt; "/>
+    <hyperlink ref="E48" r:id="rId30" display="&lt;p&gt;&lt;a href=&quot;https://en.wikipedia.org/wiki/Charles_Parsons_(philosopher)&quot;  title=&quot; Wikipedia&quot;&gt;Charles Dacre PARSONS&lt;/a&gt; était un philosophe américain connu pour ses travaux en philosophie des mathématiques et en philosophie de Kant. Il a enseigné à Columbia puis à Harvard, où il est devenu professeur émérite. Il s’est formé à Harvard, avec une thèse dirigée par Willard Van Orman Quine, ce qui le place au croisement de la logique, de la philosophie analytique et des fondements des mathématiques. Son parcours intellectuel a été marqué très tôt par la rigueur mathématique, puisqu’il avait d’abord étudié les mathématiques avant de se tourner vers la philosophie. &lt;/p&gt; &lt;p&gt; Son apport principal concerne la philosophie des mathématiques, domaine dans lequel il a travaillé sur la nature des objets mathématiques, la logique, la preuve et l’interprétation constructive des mathématiques prédicatives. Il a aussi beaucoup écrit sur Frege, Gödel, Hilbert et Quine, en lisant ces auteurs à la fois comme philosophes et comme figures majeures des fondements. &lt;/p&gt; &lt;p&gt; Il n’était pas seulement un spécialiste de logique ; il a aussi produit des travaux importants sur Kant, montrant comment les questions de connaissance, d’expérience et de structure de l’esprit se relient aux mathématiques. Cette double compétence, en philosophie des mathématiques et en histoire de la philosophie, explique pourquoi il est souvent vu comme un auteur à la fois technique et très large dans ses intérêts.&lt;/p&gt; &lt;p&gt; Son influence est restée forte dans le monde anglophone, au point d’être décrit comme l’un des philosophes des mathématiques les plus importants de sa génération. En plus de ses livres et articles, il a aussi contribué à l’édition de textes posthumes de Gödel, ce qui a renforcé son rôle dans l’étude contemporaine des fondements des mathématiques. &lt;/p&gt; &#10;&#10;&#10;"/>
+    <hyperlink ref="I48" r:id="rId31" display="https://www.laphilo.fr/photo/cparsons.webp"/>
+    <hyperlink ref="H50" r:id="rId32" display="https://www.laphilo.fr/pho/dihde-mini.webp"/>
+    <hyperlink ref="E52" r:id="rId33" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Edward_Sa%C3%AFd&quot;  title=&quot; Wikipedia&quot;&gt;Edward SAÏD&lt;/a&gt; était un intellectuel palestinien-américain, critique littéraire et professeur de littérature anglaise et comparée à l’université Columbia de New York. D’origine palestinienne et né à Jérusalem, il a grandi entre l’Égypte, les États-Unis et l’Europe, une expérience de déplacement qui a profondément marqué sa pensée sur l’identité, la colonisation et l’altérité.  &lt;/p&gt; &lt;p&gt; Sa contribution la plus célèbre est l’essai &lt;a href=&quot;https://www.youtube.com/watch?v=Ne4WRykmjhA&quot; title=&quot;Edward Said  Orientalisme par HD Doc&quot;&gt;L’Orientalisme : &lt;/a&gt;  L’Orient créé par l’Occident* (1978), considéré comme le texte fondateur des postcolonial studies. Dans cet ouvrage, Saïd montre que l’« Orient » n’est pas une réalité objective mais une invention de l’Occident : un discours façonné par des siècles de domination coloniale pour mieux contrôler et représenter l’Autre. &lt;/p&gt; &lt;p&gt; Pour lui, l’orientalisme est à la fois un savoir et un outil de pouvoir : il ne s’agit pas seulement de décrire l’Orient, mais de le hiérarchiser, de l’essentialiser et de le rendre  &lt;a href=&quot;https://www.youtube.com/watch?v=QBj-yWLnayM&quot; title=&quot;Edward Said writings on Orientalism par Middle East Eye&quot;&gt; inférieur à l’Occident. &lt;/a&gt; Il analyse quatre thèses principales : la domination politique et culturelle de l’Orient par l’Occident, la dépréciation de la langue arabe, la diabolisation de l’arabe et de l’islam, et la défense de la cause palestinienne. &lt;/p&gt; &lt;p&gt; Sa pensée articule critique littéraire, histoire, philosophie et sciences politiques, en s’inspirant notamment de Michel Foucault (discours–pouvoir) et de Jacques Derrida (déconstruction). Il montre que la violence du colonialisme n’est pas seulement matérielle (conquête, pillage), mais aussi épistémique : une violence de la raison qui classe, essentialise et dévalue les « Autres » de l’Occident. &lt;/p&gt; &lt;p&gt;  Intéressé par &lt;a href=&quot;https://www.lesclesdumoyenorient.com/Edward-W-Said-1935-2003.html&quot; title=&quot;Edward Said par lesclesdumoyenorient&quot;&gt; l’engagement politique, &lt;/a&gt; il a aussi défendu la cause palestinienne et la légitimité des revendications d’autodétermination du peuple palestinien, tout en reconnaissance du droit à une patrie juive. Il rejetait le repli identitaire et prônait une vision universelle qui défend les différences et les droits, tissant des liens entre classicisme et excentricité, histoire et actualité. &lt;/p&gt;  &lt;audio controls title=&quot;Edward Said, une conscience morale par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/12360-08.12.2017-ITEMA_21518070-2017C19327S0342-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;  &#10;&#10;&#10;"/>
+    <hyperlink ref="H52" r:id="rId34" display="https://laphilo.fr/pho/esaid-mini.webp"/>
+    <hyperlink ref="H53" r:id="rId35" display="https://www.laphilo.fr/pho/rmadams-mini.webp"/>
+    <hyperlink ref="E54" r:id="rId36" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Robert_Nozick&quot;  title=&quot; Wikipedia&quot;&gt;Robert NOZICK&lt;/a&gt; était un philosophe américain connu pour &lt;a href=&quot;https://www.youtube.com/watch?v=Q-t3cpFAk4o&quot;  title=&quot; Libertarianisme par Vadim Media&quot;&gt; son libertarianisme &lt;/a&gt; et sa critique des théories égalitaristes comme celle de John Rawls. Professeur à Harvard, il a marqué la philosophie politique, morale et épistémologique par son œuvre principale, Anarchie, État et utopie (1974), qui défend un  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Minarchisme&quot;  title=&quot; Minarchisme par Wikipédia&quot;&gt; Etat Minimal. &lt;/a&gt; &lt;/p&gt; &lt;p&gt; Il argue que seul l'État minimal, ou &quot;État gardien de nuit&quot;, est légitime, car il se limite à protéger les individus contre la force, la fraude et le vol, sans redistribuer les richesses. Il rejette l'anarcho-capitalisme en montrant, via des agences de protection privée, comment un État dominant émerge naturellement pour monopoliser la coercition légitime, justifié par le droit naturel à la personne. &lt;/p&gt; &lt;p&gt; Contrairement à la justice distributive de Rawls, il propose une théorie de l'entitlement : une acquisition initiale juste et des transferts volontaires rendent la distribution légitime, sans besoin d'égalisation par l'État. Toute intervention redistributive viole les droits individuels, traitant les personnes comme des moyens plutôt que des fins, en écho à Kant. &lt;/p&gt; &lt;p&gt; Dans Anarchie, État et utopie, Il réfute l'utilitarisme via l'expérience de pensée de la &lt;a href=&quot;https://www.youtube.com/watch?v=2FVwXaNWPQ0&quot;  title=&quot; La machine à expérience par Monsieur Phi&quot;&gt;&quot;machine à expérience&quot; :&lt;/a&gt;  même si elle offre un bonheur parfait et indistinguable de la réalité, les gens préfèrent vivre des actions réelles et façonner leur identité plutôt que des simulations. Cela prouve que le bonheur n'est pas le seul bien suprême. &lt;/p&gt; &lt;p&gt; Plus tard, dans Explications philosophiques (1981), il développe une théorie du suivi (tracking theory) en épistémologie, où la connaissance repose sur des conditionnels contrefactuels fiables, contournant le scepticisme sans justification traditionnelle. Son anti-coercitivisme intellectuel invite à une philosophie ouverte, non imposée. &lt;/p&gt; &#10;&lt;audio controls title=&quot;Qui a peur des Libertariens par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10467-14.06.2022-ITEMA_23058436-2022C12410S0165-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt;&lt;/audio&gt;&#10;"/>
+    <hyperlink ref="H60" r:id="rId37" display="https://www.laphilo.fr/pho/imyoung-mini.webp"/>
+    <hyperlink ref="H61" r:id="rId38" display="https://www.laphilo.fr/pho/bhooks-mini.webp"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>